<commit_message>
Fase 4: cierre de resultados 2026-09-13
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L133"/>
+  <dimension ref="A1:L153"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7339,6 +7339,1046 @@
         <v>2</v>
       </c>
       <c r="L133" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>Osasuna vs Espanyol</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Osasuna</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E134" t="n">
+        <v>2.61</v>
+      </c>
+      <c r="F134" t="n">
+        <v>38.3</v>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>0-2</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I134" t="n">
+        <v>0</v>
+      </c>
+      <c r="J134" t="n">
+        <v>1</v>
+      </c>
+      <c r="K134" t="n">
+        <v>0</v>
+      </c>
+      <c r="L134" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Athletic Club vs Elche</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Athletic Club</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E135" t="n">
+        <v>1.81</v>
+      </c>
+      <c r="F135" t="n">
+        <v>55.3</v>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I135" t="n">
+        <v>3</v>
+      </c>
+      <c r="J135" t="n">
+        <v>1</v>
+      </c>
+      <c r="K135" t="n">
+        <v>3</v>
+      </c>
+      <c r="L135" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Real Madrid vs Rayo Vallecano</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>Real Madrid</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E136" t="n">
+        <v>1.81</v>
+      </c>
+      <c r="F136" t="n">
+        <v>55.3</v>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>4-1</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I136" t="n">
+        <v>5</v>
+      </c>
+      <c r="J136" t="n">
+        <v>2</v>
+      </c>
+      <c r="K136" t="n">
+        <v>2</v>
+      </c>
+      <c r="L136" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>FC Twente vs ADO Den Haag</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>FC Twente</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E137" t="n">
+        <v>1.56</v>
+      </c>
+      <c r="F137" t="n">
+        <v>64.2</v>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I137" t="n">
+        <v>0</v>
+      </c>
+      <c r="J137" t="n">
+        <v>2</v>
+      </c>
+      <c r="K137" t="n">
+        <v>2</v>
+      </c>
+      <c r="L137" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Casa Pia vs FC Porto</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>FC Porto</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E138" t="n">
+        <v>1.21</v>
+      </c>
+      <c r="F138" t="n">
+        <v>82.90000000000001</v>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>1-4</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I138" t="n">
+        <v>5</v>
+      </c>
+      <c r="J138" t="n">
+        <v>2</v>
+      </c>
+      <c r="K138" t="n">
+        <v>0</v>
+      </c>
+      <c r="L138" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>Union St.-Gilloise vs Lommel SK</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>Union St.-Gilloise</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E139" t="n">
+        <v>1.51</v>
+      </c>
+      <c r="F139" t="n">
+        <v>66.40000000000001</v>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>5-0</t>
+        </is>
+      </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I139" t="n">
+        <v>3</v>
+      </c>
+      <c r="J139" t="n">
+        <v>1</v>
+      </c>
+      <c r="K139" t="n">
+        <v>1</v>
+      </c>
+      <c r="L139" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>Olympiacos vs OFI Crete</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>Olympiacos</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E140" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="F140" t="n">
+        <v>69.09999999999999</v>
+      </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H140" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I140" t="n">
+        <v>1</v>
+      </c>
+      <c r="J140" t="n">
+        <v>2</v>
+      </c>
+      <c r="K140" t="n">
+        <v>2</v>
+      </c>
+      <c r="L140" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>Independiente Rivadavia vs Aldosivi</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E141" t="n">
+        <v>1.92</v>
+      </c>
+      <c r="F141" t="n">
+        <v>51.9</v>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I141" t="n">
+        <v>6</v>
+      </c>
+      <c r="J141" t="n">
+        <v>1</v>
+      </c>
+      <c r="K141" t="n">
+        <v>1</v>
+      </c>
+      <c r="L141" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>Chelsea vs Hull City</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>Hull City</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E142" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="F142" t="n">
+        <v>42.6</v>
+      </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I142" t="n">
+        <v>0</v>
+      </c>
+      <c r="J142" t="n">
+        <v>2</v>
+      </c>
+      <c r="K142" t="n">
+        <v>0</v>
+      </c>
+      <c r="L142" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>Crystal Palace vs Ipswich Town</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Ipswich Town</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E143" t="n">
+        <v>1.51</v>
+      </c>
+      <c r="F143" t="n">
+        <v>66</v>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>2-3</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I143" t="n">
+        <v>0</v>
+      </c>
+      <c r="J143" t="n">
+        <v>1</v>
+      </c>
+      <c r="K143" t="n">
+        <v>1</v>
+      </c>
+      <c r="L143" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>Sunderland vs Arsenal</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>Arsenal</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E144" t="n">
+        <v>1.39</v>
+      </c>
+      <c r="F144" t="n">
+        <v>71.7</v>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>0-2</t>
+        </is>
+      </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I144" t="n">
+        <v>4</v>
+      </c>
+      <c r="J144" t="n">
+        <v>1</v>
+      </c>
+      <c r="K144" t="n">
+        <v>1</v>
+      </c>
+      <c r="L144" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>Swansea City vs Burnley</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>Swansea City</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E145" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="F145" t="n">
+        <v>86.8</v>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I145" t="n">
+        <v>0</v>
+      </c>
+      <c r="J145" t="n">
+        <v>2</v>
+      </c>
+      <c r="K145" t="n">
+        <v>0</v>
+      </c>
+      <c r="L145" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>Racing Santander vs Alavés</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>Racing Santander</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E146" t="n">
+        <v>1.32</v>
+      </c>
+      <c r="F146" t="n">
+        <v>75.90000000000001</v>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I146" t="n">
+        <v>0</v>
+      </c>
+      <c r="J146" t="n">
+        <v>2</v>
+      </c>
+      <c r="K146" t="n">
+        <v>0</v>
+      </c>
+      <c r="L146" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>AJ Auxerre vs Nice</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>AJ Auxerre</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E147" t="n">
+        <v>1.39</v>
+      </c>
+      <c r="F147" t="n">
+        <v>71.90000000000001</v>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I147" t="n">
+        <v>2</v>
+      </c>
+      <c r="J147" t="n">
+        <v>0</v>
+      </c>
+      <c r="K147" t="n">
+        <v>2</v>
+      </c>
+      <c r="L147" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>Fortuna Sittard vs Ajax Amsterdam</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>Fortuna Sittard</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E148" t="n">
+        <v>2.68</v>
+      </c>
+      <c r="F148" t="n">
+        <v>37.4</v>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>1-5</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I148" t="n">
+        <v>4</v>
+      </c>
+      <c r="J148" t="n">
+        <v>1</v>
+      </c>
+      <c r="K148" t="n">
+        <v>2</v>
+      </c>
+      <c r="L148" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>Académico de Viseu vs Vitória de Guimaraes</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Académico de Viseu</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E149" t="n">
+        <v>1.51</v>
+      </c>
+      <c r="F149" t="n">
+        <v>66.3</v>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I149" t="n">
+        <v>4</v>
+      </c>
+      <c r="J149" t="n">
+        <v>0</v>
+      </c>
+      <c r="K149" t="n">
+        <v>3</v>
+      </c>
+      <c r="L149" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>KVC Westerlo vs Standard Liege</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Standard Liege</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E150" t="n">
+        <v>1.53</v>
+      </c>
+      <c r="F150" t="n">
+        <v>65.5</v>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>4-2</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I150" t="n">
+        <v>0</v>
+      </c>
+      <c r="J150" t="n">
+        <v>1</v>
+      </c>
+      <c r="K150" t="n">
+        <v>0</v>
+      </c>
+      <c r="L150" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>Chapecoense vs Internacional</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Internacional</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E151" t="n">
+        <v>2.24</v>
+      </c>
+      <c r="F151" t="n">
+        <v>44.7</v>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I151" t="n">
+        <v>3</v>
+      </c>
+      <c r="J151" t="n">
+        <v>0</v>
+      </c>
+      <c r="K151" t="n">
+        <v>1</v>
+      </c>
+      <c r="L151" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>Palmeiras vs São Paulo</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>Palmeiras</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E152" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="F152" t="n">
+        <v>84.59999999999999</v>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I152" t="n">
+        <v>2</v>
+      </c>
+      <c r="J152" t="n">
+        <v>3</v>
+      </c>
+      <c r="K152" t="n">
+        <v>3</v>
+      </c>
+      <c r="L152" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>Orlando City SC vs Toronto FC</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>Orlando City SC</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E153" t="n">
+        <v>1.23</v>
+      </c>
+      <c r="F153" t="n">
+        <v>81</v>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I153" t="n">
+        <v>0</v>
+      </c>
+      <c r="J153" t="n">
+        <v>1</v>
+      </c>
+      <c r="K153" t="n">
+        <v>0</v>
+      </c>
+      <c r="L153" t="inlineStr">
         <is>
           <t>si</t>
         </is>
@@ -7355,7 +8395,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7973,6 +9013,25 @@
       </c>
       <c r="E33" t="n">
         <v>4</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>20</v>
+      </c>
+      <c r="C34" t="n">
+        <v>14</v>
+      </c>
+      <c r="D34" t="n">
+        <v>70</v>
+      </c>
+      <c r="E34" t="n">
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -7986,7 +9045,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E81"/>
+  <dimension ref="A1:E89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9696,6 +10755,174 @@
         <v>33.3</v>
       </c>
     </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>penal</t>
+        </is>
+      </c>
+      <c r="C82" t="n">
+        <v>5</v>
+      </c>
+      <c r="D82" t="n">
+        <v>2</v>
+      </c>
+      <c r="E82" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>posible_victoria_favorito</t>
+        </is>
+      </c>
+      <c r="C83" t="n">
+        <v>4</v>
+      </c>
+      <c r="D83" t="n">
+        <v>0</v>
+      </c>
+      <c r="E83" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>ampliacion_marcador</t>
+        </is>
+      </c>
+      <c r="C84" t="n">
+        <v>9</v>
+      </c>
+      <c r="D84" t="n">
+        <v>4</v>
+      </c>
+      <c r="E84" t="n">
+        <v>44.4</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>partido_resuelto</t>
+        </is>
+      </c>
+      <c r="C85" t="n">
+        <v>4</v>
+      </c>
+      <c r="D85" t="n">
+        <v>0</v>
+      </c>
+      <c r="E85" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>cuidado_rival_presiona</t>
+        </is>
+      </c>
+      <c r="C86" t="n">
+        <v>16</v>
+      </c>
+      <c r="D86" t="n">
+        <v>3</v>
+      </c>
+      <c r="E86" t="n">
+        <v>18.8</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>posible_empate</t>
+        </is>
+      </c>
+      <c r="C87" t="n">
+        <v>1</v>
+      </c>
+      <c r="D87" t="n">
+        <v>0</v>
+      </c>
+      <c r="E87" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>alerta_1er_tiempo</t>
+        </is>
+      </c>
+      <c r="C88" t="n">
+        <v>2</v>
+      </c>
+      <c r="D88" t="n">
+        <v>0</v>
+      </c>
+      <c r="E88" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>tarjeta_roja</t>
+        </is>
+      </c>
+      <c r="C89" t="n">
+        <v>1</v>
+      </c>
+      <c r="D89" t="n">
+        <v>0</v>
+      </c>
+      <c r="E89" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-09-14
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L153"/>
+  <dimension ref="A1:L174"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8379,6 +8379,1098 @@
         <v>0</v>
       </c>
       <c r="L153" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>Manchester United vs Manchester City</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>Manchester United</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E154" t="n">
+        <v>1.98</v>
+      </c>
+      <c r="F154" t="n">
+        <v>50.5</v>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I154" t="n">
+        <v>0</v>
+      </c>
+      <c r="J154" t="n">
+        <v>3</v>
+      </c>
+      <c r="K154" t="n">
+        <v>0</v>
+      </c>
+      <c r="L154" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Levante vs Barcelona</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>Barcelona</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E155" t="n">
+        <v>1.23</v>
+      </c>
+      <c r="F155" t="n">
+        <v>81.40000000000001</v>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>2-4</t>
+        </is>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I155" t="n">
+        <v>0</v>
+      </c>
+      <c r="J155" t="n">
+        <v>1</v>
+      </c>
+      <c r="K155" t="n">
+        <v>5</v>
+      </c>
+      <c r="L155" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>RB Leipzig vs Hamburg SV</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>RB Leipzig</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E156" t="n">
+        <v>1.69</v>
+      </c>
+      <c r="F156" t="n">
+        <v>59.3</v>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>5-0</t>
+        </is>
+      </c>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I156" t="n">
+        <v>0</v>
+      </c>
+      <c r="J156" t="n">
+        <v>2</v>
+      </c>
+      <c r="K156" t="n">
+        <v>0</v>
+      </c>
+      <c r="L156" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>SV Elversberg vs Bayern Munich</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Bayern Munich</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E157" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="F157" t="n">
+        <v>60.7</v>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H157" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I157" t="n">
+        <v>0</v>
+      </c>
+      <c r="J157" t="n">
+        <v>0</v>
+      </c>
+      <c r="K157" t="n">
+        <v>2</v>
+      </c>
+      <c r="L157" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>Brest vs Paris Saint-Germain</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>Paris Saint-Germain</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E158" t="n">
+        <v>2.34</v>
+      </c>
+      <c r="F158" t="n">
+        <v>42.8</v>
+      </c>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H158" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I158" t="n">
+        <v>2</v>
+      </c>
+      <c r="J158" t="n">
+        <v>0</v>
+      </c>
+      <c r="K158" t="n">
+        <v>2</v>
+      </c>
+      <c r="L158" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>Excelsior vs FC Utrecht</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>Excelsior</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E159" t="n">
+        <v>1.78</v>
+      </c>
+      <c r="F159" t="n">
+        <v>56.2</v>
+      </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H159" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I159" t="n">
+        <v>0</v>
+      </c>
+      <c r="J159" t="n">
+        <v>3</v>
+      </c>
+      <c r="K159" t="n">
+        <v>3</v>
+      </c>
+      <c r="L159" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>Heerenveen vs Telstar</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>Heerenveen</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E160" t="n">
+        <v>1.82</v>
+      </c>
+      <c r="F160" t="n">
+        <v>54.9</v>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I160" t="n">
+        <v>0</v>
+      </c>
+      <c r="J160" t="n">
+        <v>2</v>
+      </c>
+      <c r="K160" t="n">
+        <v>4</v>
+      </c>
+      <c r="L160" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>PEC Zwolle vs Feyenoord Rotterdam</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>Feyenoord Rotterdam</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E161" t="n">
+        <v>1.13</v>
+      </c>
+      <c r="F161" t="n">
+        <v>88.7</v>
+      </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>0-7</t>
+        </is>
+      </c>
+      <c r="H161" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I161" t="n">
+        <v>0</v>
+      </c>
+      <c r="J161" t="n">
+        <v>1</v>
+      </c>
+      <c r="K161" t="n">
+        <v>3</v>
+      </c>
+      <c r="L161" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>PSV Eindhoven vs Sparta Rotterdam</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>PSV Eindhoven</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E162" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="F162" t="n">
+        <v>79</v>
+      </c>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>4-1</t>
+        </is>
+      </c>
+      <c r="H162" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I162" t="n">
+        <v>4</v>
+      </c>
+      <c r="J162" t="n">
+        <v>3</v>
+      </c>
+      <c r="K162" t="n">
+        <v>4</v>
+      </c>
+      <c r="L162" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>Benfica vs Gil Vicente</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>Benfica</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E163" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="F163" t="n">
+        <v>89.40000000000001</v>
+      </c>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="H163" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I163" t="n">
+        <v>4</v>
+      </c>
+      <c r="J163" t="n">
+        <v>4</v>
+      </c>
+      <c r="K163" t="n">
+        <v>1</v>
+      </c>
+      <c r="L163" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>Galatasaray vs Kocaelispor</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>Galatasaray</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E164" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="F164" t="n">
+        <v>86.40000000000001</v>
+      </c>
+      <c r="G164" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I164" t="n">
+        <v>1</v>
+      </c>
+      <c r="J164" t="n">
+        <v>3</v>
+      </c>
+      <c r="K164" t="n">
+        <v>0</v>
+      </c>
+      <c r="L164" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>Kifisia vs Levadiakos</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>Levadiakos</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E165" t="n">
+        <v>1.79</v>
+      </c>
+      <c r="F165" t="n">
+        <v>55.7</v>
+      </c>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H165" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I165" t="n">
+        <v>0</v>
+      </c>
+      <c r="J165" t="n">
+        <v>3</v>
+      </c>
+      <c r="K165" t="n">
+        <v>0</v>
+      </c>
+      <c r="L165" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>Panathinaikos vs Panetolikos</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>Panathinaikos</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E166" t="n">
+        <v>2.02</v>
+      </c>
+      <c r="F166" t="n">
+        <v>49.4</v>
+      </c>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I166" t="n">
+        <v>0</v>
+      </c>
+      <c r="J166" t="n">
+        <v>1</v>
+      </c>
+      <c r="K166" t="n">
+        <v>0</v>
+      </c>
+      <c r="L166" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>Flamengo vs Corinthians</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>Flamengo</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E167" t="n">
+        <v>2.03</v>
+      </c>
+      <c r="F167" t="n">
+        <v>49.2</v>
+      </c>
+      <c r="G167" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H167" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I167" t="n">
+        <v>7</v>
+      </c>
+      <c r="J167" t="n">
+        <v>1</v>
+      </c>
+      <c r="K167" t="n">
+        <v>0</v>
+      </c>
+      <c r="L167" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>Vancouver Whitecaps vs Austin FC</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>Vancouver Whitecaps</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E168" t="n">
+        <v>1.88</v>
+      </c>
+      <c r="F168" t="n">
+        <v>53.2</v>
+      </c>
+      <c r="G168" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H168" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I168" t="n">
+        <v>1</v>
+      </c>
+      <c r="J168" t="n">
+        <v>4</v>
+      </c>
+      <c r="K168" t="n">
+        <v>0</v>
+      </c>
+      <c r="L168" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>Coventry City vs Brighton &amp; Hove Albion</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>Coventry City</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E169" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="F169" t="n">
+        <v>72.2</v>
+      </c>
+      <c r="G169" t="inlineStr">
+        <is>
+          <t>0-5</t>
+        </is>
+      </c>
+      <c r="H169" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I169" t="n">
+        <v>0</v>
+      </c>
+      <c r="J169" t="n">
+        <v>0</v>
+      </c>
+      <c r="K169" t="n">
+        <v>1</v>
+      </c>
+      <c r="L169" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>Celta Vigo vs Málaga</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>Málaga</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E170" t="n">
+        <v>2.09</v>
+      </c>
+      <c r="F170" t="n">
+        <v>47.8</v>
+      </c>
+      <c r="G170" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H170" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I170" t="n">
+        <v>0</v>
+      </c>
+      <c r="J170" t="n">
+        <v>1</v>
+      </c>
+      <c r="K170" t="n">
+        <v>3</v>
+      </c>
+      <c r="L170" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>Real Valladolid vs Real Oviedo</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>Real Valladolid</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E171" t="n">
+        <v>1.41</v>
+      </c>
+      <c r="F171" t="n">
+        <v>71</v>
+      </c>
+      <c r="G171" t="inlineStr">
+        <is>
+          <t>0-3</t>
+        </is>
+      </c>
+      <c r="H171" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I171" t="n">
+        <v>0</v>
+      </c>
+      <c r="J171" t="n">
+        <v>0</v>
+      </c>
+      <c r="K171" t="n">
+        <v>1</v>
+      </c>
+      <c r="L171" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>Club Brugge vs Antwerp</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>Club Brugge</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E172" t="n">
+        <v>1.13</v>
+      </c>
+      <c r="F172" t="n">
+        <v>88.59999999999999</v>
+      </c>
+      <c r="G172" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="H172" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I172" t="n">
+        <v>0</v>
+      </c>
+      <c r="J172" t="n">
+        <v>2</v>
+      </c>
+      <c r="K172" t="n">
+        <v>0</v>
+      </c>
+      <c r="L172" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>Kalamata vs Volos NFC</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>Kalamata</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E173" t="n">
+        <v>1.23</v>
+      </c>
+      <c r="F173" t="n">
+        <v>81</v>
+      </c>
+      <c r="G173" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="H173" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I173" t="n">
+        <v>0</v>
+      </c>
+      <c r="J173" t="n">
+        <v>0</v>
+      </c>
+      <c r="K173" t="n">
+        <v>1</v>
+      </c>
+      <c r="L173" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>Asteras Tripoli vs AEK Athens</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>Asteras Tripoli</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E174" t="n">
+        <v>2.67</v>
+      </c>
+      <c r="F174" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="G174" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H174" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I174" t="n">
+        <v>0</v>
+      </c>
+      <c r="J174" t="n">
+        <v>1</v>
+      </c>
+      <c r="K174" t="n">
+        <v>2</v>
+      </c>
+      <c r="L174" t="inlineStr">
         <is>
           <t>si</t>
         </is>
@@ -8395,7 +9487,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9032,6 +10124,25 @@
       </c>
       <c r="E34" t="n">
         <v>20</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>21</v>
+      </c>
+      <c r="C35" t="n">
+        <v>12</v>
+      </c>
+      <c r="D35" t="n">
+        <v>57.1</v>
+      </c>
+      <c r="E35" t="n">
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -9045,7 +10156,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E89"/>
+  <dimension ref="A1:E95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10923,6 +12034,132 @@
         <v>0</v>
       </c>
     </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>cuidado_rival_presiona</t>
+        </is>
+      </c>
+      <c r="C90" t="n">
+        <v>1</v>
+      </c>
+      <c r="D90" t="n">
+        <v>0</v>
+      </c>
+      <c r="E90" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>ampliacion_marcador</t>
+        </is>
+      </c>
+      <c r="C91" t="n">
+        <v>9</v>
+      </c>
+      <c r="D91" t="n">
+        <v>0</v>
+      </c>
+      <c r="E91" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>posible_victoria_favorito</t>
+        </is>
+      </c>
+      <c r="C92" t="n">
+        <v>5</v>
+      </c>
+      <c r="D92" t="n">
+        <v>1</v>
+      </c>
+      <c r="E92" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>gol_de_cierre</t>
+        </is>
+      </c>
+      <c r="C93" t="n">
+        <v>1</v>
+      </c>
+      <c r="D93" t="n">
+        <v>0</v>
+      </c>
+      <c r="E93" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>penal</t>
+        </is>
+      </c>
+      <c r="C94" t="n">
+        <v>2</v>
+      </c>
+      <c r="D94" t="n">
+        <v>0</v>
+      </c>
+      <c r="E94" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>alerta_1er_tiempo</t>
+        </is>
+      </c>
+      <c r="C95" t="n">
+        <v>1</v>
+      </c>
+      <c r="D95" t="n">
+        <v>0</v>
+      </c>
+      <c r="E95" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-09-20
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L198"/>
+  <dimension ref="A1:L217"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10719,6 +10719,994 @@
         <v>2</v>
       </c>
       <c r="L198" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>Cardiff City vs Charlton Athletic</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>Cardiff City</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E199" t="n">
+        <v>1.21</v>
+      </c>
+      <c r="F199" t="n">
+        <v>82.8</v>
+      </c>
+      <c r="G199" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="H199" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I199" t="n">
+        <v>0</v>
+      </c>
+      <c r="J199" t="n">
+        <v>2</v>
+      </c>
+      <c r="K199" t="n">
+        <v>0</v>
+      </c>
+      <c r="L199" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>Millwall vs West Ham United</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>Millwall</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E200" t="n">
+        <v>1.69</v>
+      </c>
+      <c r="F200" t="n">
+        <v>59.2</v>
+      </c>
+      <c r="G200" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="H200" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I200" t="n">
+        <v>0</v>
+      </c>
+      <c r="J200" t="n">
+        <v>2</v>
+      </c>
+      <c r="K200" t="n">
+        <v>3</v>
+      </c>
+      <c r="L200" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>Stoke City vs Sheffield United</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>Sheffield United</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E201" t="n">
+        <v>1.67</v>
+      </c>
+      <c r="F201" t="n">
+        <v>60</v>
+      </c>
+      <c r="G201" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H201" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I201" t="n">
+        <v>0</v>
+      </c>
+      <c r="J201" t="n">
+        <v>0</v>
+      </c>
+      <c r="K201" t="n">
+        <v>1</v>
+      </c>
+      <c r="L201" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>Sevilla vs Barcelona</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>Barcelona</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E202" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="F202" t="n">
+        <v>79.8</v>
+      </c>
+      <c r="G202" t="inlineStr">
+        <is>
+          <t>1-3</t>
+        </is>
+      </c>
+      <c r="H202" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I202" t="n">
+        <v>5</v>
+      </c>
+      <c r="J202" t="n">
+        <v>1</v>
+      </c>
+      <c r="K202" t="n">
+        <v>7</v>
+      </c>
+      <c r="L202" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>Hamburg SV vs FC Cologne</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>Hamburg SV</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E203" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="F203" t="n">
+        <v>39.4</v>
+      </c>
+      <c r="G203" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H203" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I203" t="n">
+        <v>0</v>
+      </c>
+      <c r="J203" t="n">
+        <v>1</v>
+      </c>
+      <c r="K203" t="n">
+        <v>0</v>
+      </c>
+      <c r="L203" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>Werder Bremen vs FC Augsburg</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>FC Augsburg</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E204" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="F204" t="n">
+        <v>52.5</v>
+      </c>
+      <c r="G204" t="inlineStr">
+        <is>
+          <t>3-2</t>
+        </is>
+      </c>
+      <c r="H204" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I204" t="n">
+        <v>0</v>
+      </c>
+      <c r="J204" t="n">
+        <v>2</v>
+      </c>
+      <c r="K204" t="n">
+        <v>1</v>
+      </c>
+      <c r="L204" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>Le Mans vs Lorient</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>Le Mans</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E205" t="n">
+        <v>1.57</v>
+      </c>
+      <c r="F205" t="n">
+        <v>63.8</v>
+      </c>
+      <c r="G205" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H205" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I205" t="n">
+        <v>3</v>
+      </c>
+      <c r="J205" t="n">
+        <v>2</v>
+      </c>
+      <c r="K205" t="n">
+        <v>0</v>
+      </c>
+      <c r="L205" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>Ajax Amsterdam vs Excelsior</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>Ajax Amsterdam</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E206" t="n">
+        <v>2.04</v>
+      </c>
+      <c r="F206" t="n">
+        <v>49</v>
+      </c>
+      <c r="G206" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="H206" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I206" t="n">
+        <v>4</v>
+      </c>
+      <c r="J206" t="n">
+        <v>4</v>
+      </c>
+      <c r="K206" t="n">
+        <v>4</v>
+      </c>
+      <c r="L206" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>Sporting CP vs Arouca</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>Sporting CP</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E207" t="n">
+        <v>1.62</v>
+      </c>
+      <c r="F207" t="n">
+        <v>61.6</v>
+      </c>
+      <c r="G207" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="H207" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I207" t="n">
+        <v>6</v>
+      </c>
+      <c r="J207" t="n">
+        <v>4</v>
+      </c>
+      <c r="K207" t="n">
+        <v>0</v>
+      </c>
+      <c r="L207" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>Atlético-MG vs Chapecoense</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>Atlético-MG</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E208" t="n">
+        <v>1.62</v>
+      </c>
+      <c r="F208" t="n">
+        <v>61.9</v>
+      </c>
+      <c r="G208" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H208" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I208" t="n">
+        <v>9</v>
+      </c>
+      <c r="J208" t="n">
+        <v>0</v>
+      </c>
+      <c r="K208" t="n">
+        <v>1</v>
+      </c>
+      <c r="L208" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>Vasco da Gama vs Coritiba</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>Vasco da Gama</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E209" t="n">
+        <v>2.18</v>
+      </c>
+      <c r="F209" t="n">
+        <v>45.9</v>
+      </c>
+      <c r="G209" t="inlineStr">
+        <is>
+          <t>5-0</t>
+        </is>
+      </c>
+      <c r="H209" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I209" t="n">
+        <v>0</v>
+      </c>
+      <c r="J209" t="n">
+        <v>0</v>
+      </c>
+      <c r="K209" t="n">
+        <v>1</v>
+      </c>
+      <c r="L209" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>Real Salt Lake vs Vancouver Whitecaps</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>Real Salt Lake</t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E210" t="n">
+        <v>2.37</v>
+      </c>
+      <c r="F210" t="n">
+        <v>42.2</v>
+      </c>
+      <c r="G210" t="inlineStr">
+        <is>
+          <t>0-3</t>
+        </is>
+      </c>
+      <c r="H210" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I210" t="n">
+        <v>0</v>
+      </c>
+      <c r="J210" t="n">
+        <v>0</v>
+      </c>
+      <c r="K210" t="n">
+        <v>5</v>
+      </c>
+      <c r="L210" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>Brighton &amp; Hove Albion vs Arsenal</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>Arsenal</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E211" t="n">
+        <v>1.64</v>
+      </c>
+      <c r="F211" t="n">
+        <v>60.9</v>
+      </c>
+      <c r="G211" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="H211" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I211" t="n">
+        <v>0</v>
+      </c>
+      <c r="J211" t="n">
+        <v>2</v>
+      </c>
+      <c r="K211" t="n">
+        <v>2</v>
+      </c>
+      <c r="L211" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>Wrexham vs Southampton</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>Southampton</t>
+        </is>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E212" t="n">
+        <v>1.52</v>
+      </c>
+      <c r="F212" t="n">
+        <v>65.8</v>
+      </c>
+      <c r="G212" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H212" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I212" t="n">
+        <v>0</v>
+      </c>
+      <c r="J212" t="n">
+        <v>5</v>
+      </c>
+      <c r="K212" t="n">
+        <v>0</v>
+      </c>
+      <c r="L212" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>Paris FC vs Strasbourg</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>Paris FC</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E213" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F213" t="n">
+        <v>66.8</v>
+      </c>
+      <c r="G213" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H213" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I213" t="n">
+        <v>0</v>
+      </c>
+      <c r="J213" t="n">
+        <v>1</v>
+      </c>
+      <c r="K213" t="n">
+        <v>0</v>
+      </c>
+      <c r="L213" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>Anderlecht vs Zulte-Waregem</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>Zulte-Waregem</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E214" t="n">
+        <v>1.44</v>
+      </c>
+      <c r="F214" t="n">
+        <v>69.59999999999999</v>
+      </c>
+      <c r="G214" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="H214" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I214" t="n">
+        <v>3</v>
+      </c>
+      <c r="J214" t="n">
+        <v>2</v>
+      </c>
+      <c r="K214" t="n">
+        <v>1</v>
+      </c>
+      <c r="L214" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>Atromitos vs Kifisia</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>Atromitos</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E215" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="F215" t="n">
+        <v>76.90000000000001</v>
+      </c>
+      <c r="G215" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H215" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I215" t="n">
+        <v>0</v>
+      </c>
+      <c r="J215" t="n">
+        <v>0</v>
+      </c>
+      <c r="K215" t="n">
+        <v>4</v>
+      </c>
+      <c r="L215" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>São Paulo vs Internacional</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>Internacional</t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E216" t="n">
+        <v>1.31</v>
+      </c>
+      <c r="F216" t="n">
+        <v>76.2</v>
+      </c>
+      <c r="G216" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H216" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I216" t="n">
+        <v>0</v>
+      </c>
+      <c r="J216" t="n">
+        <v>4</v>
+      </c>
+      <c r="K216" t="n">
+        <v>2</v>
+      </c>
+      <c r="L216" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>Minnesota United FC vs LA Galaxy</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>Minnesota United FC</t>
+        </is>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E217" t="n">
+        <v>1.46</v>
+      </c>
+      <c r="F217" t="n">
+        <v>68.3</v>
+      </c>
+      <c r="G217" t="inlineStr">
+        <is>
+          <t>2-3</t>
+        </is>
+      </c>
+      <c r="H217" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I217" t="n">
+        <v>0</v>
+      </c>
+      <c r="J217" t="n">
+        <v>1</v>
+      </c>
+      <c r="K217" t="n">
+        <v>1</v>
+      </c>
+      <c r="L217" t="inlineStr">
         <is>
           <t>si</t>
         </is>
@@ -10735,7 +11723,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E40"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11486,6 +12474,25 @@
       </c>
       <c r="E40" t="n">
         <v>4</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>19</v>
+      </c>
+      <c r="C41" t="n">
+        <v>6</v>
+      </c>
+      <c r="D41" t="n">
+        <v>31.6</v>
+      </c>
+      <c r="E41" t="n">
+        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -11499,7 +12506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E126"/>
+  <dimension ref="A1:E135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14154,6 +15161,195 @@
         <v>50</v>
       </c>
     </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>posible_victoria_favorito</t>
+        </is>
+      </c>
+      <c r="C127" t="n">
+        <v>6</v>
+      </c>
+      <c r="D127" t="n">
+        <v>1</v>
+      </c>
+      <c r="E127" t="n">
+        <v>16.7</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>ampliacion_marcador</t>
+        </is>
+      </c>
+      <c r="C128" t="n">
+        <v>9</v>
+      </c>
+      <c r="D128" t="n">
+        <v>1</v>
+      </c>
+      <c r="E128" t="n">
+        <v>11.1</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>cuidado_rival_presiona</t>
+        </is>
+      </c>
+      <c r="C129" t="n">
+        <v>6</v>
+      </c>
+      <c r="D129" t="n">
+        <v>2</v>
+      </c>
+      <c r="E129" t="n">
+        <v>33.3</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>gol_de_cierre</t>
+        </is>
+      </c>
+      <c r="C130" t="n">
+        <v>4</v>
+      </c>
+      <c r="D130" t="n">
+        <v>0</v>
+      </c>
+      <c r="E130" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>tarjeta_roja</t>
+        </is>
+      </c>
+      <c r="C131" t="n">
+        <v>1</v>
+      </c>
+      <c r="D131" t="n">
+        <v>0</v>
+      </c>
+      <c r="E131" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>penal</t>
+        </is>
+      </c>
+      <c r="C132" t="n">
+        <v>1</v>
+      </c>
+      <c r="D132" t="n">
+        <v>0</v>
+      </c>
+      <c r="E132" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>alerta_1er_tiempo</t>
+        </is>
+      </c>
+      <c r="C133" t="n">
+        <v>1</v>
+      </c>
+      <c r="D133" t="n">
+        <v>0</v>
+      </c>
+      <c r="E133" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>posible_empate</t>
+        </is>
+      </c>
+      <c r="C134" t="n">
+        <v>1</v>
+      </c>
+      <c r="D134" t="n">
+        <v>1</v>
+      </c>
+      <c r="E134" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>partido_resuelto</t>
+        </is>
+      </c>
+      <c r="C135" t="n">
+        <v>1</v>
+      </c>
+      <c r="D135" t="n">
+        <v>0</v>
+      </c>
+      <c r="E135" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-09-21
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L217"/>
+  <dimension ref="A1:L241"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11707,6 +11707,1254 @@
         <v>1</v>
       </c>
       <c r="L217" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>Leeds United vs Crystal Palace</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>Leeds United</t>
+        </is>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E218" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="F218" t="n">
+        <v>72.2</v>
+      </c>
+      <c r="G218" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H218" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I218" t="n">
+        <v>0</v>
+      </c>
+      <c r="J218" t="n">
+        <v>2</v>
+      </c>
+      <c r="K218" t="n">
+        <v>3</v>
+      </c>
+      <c r="L218" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>Manchester City vs Sunderland</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>Manchester City</t>
+        </is>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E219" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="F219" t="n">
+        <v>83.2</v>
+      </c>
+      <c r="G219" t="inlineStr">
+        <is>
+          <t>5-3</t>
+        </is>
+      </c>
+      <c r="H219" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I219" t="n">
+        <v>0</v>
+      </c>
+      <c r="J219" t="n">
+        <v>1</v>
+      </c>
+      <c r="K219" t="n">
+        <v>2</v>
+      </c>
+      <c r="L219" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>Parma vs Genoa</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>Parma</t>
+        </is>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E220" t="n">
+        <v>2.32</v>
+      </c>
+      <c r="F220" t="n">
+        <v>43.1</v>
+      </c>
+      <c r="G220" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H220" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I220" t="n">
+        <v>0</v>
+      </c>
+      <c r="J220" t="n">
+        <v>1</v>
+      </c>
+      <c r="K220" t="n">
+        <v>0</v>
+      </c>
+      <c r="L220" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>AC Milan vs Lecce</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>AC Milan</t>
+        </is>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E221" t="n">
+        <v>2.28</v>
+      </c>
+      <c r="F221" t="n">
+        <v>43.8</v>
+      </c>
+      <c r="G221" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="H221" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I221" t="n">
+        <v>4</v>
+      </c>
+      <c r="J221" t="n">
+        <v>1</v>
+      </c>
+      <c r="K221" t="n">
+        <v>0</v>
+      </c>
+      <c r="L221" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>SC Paderborn 07 vs TSG Hoffenheim</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>SC Paderborn 07</t>
+        </is>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E222" t="n">
+        <v>2.16</v>
+      </c>
+      <c r="F222" t="n">
+        <v>46.4</v>
+      </c>
+      <c r="G222" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="H222" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I222" t="n">
+        <v>3</v>
+      </c>
+      <c r="J222" t="n">
+        <v>0</v>
+      </c>
+      <c r="K222" t="n">
+        <v>1</v>
+      </c>
+      <c r="L222" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>AJ Auxerre vs Brest</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>AJ Auxerre</t>
+        </is>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E223" t="n">
+        <v>1.24</v>
+      </c>
+      <c r="F223" t="n">
+        <v>80.40000000000001</v>
+      </c>
+      <c r="G223" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H223" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I223" t="n">
+        <v>0</v>
+      </c>
+      <c r="J223" t="n">
+        <v>1</v>
+      </c>
+      <c r="K223" t="n">
+        <v>1</v>
+      </c>
+      <c r="L223" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>AZ Alkmaar vs Telstar</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>AZ Alkmaar</t>
+        </is>
+      </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E224" t="n">
+        <v>1.37</v>
+      </c>
+      <c r="F224" t="n">
+        <v>73</v>
+      </c>
+      <c r="G224" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H224" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I224" t="n">
+        <v>0</v>
+      </c>
+      <c r="J224" t="n">
+        <v>2</v>
+      </c>
+      <c r="K224" t="n">
+        <v>5</v>
+      </c>
+      <c r="L224" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>Volos NFC vs AEK Athens</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>AEK Athens</t>
+        </is>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E225" t="n">
+        <v>1.67</v>
+      </c>
+      <c r="F225" t="n">
+        <v>60</v>
+      </c>
+      <c r="G225" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H225" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I225" t="n">
+        <v>0</v>
+      </c>
+      <c r="J225" t="n">
+        <v>2</v>
+      </c>
+      <c r="K225" t="n">
+        <v>3</v>
+      </c>
+      <c r="L225" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>Flamengo vs Red Bull Bragantino</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>Flamengo</t>
+        </is>
+      </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E226" t="n">
+        <v>1.84</v>
+      </c>
+      <c r="F226" t="n">
+        <v>54.3</v>
+      </c>
+      <c r="G226" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H226" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I226" t="n">
+        <v>5</v>
+      </c>
+      <c r="J226" t="n">
+        <v>3</v>
+      </c>
+      <c r="K226" t="n">
+        <v>0</v>
+      </c>
+      <c r="L226" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>Belgrano (Córdoba) vs Estudiantes de Río Cuarto</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>Belgrano (Córdoba)</t>
+        </is>
+      </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E227" t="n">
+        <v>2.04</v>
+      </c>
+      <c r="F227" t="n">
+        <v>49.1</v>
+      </c>
+      <c r="G227" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H227" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I227" t="n">
+        <v>1</v>
+      </c>
+      <c r="J227" t="n">
+        <v>1</v>
+      </c>
+      <c r="K227" t="n">
+        <v>0</v>
+      </c>
+      <c r="L227" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>Toluca vs Santos</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>Toluca</t>
+        </is>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E228" t="n">
+        <v>1.34</v>
+      </c>
+      <c r="F228" t="n">
+        <v>74.40000000000001</v>
+      </c>
+      <c r="G228" t="inlineStr">
+        <is>
+          <t>2-3</t>
+        </is>
+      </c>
+      <c r="H228" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I228" t="n">
+        <v>0</v>
+      </c>
+      <c r="J228" t="n">
+        <v>4</v>
+      </c>
+      <c r="K228" t="n">
+        <v>0</v>
+      </c>
+      <c r="L228" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>Fulham vs Manchester United</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>Manchester United</t>
+        </is>
+      </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E229" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="F229" t="n">
+        <v>72.59999999999999</v>
+      </c>
+      <c r="G229" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H229" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I229" t="n">
+        <v>0</v>
+      </c>
+      <c r="J229" t="n">
+        <v>2</v>
+      </c>
+      <c r="K229" t="n">
+        <v>4</v>
+      </c>
+      <c r="L229" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>Getafe vs Málaga</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>Málaga</t>
+        </is>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E230" t="n">
+        <v>1.86</v>
+      </c>
+      <c r="F230" t="n">
+        <v>53.7</v>
+      </c>
+      <c r="G230" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H230" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I230" t="n">
+        <v>0</v>
+      </c>
+      <c r="J230" t="n">
+        <v>1</v>
+      </c>
+      <c r="K230" t="n">
+        <v>5</v>
+      </c>
+      <c r="L230" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>Atlético Madrid vs Real Madrid</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>Real Madrid</t>
+        </is>
+      </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E231" t="n">
+        <v>1.79</v>
+      </c>
+      <c r="F231" t="n">
+        <v>55.8</v>
+      </c>
+      <c r="G231" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H231" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I231" t="n">
+        <v>0</v>
+      </c>
+      <c r="J231" t="n">
+        <v>1</v>
+      </c>
+      <c r="K231" t="n">
+        <v>4</v>
+      </c>
+      <c r="L231" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>Villarreal vs Levante</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>Villarreal</t>
+        </is>
+      </c>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E232" t="n">
+        <v>1.34</v>
+      </c>
+      <c r="F232" t="n">
+        <v>74.5</v>
+      </c>
+      <c r="G232" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="H232" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I232" t="n">
+        <v>0</v>
+      </c>
+      <c r="J232" t="n">
+        <v>2</v>
+      </c>
+      <c r="K232" t="n">
+        <v>2</v>
+      </c>
+      <c r="L232" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>Nice vs Lille</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>Lille</t>
+        </is>
+      </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E233" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="F233" t="n">
+        <v>69.8</v>
+      </c>
+      <c r="G233" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H233" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I233" t="n">
+        <v>0</v>
+      </c>
+      <c r="J233" t="n">
+        <v>3</v>
+      </c>
+      <c r="K233" t="n">
+        <v>0</v>
+      </c>
+      <c r="L233" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>Marseille vs Paris Saint-Germain</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>Marseille</t>
+        </is>
+      </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E234" t="n">
+        <v>2.55</v>
+      </c>
+      <c r="F234" t="n">
+        <v>39.2</v>
+      </c>
+      <c r="G234" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H234" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I234" t="n">
+        <v>3</v>
+      </c>
+      <c r="J234" t="n">
+        <v>1</v>
+      </c>
+      <c r="K234" t="n">
+        <v>3</v>
+      </c>
+      <c r="L234" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>FC Twente vs PSV Eindhoven</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>PSV Eindhoven</t>
+        </is>
+      </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E235" t="n">
+        <v>1.41</v>
+      </c>
+      <c r="F235" t="n">
+        <v>70.7</v>
+      </c>
+      <c r="G235" t="inlineStr">
+        <is>
+          <t>3-2</t>
+        </is>
+      </c>
+      <c r="H235" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I235" t="n">
+        <v>0</v>
+      </c>
+      <c r="J235" t="n">
+        <v>3</v>
+      </c>
+      <c r="K235" t="n">
+        <v>4</v>
+      </c>
+      <c r="L235" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>Vitória de Guimaraes vs Moreirense</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>Moreirense</t>
+        </is>
+      </c>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E236" t="n">
+        <v>2.24</v>
+      </c>
+      <c r="F236" t="n">
+        <v>44.7</v>
+      </c>
+      <c r="G236" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H236" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I236" t="n">
+        <v>0</v>
+      </c>
+      <c r="J236" t="n">
+        <v>4</v>
+      </c>
+      <c r="K236" t="n">
+        <v>1</v>
+      </c>
+      <c r="L236" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>Antwerp vs Union St.-Gilloise</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>Union St.-Gilloise</t>
+        </is>
+      </c>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E237" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="F237" t="n">
+        <v>75.2</v>
+      </c>
+      <c r="G237" t="inlineStr">
+        <is>
+          <t>0-2</t>
+        </is>
+      </c>
+      <c r="H237" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I237" t="n">
+        <v>0</v>
+      </c>
+      <c r="J237" t="n">
+        <v>1</v>
+      </c>
+      <c r="K237" t="n">
+        <v>2</v>
+      </c>
+      <c r="L237" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>Sint-Truidense vs KVC Westerlo</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>Sint-Truidense</t>
+        </is>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E238" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="F238" t="n">
+        <v>74</v>
+      </c>
+      <c r="G238" t="inlineStr">
+        <is>
+          <t>0-2</t>
+        </is>
+      </c>
+      <c r="H238" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I238" t="n">
+        <v>0</v>
+      </c>
+      <c r="J238" t="n">
+        <v>0</v>
+      </c>
+      <c r="K238" t="n">
+        <v>2</v>
+      </c>
+      <c r="L238" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>Club Brugge vs Racing Genk</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>Club Brugge</t>
+        </is>
+      </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E239" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="F239" t="n">
+        <v>80</v>
+      </c>
+      <c r="G239" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="H239" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I239" t="n">
+        <v>1</v>
+      </c>
+      <c r="J239" t="n">
+        <v>3</v>
+      </c>
+      <c r="K239" t="n">
+        <v>0</v>
+      </c>
+      <c r="L239" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>Levadiakos vs Olympiacos</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>Levadiakos</t>
+        </is>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E240" t="n">
+        <v>2.57</v>
+      </c>
+      <c r="F240" t="n">
+        <v>38.9</v>
+      </c>
+      <c r="G240" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H240" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I240" t="n">
+        <v>0</v>
+      </c>
+      <c r="J240" t="n">
+        <v>1</v>
+      </c>
+      <c r="K240" t="n">
+        <v>4</v>
+      </c>
+      <c r="L240" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>Kalamata vs Panathinaikos</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>Kalamata</t>
+        </is>
+      </c>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E241" t="n">
+        <v>1.99</v>
+      </c>
+      <c r="F241" t="n">
+        <v>50.3</v>
+      </c>
+      <c r="G241" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H241" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I241" t="n">
+        <v>0</v>
+      </c>
+      <c r="J241" t="n">
+        <v>1</v>
+      </c>
+      <c r="K241" t="n">
+        <v>2</v>
+      </c>
+      <c r="L241" t="inlineStr">
         <is>
           <t>si</t>
         </is>
@@ -11723,7 +12971,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12493,6 +13741,25 @@
       </c>
       <c r="E41" t="n">
         <v>19</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>24</v>
+      </c>
+      <c r="C42" t="n">
+        <v>12</v>
+      </c>
+      <c r="D42" t="n">
+        <v>50</v>
+      </c>
+      <c r="E42" t="n">
+        <v>24</v>
       </c>
     </row>
   </sheetData>
@@ -12506,7 +13773,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E135"/>
+  <dimension ref="A1:E140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15350,6 +16617,111 @@
         <v>0</v>
       </c>
     </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>ampliacion_marcador</t>
+        </is>
+      </c>
+      <c r="C136" t="n">
+        <v>6</v>
+      </c>
+      <c r="D136" t="n">
+        <v>2</v>
+      </c>
+      <c r="E136" t="n">
+        <v>33.3</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>partido_resuelto</t>
+        </is>
+      </c>
+      <c r="C137" t="n">
+        <v>2</v>
+      </c>
+      <c r="D137" t="n">
+        <v>0</v>
+      </c>
+      <c r="E137" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>cuidado_rival_presiona</t>
+        </is>
+      </c>
+      <c r="C138" t="n">
+        <v>7</v>
+      </c>
+      <c r="D138" t="n">
+        <v>0</v>
+      </c>
+      <c r="E138" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>posible_victoria_favorito</t>
+        </is>
+      </c>
+      <c r="C139" t="n">
+        <v>1</v>
+      </c>
+      <c r="D139" t="n">
+        <v>0</v>
+      </c>
+      <c r="E139" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>tarjeta_roja</t>
+        </is>
+      </c>
+      <c r="C140" t="n">
+        <v>1</v>
+      </c>
+      <c r="D140" t="n">
+        <v>0</v>
+      </c>
+      <c r="E140" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-09-27
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L242"/>
+  <dimension ref="A1:L246"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13007,6 +13007,214 @@
         <v>1</v>
       </c>
       <c r="L242" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>Nashville SC vs Toronto FC</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>Nashville SC</t>
+        </is>
+      </c>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E243" t="n">
+        <v>1.73</v>
+      </c>
+      <c r="F243" t="n">
+        <v>57.7</v>
+      </c>
+      <c r="G243" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H243" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I243" t="n">
+        <v>0</v>
+      </c>
+      <c r="J243" t="n">
+        <v>0</v>
+      </c>
+      <c r="K243" t="n">
+        <v>1</v>
+      </c>
+      <c r="L243" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>Philadelphia Union vs Orlando City SC</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>Orlando City SC</t>
+        </is>
+      </c>
+      <c r="D244" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E244" t="n">
+        <v>1.99</v>
+      </c>
+      <c r="F244" t="n">
+        <v>50.2</v>
+      </c>
+      <c r="G244" t="inlineStr">
+        <is>
+          <t>4-2</t>
+        </is>
+      </c>
+      <c r="H244" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I244" t="n">
+        <v>2</v>
+      </c>
+      <c r="J244" t="n">
+        <v>0</v>
+      </c>
+      <c r="K244" t="n">
+        <v>2</v>
+      </c>
+      <c r="L244" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>Seattle Sounders FC vs Minnesota United FC</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>Minnesota United FC</t>
+        </is>
+      </c>
+      <c r="D245" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E245" t="n">
+        <v>2.53</v>
+      </c>
+      <c r="F245" t="n">
+        <v>39.6</v>
+      </c>
+      <c r="G245" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="H245" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I245" t="n">
+        <v>0</v>
+      </c>
+      <c r="J245" t="n">
+        <v>1</v>
+      </c>
+      <c r="K245" t="n">
+        <v>2</v>
+      </c>
+      <c r="L245" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>Vancouver Whitecaps vs D.C. United</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>D.C. United</t>
+        </is>
+      </c>
+      <c r="D246" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E246" t="n">
+        <v>2.62</v>
+      </c>
+      <c r="F246" t="n">
+        <v>38.1</v>
+      </c>
+      <c r="G246" t="inlineStr">
+        <is>
+          <t>3-3</t>
+        </is>
+      </c>
+      <c r="H246" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I246" t="n">
+        <v>0</v>
+      </c>
+      <c r="J246" t="n">
+        <v>6</v>
+      </c>
+      <c r="K246" t="n">
+        <v>0</v>
+      </c>
+      <c r="L246" t="inlineStr">
         <is>
           <t>si</t>
         </is>
@@ -13023,7 +13231,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E47"/>
+  <dimension ref="A1:E48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13895,6 +14103,25 @@
       </c>
       <c r="E47" t="n">
         <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>4</v>
+      </c>
+      <c r="C48" t="n">
+        <v>1</v>
+      </c>
+      <c r="D48" t="n">
+        <v>25</v>
+      </c>
+      <c r="E48" t="n">
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -13908,7 +14135,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E141"/>
+  <dimension ref="A1:E143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16878,6 +17105,48 @@
         <v>0</v>
       </c>
     </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>penal</t>
+        </is>
+      </c>
+      <c r="C142" t="n">
+        <v>1</v>
+      </c>
+      <c r="D142" t="n">
+        <v>1</v>
+      </c>
+      <c r="E142" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>cuidado_rival_presiona</t>
+        </is>
+      </c>
+      <c r="C143" t="n">
+        <v>1</v>
+      </c>
+      <c r="D143" t="n">
+        <v>1</v>
+      </c>
+      <c r="E143" t="n">
+        <v>100</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-10-01
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -13335,7 +13335,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E51"/>
+  <dimension ref="A1:E52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14279,6 +14279,22 @@
         <v>0</v>
       </c>
       <c r="E51" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>0</v>
+      </c>
+      <c r="C52" t="n">
+        <v>0</v>
+      </c>
+      <c r="E52" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-10-02
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L248"/>
+  <dimension ref="A1:L249"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13319,6 +13319,58 @@
         <v>1</v>
       </c>
       <c r="L248" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>Seattle Sounders FC vs Sporting Kansas City</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>Seattle Sounders FC</t>
+        </is>
+      </c>
+      <c r="D249" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E249" t="n">
+        <v>1.52</v>
+      </c>
+      <c r="F249" t="n">
+        <v>65.90000000000001</v>
+      </c>
+      <c r="G249" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H249" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I249" t="n">
+        <v>0</v>
+      </c>
+      <c r="J249" t="n">
+        <v>2</v>
+      </c>
+      <c r="K249" t="n">
+        <v>2</v>
+      </c>
+      <c r="L249" t="inlineStr">
         <is>
           <t>si</t>
         </is>
@@ -13335,7 +13387,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E52"/>
+  <dimension ref="A1:E53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14296,6 +14348,25 @@
       </c>
       <c r="E52" t="n">
         <v>0</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>1</v>
+      </c>
+      <c r="C53" t="n">
+        <v>1</v>
+      </c>
+      <c r="D53" t="n">
+        <v>100</v>
+      </c>
+      <c r="E53" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-10-03
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -13387,7 +13387,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E53"/>
+  <dimension ref="A1:E54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14367,6 +14367,22 @@
       </c>
       <c r="E53" t="n">
         <v>1</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>0</v>
+      </c>
+      <c r="C54" t="n">
+        <v>0</v>
+      </c>
+      <c r="E54" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-10-04
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -13387,7 +13387,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E54"/>
+  <dimension ref="A1:E55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14382,6 +14382,22 @@
         <v>0</v>
       </c>
       <c r="E54" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>0</v>
+      </c>
+      <c r="C55" t="n">
+        <v>0</v>
+      </c>
+      <c r="E55" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-10-05
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L249"/>
+  <dimension ref="A1:L252"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13371,6 +13371,162 @@
         <v>2</v>
       </c>
       <c r="L249" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>Castellón vs Ceuta</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>Castellón</t>
+        </is>
+      </c>
+      <c r="D250" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E250" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="F250" t="n">
+        <v>75</v>
+      </c>
+      <c r="G250" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H250" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I250" t="n">
+        <v>0</v>
+      </c>
+      <c r="J250" t="n">
+        <v>2</v>
+      </c>
+      <c r="K250" t="n">
+        <v>2</v>
+      </c>
+      <c r="L250" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>Estudiantes de Río Cuarto vs Racing Club</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>Estudiantes de Río Cuarto</t>
+        </is>
+      </c>
+      <c r="D251" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E251" t="n">
+        <v>2.36</v>
+      </c>
+      <c r="F251" t="n">
+        <v>42.3</v>
+      </c>
+      <c r="G251" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H251" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I251" t="n">
+        <v>5</v>
+      </c>
+      <c r="J251" t="n">
+        <v>1</v>
+      </c>
+      <c r="K251" t="n">
+        <v>0</v>
+      </c>
+      <c r="L251" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>Las Palmas vs Real Valladolid</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>Las Palmas</t>
+        </is>
+      </c>
+      <c r="D252" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E252" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="F252" t="n">
+        <v>69.09999999999999</v>
+      </c>
+      <c r="G252" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="H252" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I252" t="n">
+        <v>0</v>
+      </c>
+      <c r="J252" t="n">
+        <v>0</v>
+      </c>
+      <c r="K252" t="n">
+        <v>1</v>
+      </c>
+      <c r="L252" t="inlineStr">
         <is>
           <t>si</t>
         </is>
@@ -13387,7 +13543,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E55"/>
+  <dimension ref="A1:E56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14399,6 +14555,25 @@
       </c>
       <c r="E55" t="n">
         <v>0</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>3</v>
+      </c>
+      <c r="C56" t="n">
+        <v>0</v>
+      </c>
+      <c r="D56" t="n">
+        <v>0</v>
+      </c>
+      <c r="E56" t="n">
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -14412,7 +14587,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E146"/>
+  <dimension ref="A1:E149"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17487,6 +17662,69 @@
         <v>0</v>
       </c>
     </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>cuidado_rival_presiona</t>
+        </is>
+      </c>
+      <c r="C147" t="n">
+        <v>3</v>
+      </c>
+      <c r="D147" t="n">
+        <v>1</v>
+      </c>
+      <c r="E147" t="n">
+        <v>33.3</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>posible_empate</t>
+        </is>
+      </c>
+      <c r="C148" t="n">
+        <v>1</v>
+      </c>
+      <c r="D148" t="n">
+        <v>0</v>
+      </c>
+      <c r="E148" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>gol_de_cierre</t>
+        </is>
+      </c>
+      <c r="C149" t="n">
+        <v>1</v>
+      </c>
+      <c r="D149" t="n">
+        <v>1</v>
+      </c>
+      <c r="E149" t="n">
+        <v>100</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-10-06
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -13543,7 +13543,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E56"/>
+  <dimension ref="A1:E57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14574,6 +14574,22 @@
       </c>
       <c r="E56" t="n">
         <v>3</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>0</v>
+      </c>
+      <c r="C57" t="n">
+        <v>0</v>
+      </c>
+      <c r="E57" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-10-07
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -13543,7 +13543,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E57"/>
+  <dimension ref="A1:E58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14589,6 +14589,22 @@
         <v>0</v>
       </c>
       <c r="E57" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>0</v>
+      </c>
+      <c r="C58" t="n">
+        <v>0</v>
+      </c>
+      <c r="E58" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-10-08
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L252"/>
+  <dimension ref="A1:L254"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13527,6 +13527,110 @@
         <v>1</v>
       </c>
       <c r="L252" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>Botafogo vs Vasco da Gama</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>Botafogo</t>
+        </is>
+      </c>
+      <c r="D253" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E253" t="n">
+        <v>2.46</v>
+      </c>
+      <c r="F253" t="n">
+        <v>40.6</v>
+      </c>
+      <c r="G253" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H253" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I253" t="n">
+        <v>4</v>
+      </c>
+      <c r="J253" t="n">
+        <v>0</v>
+      </c>
+      <c r="K253" t="n">
+        <v>1</v>
+      </c>
+      <c r="L253" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>Cruzeiro vs São Paulo</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>Cruzeiro</t>
+        </is>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E254" t="n">
+        <v>1.51</v>
+      </c>
+      <c r="F254" t="n">
+        <v>66.3</v>
+      </c>
+      <c r="G254" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H254" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I254" t="n">
+        <v>2</v>
+      </c>
+      <c r="J254" t="n">
+        <v>0</v>
+      </c>
+      <c r="K254" t="n">
+        <v>5</v>
+      </c>
+      <c r="L254" t="inlineStr">
         <is>
           <t>si</t>
         </is>
@@ -13543,7 +13647,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E58"/>
+  <dimension ref="A1:E59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14606,6 +14710,25 @@
       </c>
       <c r="E58" t="n">
         <v>0</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>2</v>
+      </c>
+      <c r="C59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D59" t="n">
+        <v>50</v>
+      </c>
+      <c r="E59" t="n">
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -14619,7 +14742,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E149"/>
+  <dimension ref="A1:E152"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17757,6 +17880,69 @@
         <v>100</v>
       </c>
     </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>cuidado_rival_presiona</t>
+        </is>
+      </c>
+      <c r="C150" t="n">
+        <v>4</v>
+      </c>
+      <c r="D150" t="n">
+        <v>1</v>
+      </c>
+      <c r="E150" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>alerta_1er_tiempo</t>
+        </is>
+      </c>
+      <c r="C151" t="n">
+        <v>1</v>
+      </c>
+      <c r="D151" t="n">
+        <v>1</v>
+      </c>
+      <c r="E151" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>ampliacion_marcador</t>
+        </is>
+      </c>
+      <c r="C152" t="n">
+        <v>1</v>
+      </c>
+      <c r="D152" t="n">
+        <v>0</v>
+      </c>
+      <c r="E152" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-10-09
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L254"/>
+  <dimension ref="A1:L256"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13631,6 +13631,110 @@
         <v>5</v>
       </c>
       <c r="L254" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>Santos vs Flamengo</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>Flamengo</t>
+        </is>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E255" t="n">
+        <v>1.99</v>
+      </c>
+      <c r="F255" t="n">
+        <v>50.3</v>
+      </c>
+      <c r="G255" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="H255" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I255" t="n">
+        <v>4</v>
+      </c>
+      <c r="J255" t="n">
+        <v>0</v>
+      </c>
+      <c r="K255" t="n">
+        <v>4</v>
+      </c>
+      <c r="L255" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>Fluminense vs Coritiba</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>Coritiba</t>
+        </is>
+      </c>
+      <c r="D256" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E256" t="n">
+        <v>1.81</v>
+      </c>
+      <c r="F256" t="n">
+        <v>55.2</v>
+      </c>
+      <c r="G256" t="inlineStr">
+        <is>
+          <t>4-0</t>
+        </is>
+      </c>
+      <c r="H256" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I256" t="n">
+        <v>4</v>
+      </c>
+      <c r="J256" t="n">
+        <v>4</v>
+      </c>
+      <c r="K256" t="n">
+        <v>2</v>
+      </c>
+      <c r="L256" t="inlineStr">
         <is>
           <t>si</t>
         </is>
@@ -13647,7 +13751,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E59"/>
+  <dimension ref="A1:E60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14728,6 +14832,25 @@
         <v>50</v>
       </c>
       <c r="E59" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>2</v>
+      </c>
+      <c r="C60" t="n">
+        <v>0</v>
+      </c>
+      <c r="D60" t="n">
+        <v>0</v>
+      </c>
+      <c r="E60" t="n">
         <v>2</v>
       </c>
     </row>
@@ -14742,7 +14865,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E152"/>
+  <dimension ref="A1:E157"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17943,6 +18066,111 @@
         <v>0</v>
       </c>
     </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>cuidado_rival_presiona</t>
+        </is>
+      </c>
+      <c r="C153" t="n">
+        <v>4</v>
+      </c>
+      <c r="D153" t="n">
+        <v>2</v>
+      </c>
+      <c r="E153" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>ampliacion_marcador</t>
+        </is>
+      </c>
+      <c r="C154" t="n">
+        <v>1</v>
+      </c>
+      <c r="D154" t="n">
+        <v>0</v>
+      </c>
+      <c r="E154" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>tarjeta_roja</t>
+        </is>
+      </c>
+      <c r="C155" t="n">
+        <v>1</v>
+      </c>
+      <c r="D155" t="n">
+        <v>0</v>
+      </c>
+      <c r="E155" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>penal</t>
+        </is>
+      </c>
+      <c r="C156" t="n">
+        <v>1</v>
+      </c>
+      <c r="D156" t="n">
+        <v>0</v>
+      </c>
+      <c r="E156" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>partido_resuelto</t>
+        </is>
+      </c>
+      <c r="C157" t="n">
+        <v>1</v>
+      </c>
+      <c r="D157" t="n">
+        <v>0</v>
+      </c>
+      <c r="E157" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-10-10
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L256"/>
+  <dimension ref="A1:L260"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13735,6 +13735,214 @@
         <v>2</v>
       </c>
       <c r="L256" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>West Ham United vs Queens Park Rangers</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>West Ham United</t>
+        </is>
+      </c>
+      <c r="D257" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E257" t="n">
+        <v>2.21</v>
+      </c>
+      <c r="F257" t="n">
+        <v>45.3</v>
+      </c>
+      <c r="G257" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H257" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I257" t="n">
+        <v>3</v>
+      </c>
+      <c r="J257" t="n">
+        <v>4</v>
+      </c>
+      <c r="K257" t="n">
+        <v>0</v>
+      </c>
+      <c r="L257" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>Borussia Dortmund vs Werder Bremen</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>Borussia Dortmund</t>
+        </is>
+      </c>
+      <c r="D258" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E258" t="n">
+        <v>1.23</v>
+      </c>
+      <c r="F258" t="n">
+        <v>81.09999999999999</v>
+      </c>
+      <c r="G258" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="H258" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I258" t="n">
+        <v>1</v>
+      </c>
+      <c r="J258" t="n">
+        <v>0</v>
+      </c>
+      <c r="K258" t="n">
+        <v>3</v>
+      </c>
+      <c r="L258" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>PSV Eindhoven vs Heerenveen</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>PSV Eindhoven</t>
+        </is>
+      </c>
+      <c r="D259" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E259" t="n">
+        <v>1.19</v>
+      </c>
+      <c r="F259" t="n">
+        <v>84</v>
+      </c>
+      <c r="G259" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H259" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I259" t="n">
+        <v>0</v>
+      </c>
+      <c r="J259" t="n">
+        <v>5</v>
+      </c>
+      <c r="K259" t="n">
+        <v>3</v>
+      </c>
+      <c r="L259" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>Galatasaray vs Kasimpasa</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>Galatasaray</t>
+        </is>
+      </c>
+      <c r="D260" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E260" t="n">
+        <v>1.17</v>
+      </c>
+      <c r="F260" t="n">
+        <v>85.8</v>
+      </c>
+      <c r="G260" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="H260" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I260" t="n">
+        <v>0</v>
+      </c>
+      <c r="J260" t="n">
+        <v>4</v>
+      </c>
+      <c r="K260" t="n">
+        <v>0</v>
+      </c>
+      <c r="L260" t="inlineStr">
         <is>
           <t>si</t>
         </is>
@@ -13751,7 +13959,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E60"/>
+  <dimension ref="A1:E61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14852,6 +15060,25 @@
       </c>
       <c r="E60" t="n">
         <v>2</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>4</v>
+      </c>
+      <c r="C61" t="n">
+        <v>2</v>
+      </c>
+      <c r="D61" t="n">
+        <v>50</v>
+      </c>
+      <c r="E61" t="n">
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -14865,7 +15092,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E157"/>
+  <dimension ref="A1:E161"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18171,6 +18398,90 @@
         <v>0</v>
       </c>
     </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>penal</t>
+        </is>
+      </c>
+      <c r="C158" t="n">
+        <v>1</v>
+      </c>
+      <c r="D158" t="n">
+        <v>0</v>
+      </c>
+      <c r="E158" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>gol_de_cierre</t>
+        </is>
+      </c>
+      <c r="C159" t="n">
+        <v>1</v>
+      </c>
+      <c r="D159" t="n">
+        <v>0</v>
+      </c>
+      <c r="E159" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>posible_victoria_favorito</t>
+        </is>
+      </c>
+      <c r="C160" t="n">
+        <v>1</v>
+      </c>
+      <c r="D160" t="n">
+        <v>0</v>
+      </c>
+      <c r="E160" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>cuidado_rival_presiona</t>
+        </is>
+      </c>
+      <c r="C161" t="n">
+        <v>1</v>
+      </c>
+      <c r="D161" t="n">
+        <v>0</v>
+      </c>
+      <c r="E161" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-10-11
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L260"/>
+  <dimension ref="A1:L293"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13943,6 +13943,1722 @@
         <v>0</v>
       </c>
       <c r="L260" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>Manchester United vs Tottenham Hotspur</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>Manchester United</t>
+        </is>
+      </c>
+      <c r="D261" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E261" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="F261" t="n">
+        <v>68.8</v>
+      </c>
+      <c r="G261" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H261" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I261" t="n">
+        <v>0</v>
+      </c>
+      <c r="J261" t="n">
+        <v>5</v>
+      </c>
+      <c r="K261" t="n">
+        <v>0</v>
+      </c>
+      <c r="L261" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>Middlesbrough vs Wolverhampton Wanderers</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>Middlesbrough</t>
+        </is>
+      </c>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E262" t="n">
+        <v>1.68</v>
+      </c>
+      <c r="F262" t="n">
+        <v>59.5</v>
+      </c>
+      <c r="G262" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H262" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I262" t="n">
+        <v>0</v>
+      </c>
+      <c r="J262" t="n">
+        <v>1</v>
+      </c>
+      <c r="K262" t="n">
+        <v>2</v>
+      </c>
+      <c r="L262" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>Sheffield United vs Lincoln City</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>Sheffield United</t>
+        </is>
+      </c>
+      <c r="D263" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E263" t="n">
+        <v>2.46</v>
+      </c>
+      <c r="F263" t="n">
+        <v>40.6</v>
+      </c>
+      <c r="G263" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="H263" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I263" t="n">
+        <v>0</v>
+      </c>
+      <c r="J263" t="n">
+        <v>2</v>
+      </c>
+      <c r="K263" t="n">
+        <v>0</v>
+      </c>
+      <c r="L263" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>Watford vs Burnley</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>Burnley</t>
+        </is>
+      </c>
+      <c r="D264" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E264" t="n">
+        <v>1.87</v>
+      </c>
+      <c r="F264" t="n">
+        <v>53.5</v>
+      </c>
+      <c r="G264" t="inlineStr">
+        <is>
+          <t>0-4</t>
+        </is>
+      </c>
+      <c r="H264" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I264" t="n">
+        <v>0</v>
+      </c>
+      <c r="J264" t="n">
+        <v>5</v>
+      </c>
+      <c r="K264" t="n">
+        <v>1</v>
+      </c>
+      <c r="L264" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>Barcelona vs Getafe</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>Barcelona</t>
+        </is>
+      </c>
+      <c r="D265" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E265" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="F265" t="n">
+        <v>89.2</v>
+      </c>
+      <c r="G265" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="H265" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I265" t="n">
+        <v>0</v>
+      </c>
+      <c r="J265" t="n">
+        <v>8</v>
+      </c>
+      <c r="K265" t="n">
+        <v>2</v>
+      </c>
+      <c r="L265" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>Real Madrid vs Villarreal</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>Real Madrid</t>
+        </is>
+      </c>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E266" t="n">
+        <v>2.03</v>
+      </c>
+      <c r="F266" t="n">
+        <v>49.2</v>
+      </c>
+      <c r="G266" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H266" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I266" t="n">
+        <v>4</v>
+      </c>
+      <c r="J266" t="n">
+        <v>5</v>
+      </c>
+      <c r="K266" t="n">
+        <v>3</v>
+      </c>
+      <c r="L266" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>Internazionale vs Parma</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>Internazionale</t>
+        </is>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E267" t="n">
+        <v>1.69</v>
+      </c>
+      <c r="F267" t="n">
+        <v>59.2</v>
+      </c>
+      <c r="G267" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="H267" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I267" t="n">
+        <v>0</v>
+      </c>
+      <c r="J267" t="n">
+        <v>2</v>
+      </c>
+      <c r="K267" t="n">
+        <v>2</v>
+      </c>
+      <c r="L267" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>FC Augsburg vs Bayern Munich</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>Bayern Munich</t>
+        </is>
+      </c>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E268" t="n">
+        <v>1.26</v>
+      </c>
+      <c r="F268" t="n">
+        <v>79.59999999999999</v>
+      </c>
+      <c r="G268" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="H268" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I268" t="n">
+        <v>0</v>
+      </c>
+      <c r="J268" t="n">
+        <v>2</v>
+      </c>
+      <c r="K268" t="n">
+        <v>4</v>
+      </c>
+      <c r="L268" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>SC Paderborn 07 vs VfB Stuttgart</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>VfB Stuttgart</t>
+        </is>
+      </c>
+      <c r="D269" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E269" t="n">
+        <v>2.16</v>
+      </c>
+      <c r="F269" t="n">
+        <v>46.3</v>
+      </c>
+      <c r="G269" t="inlineStr">
+        <is>
+          <t>0-2</t>
+        </is>
+      </c>
+      <c r="H269" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I269" t="n">
+        <v>0</v>
+      </c>
+      <c r="J269" t="n">
+        <v>1</v>
+      </c>
+      <c r="K269" t="n">
+        <v>0</v>
+      </c>
+      <c r="L269" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>TSG Hoffenheim vs Hamburg SV</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>TSG Hoffenheim</t>
+        </is>
+      </c>
+      <c r="D270" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E270" t="n">
+        <v>1.66</v>
+      </c>
+      <c r="F270" t="n">
+        <v>60.2</v>
+      </c>
+      <c r="G270" t="inlineStr">
+        <is>
+          <t>2-3</t>
+        </is>
+      </c>
+      <c r="H270" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I270" t="n">
+        <v>0</v>
+      </c>
+      <c r="J270" t="n">
+        <v>2</v>
+      </c>
+      <c r="K270" t="n">
+        <v>2</v>
+      </c>
+      <c r="L270" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>Paris Saint-Germain vs Le Mans</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>Paris Saint-Germain</t>
+        </is>
+      </c>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E271" t="n">
+        <v>2.48</v>
+      </c>
+      <c r="F271" t="n">
+        <v>40.4</v>
+      </c>
+      <c r="G271" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="H271" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I271" t="n">
+        <v>4</v>
+      </c>
+      <c r="J271" t="n">
+        <v>4</v>
+      </c>
+      <c r="K271" t="n">
+        <v>3</v>
+      </c>
+      <c r="L271" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>Fortuna Sittard vs FC Twente</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>FC Twente</t>
+        </is>
+      </c>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E272" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="F272" t="n">
+        <v>77.2</v>
+      </c>
+      <c r="G272" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H272" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I272" t="n">
+        <v>0</v>
+      </c>
+      <c r="J272" t="n">
+        <v>2</v>
+      </c>
+      <c r="K272" t="n">
+        <v>4</v>
+      </c>
+      <c r="L272" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>Ajax Amsterdam vs NEC Nijmegen</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>Ajax Amsterdam</t>
+        </is>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E273" t="n">
+        <v>1.83</v>
+      </c>
+      <c r="F273" t="n">
+        <v>54.8</v>
+      </c>
+      <c r="G273" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H273" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I273" t="n">
+        <v>6</v>
+      </c>
+      <c r="J273" t="n">
+        <v>5</v>
+      </c>
+      <c r="K273" t="n">
+        <v>3</v>
+      </c>
+      <c r="L273" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>Maritimo vs FC Porto</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>FC Porto</t>
+        </is>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E274" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="F274" t="n">
+        <v>52.5</v>
+      </c>
+      <c r="G274" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H274" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I274" t="n">
+        <v>0</v>
+      </c>
+      <c r="J274" t="n">
+        <v>1</v>
+      </c>
+      <c r="K274" t="n">
+        <v>1</v>
+      </c>
+      <c r="L274" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>RAAL La Louvière vs Club Brugge</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>Club Brugge</t>
+        </is>
+      </c>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E275" t="n">
+        <v>1.14</v>
+      </c>
+      <c r="F275" t="n">
+        <v>87.59999999999999</v>
+      </c>
+      <c r="G275" t="inlineStr">
+        <is>
+          <t>1-4</t>
+        </is>
+      </c>
+      <c r="H275" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I275" t="n">
+        <v>0</v>
+      </c>
+      <c r="J275" t="n">
+        <v>0</v>
+      </c>
+      <c r="K275" t="n">
+        <v>4</v>
+      </c>
+      <c r="L275" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>Racing Genk vs KV Kortrijk</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>Racing Genk</t>
+        </is>
+      </c>
+      <c r="D276" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E276" t="n">
+        <v>2.13</v>
+      </c>
+      <c r="F276" t="n">
+        <v>47</v>
+      </c>
+      <c r="G276" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="H276" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I276" t="n">
+        <v>3</v>
+      </c>
+      <c r="J276" t="n">
+        <v>1</v>
+      </c>
+      <c r="K276" t="n">
+        <v>1</v>
+      </c>
+      <c r="L276" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>AEK Athens vs OFI Crete</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>AEK Athens</t>
+        </is>
+      </c>
+      <c r="D277" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E277" t="n">
+        <v>2.13</v>
+      </c>
+      <c r="F277" t="n">
+        <v>47</v>
+      </c>
+      <c r="G277" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="H277" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I277" t="n">
+        <v>0</v>
+      </c>
+      <c r="J277" t="n">
+        <v>4</v>
+      </c>
+      <c r="K277" t="n">
+        <v>4</v>
+      </c>
+      <c r="L277" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>Vasco da Gama vs Remo</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>Vasco da Gama</t>
+        </is>
+      </c>
+      <c r="D278" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E278" t="n">
+        <v>1.69</v>
+      </c>
+      <c r="F278" t="n">
+        <v>59.1</v>
+      </c>
+      <c r="G278" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H278" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I278" t="n">
+        <v>6</v>
+      </c>
+      <c r="J278" t="n">
+        <v>2</v>
+      </c>
+      <c r="K278" t="n">
+        <v>4</v>
+      </c>
+      <c r="L278" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>River Plate vs Estudiantes de Río Cuarto</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>River Plate</t>
+        </is>
+      </c>
+      <c r="D279" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E279" t="n">
+        <v>1.87</v>
+      </c>
+      <c r="F279" t="n">
+        <v>53.5</v>
+      </c>
+      <c r="G279" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H279" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I279" t="n">
+        <v>1</v>
+      </c>
+      <c r="J279" t="n">
+        <v>0</v>
+      </c>
+      <c r="K279" t="n">
+        <v>2</v>
+      </c>
+      <c r="L279" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>Philadelphia Union vs Real Salt Lake</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>Philadelphia Union</t>
+        </is>
+      </c>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E280" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="F280" t="n">
+        <v>61.2</v>
+      </c>
+      <c r="G280" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H280" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I280" t="n">
+        <v>1</v>
+      </c>
+      <c r="J280" t="n">
+        <v>1</v>
+      </c>
+      <c r="K280" t="n">
+        <v>2</v>
+      </c>
+      <c r="L280" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>Austin FC vs Nashville SC</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>Austin FC</t>
+        </is>
+      </c>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E281" t="n">
+        <v>2.01</v>
+      </c>
+      <c r="F281" t="n">
+        <v>49.7</v>
+      </c>
+      <c r="G281" t="inlineStr">
+        <is>
+          <t>1-4</t>
+        </is>
+      </c>
+      <c r="H281" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I281" t="n">
+        <v>0</v>
+      </c>
+      <c r="J281" t="n">
+        <v>1</v>
+      </c>
+      <c r="K281" t="n">
+        <v>1</v>
+      </c>
+      <c r="L281" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>Arsenal vs Leeds United</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>Arsenal</t>
+        </is>
+      </c>
+      <c r="D282" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E282" t="n">
+        <v>1.21</v>
+      </c>
+      <c r="F282" t="n">
+        <v>82.59999999999999</v>
+      </c>
+      <c r="G282" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H282" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I282" t="n">
+        <v>0</v>
+      </c>
+      <c r="J282" t="n">
+        <v>3</v>
+      </c>
+      <c r="K282" t="n">
+        <v>3</v>
+      </c>
+      <c r="L282" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>Chelsea vs AFC Bournemouth</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>AFC Bournemouth</t>
+        </is>
+      </c>
+      <c r="D283" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E283" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="F283" t="n">
+        <v>60.7</v>
+      </c>
+      <c r="G283" t="inlineStr">
+        <is>
+          <t>5-1</t>
+        </is>
+      </c>
+      <c r="H283" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I283" t="n">
+        <v>0</v>
+      </c>
+      <c r="J283" t="n">
+        <v>3</v>
+      </c>
+      <c r="K283" t="n">
+        <v>0</v>
+      </c>
+      <c r="L283" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>Ipswich Town vs Fulham</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>Ipswich Town</t>
+        </is>
+      </c>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E284" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="F284" t="n">
+        <v>74</v>
+      </c>
+      <c r="G284" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H284" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I284" t="n">
+        <v>0</v>
+      </c>
+      <c r="J284" t="n">
+        <v>2</v>
+      </c>
+      <c r="K284" t="n">
+        <v>3</v>
+      </c>
+      <c r="L284" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>Blackburn Rovers vs Cardiff City</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>Cardiff City</t>
+        </is>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E285" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="F285" t="n">
+        <v>77</v>
+      </c>
+      <c r="G285" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H285" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I285" t="n">
+        <v>0</v>
+      </c>
+      <c r="J285" t="n">
+        <v>2</v>
+      </c>
+      <c r="K285" t="n">
+        <v>3</v>
+      </c>
+      <c r="L285" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>Genoa vs Fiorentina</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>Fiorentina</t>
+        </is>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E286" t="n">
+        <v>2.92</v>
+      </c>
+      <c r="F286" t="n">
+        <v>34.2</v>
+      </c>
+      <c r="G286" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H286" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I286" t="n">
+        <v>0</v>
+      </c>
+      <c r="J286" t="n">
+        <v>1</v>
+      </c>
+      <c r="K286" t="n">
+        <v>0</v>
+      </c>
+      <c r="L286" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>Go Ahead Eagles vs Sparta Rotterdam</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>Go Ahead Eagles</t>
+        </is>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E287" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="F287" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="G287" t="inlineStr">
+        <is>
+          <t>3-3</t>
+        </is>
+      </c>
+      <c r="H287" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I287" t="n">
+        <v>0</v>
+      </c>
+      <c r="J287" t="n">
+        <v>1</v>
+      </c>
+      <c r="K287" t="n">
+        <v>5</v>
+      </c>
+      <c r="L287" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>Feyenoord Rotterdam vs AZ Alkmaar</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>Feyenoord Rotterdam</t>
+        </is>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E288" t="n">
+        <v>1.89</v>
+      </c>
+      <c r="F288" t="n">
+        <v>52.9</v>
+      </c>
+      <c r="G288" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H288" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I288" t="n">
+        <v>0</v>
+      </c>
+      <c r="J288" t="n">
+        <v>4</v>
+      </c>
+      <c r="K288" t="n">
+        <v>3</v>
+      </c>
+      <c r="L288" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>Académico de Viseu vs Estoril</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>Académico de Viseu</t>
+        </is>
+      </c>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E289" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F289" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="G289" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H289" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I289" t="n">
+        <v>3</v>
+      </c>
+      <c r="J289" t="n">
+        <v>1</v>
+      </c>
+      <c r="K289" t="n">
+        <v>2</v>
+      </c>
+      <c r="L289" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>Zulte-Waregem vs KAA Gent</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>Zulte-Waregem</t>
+        </is>
+      </c>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E290" t="n">
+        <v>1.26</v>
+      </c>
+      <c r="F290" t="n">
+        <v>79.09999999999999</v>
+      </c>
+      <c r="G290" t="inlineStr">
+        <is>
+          <t>0-2</t>
+        </is>
+      </c>
+      <c r="H290" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I290" t="n">
+        <v>2</v>
+      </c>
+      <c r="J290" t="n">
+        <v>2</v>
+      </c>
+      <c r="K290" t="n">
+        <v>2</v>
+      </c>
+      <c r="L290" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>Asteras Tripoli vs Atromitos</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>Atromitos</t>
+        </is>
+      </c>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E291" t="n">
+        <v>2.52</v>
+      </c>
+      <c r="F291" t="n">
+        <v>39.7</v>
+      </c>
+      <c r="G291" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H291" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I291" t="n">
+        <v>0</v>
+      </c>
+      <c r="J291" t="n">
+        <v>2</v>
+      </c>
+      <c r="K291" t="n">
+        <v>1</v>
+      </c>
+      <c r="L291" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>Atlanta United FC vs FC Cincinnati</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>Atlanta United FC</t>
+        </is>
+      </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E292" t="n">
+        <v>1.54</v>
+      </c>
+      <c r="F292" t="n">
+        <v>65</v>
+      </c>
+      <c r="G292" t="inlineStr">
+        <is>
+          <t>1-3</t>
+        </is>
+      </c>
+      <c r="H292" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I292" t="n">
+        <v>2</v>
+      </c>
+      <c r="J292" t="n">
+        <v>0</v>
+      </c>
+      <c r="K292" t="n">
+        <v>2</v>
+      </c>
+      <c r="L292" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>Inter Miami CF vs D.C. United</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>D.C. United</t>
+        </is>
+      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E293" t="n">
+        <v>2.16</v>
+      </c>
+      <c r="F293" t="n">
+        <v>46.4</v>
+      </c>
+      <c r="G293" t="inlineStr">
+        <is>
+          <t>4-0</t>
+        </is>
+      </c>
+      <c r="H293" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I293" t="n">
+        <v>2</v>
+      </c>
+      <c r="J293" t="n">
+        <v>0</v>
+      </c>
+      <c r="K293" t="n">
+        <v>1</v>
+      </c>
+      <c r="L293" t="inlineStr">
         <is>
           <t>si</t>
         </is>
@@ -13959,7 +15675,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E61"/>
+  <dimension ref="A1:E62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15079,6 +16795,25 @@
       </c>
       <c r="E61" t="n">
         <v>4</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>33</v>
+      </c>
+      <c r="C62" t="n">
+        <v>18</v>
+      </c>
+      <c r="D62" t="n">
+        <v>54.5</v>
+      </c>
+      <c r="E62" t="n">
+        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -15092,7 +16827,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E161"/>
+  <dimension ref="A1:E169"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18482,6 +20217,174 @@
         <v>0</v>
       </c>
     </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>alerta_1er_tiempo</t>
+        </is>
+      </c>
+      <c r="C162" t="n">
+        <v>3</v>
+      </c>
+      <c r="D162" t="n">
+        <v>0</v>
+      </c>
+      <c r="E162" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>posible_victoria_favorito</t>
+        </is>
+      </c>
+      <c r="C163" t="n">
+        <v>11</v>
+      </c>
+      <c r="D163" t="n">
+        <v>1</v>
+      </c>
+      <c r="E163" t="n">
+        <v>9.1</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>tarjeta_roja</t>
+        </is>
+      </c>
+      <c r="C164" t="n">
+        <v>3</v>
+      </c>
+      <c r="D164" t="n">
+        <v>0</v>
+      </c>
+      <c r="E164" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>penal</t>
+        </is>
+      </c>
+      <c r="C165" t="n">
+        <v>2</v>
+      </c>
+      <c r="D165" t="n">
+        <v>0</v>
+      </c>
+      <c r="E165" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>ampliacion_marcador</t>
+        </is>
+      </c>
+      <c r="C166" t="n">
+        <v>6</v>
+      </c>
+      <c r="D166" t="n">
+        <v>2</v>
+      </c>
+      <c r="E166" t="n">
+        <v>33.3</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>cuidado_rival_presiona</t>
+        </is>
+      </c>
+      <c r="C167" t="n">
+        <v>6</v>
+      </c>
+      <c r="D167" t="n">
+        <v>1</v>
+      </c>
+      <c r="E167" t="n">
+        <v>16.7</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>partido_resuelto</t>
+        </is>
+      </c>
+      <c r="C168" t="n">
+        <v>2</v>
+      </c>
+      <c r="D168" t="n">
+        <v>0</v>
+      </c>
+      <c r="E168" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>posible_empate</t>
+        </is>
+      </c>
+      <c r="C169" t="n">
+        <v>1</v>
+      </c>
+      <c r="D169" t="n">
+        <v>0</v>
+      </c>
+      <c r="E169" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-10-12
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L293"/>
+  <dimension ref="A1:L319"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15659,6 +15659,1358 @@
         <v>1</v>
       </c>
       <c r="L293" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>Hull City vs Everton</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>Hull City</t>
+        </is>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E294" t="n">
+        <v>1.73</v>
+      </c>
+      <c r="F294" t="n">
+        <v>57.7</v>
+      </c>
+      <c r="G294" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="H294" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I294" t="n">
+        <v>0</v>
+      </c>
+      <c r="J294" t="n">
+        <v>1</v>
+      </c>
+      <c r="K294" t="n">
+        <v>1</v>
+      </c>
+      <c r="L294" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>Real Sociedad vs Deportivo</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>Real Sociedad</t>
+        </is>
+      </c>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E295" t="n">
+        <v>2.71</v>
+      </c>
+      <c r="F295" t="n">
+        <v>36.9</v>
+      </c>
+      <c r="G295" t="inlineStr">
+        <is>
+          <t>3-2</t>
+        </is>
+      </c>
+      <c r="H295" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I295" t="n">
+        <v>0</v>
+      </c>
+      <c r="J295" t="n">
+        <v>0</v>
+      </c>
+      <c r="K295" t="n">
+        <v>5</v>
+      </c>
+      <c r="L295" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>Como vs AS Roma</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>Como</t>
+        </is>
+      </c>
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E296" t="n">
+        <v>2.44</v>
+      </c>
+      <c r="F296" t="n">
+        <v>41</v>
+      </c>
+      <c r="G296" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H296" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I296" t="n">
+        <v>0</v>
+      </c>
+      <c r="J296" t="n">
+        <v>2</v>
+      </c>
+      <c r="K296" t="n">
+        <v>0</v>
+      </c>
+      <c r="L296" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>Nice vs Strasbourg</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>Strasbourg</t>
+        </is>
+      </c>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E297" t="n">
+        <v>2.28</v>
+      </c>
+      <c r="F297" t="n">
+        <v>43.8</v>
+      </c>
+      <c r="G297" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H297" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I297" t="n">
+        <v>0</v>
+      </c>
+      <c r="J297" t="n">
+        <v>4</v>
+      </c>
+      <c r="K297" t="n">
+        <v>1</v>
+      </c>
+      <c r="L297" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>Stade Rennais vs AJ Auxerre</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>Stade Rennais</t>
+        </is>
+      </c>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E298" t="n">
+        <v>2.68</v>
+      </c>
+      <c r="F298" t="n">
+        <v>37.3</v>
+      </c>
+      <c r="G298" t="inlineStr">
+        <is>
+          <t>4-1</t>
+        </is>
+      </c>
+      <c r="H298" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I298" t="n">
+        <v>0</v>
+      </c>
+      <c r="J298" t="n">
+        <v>1</v>
+      </c>
+      <c r="K298" t="n">
+        <v>2</v>
+      </c>
+      <c r="L298" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>FC Utrecht vs Willem II</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>FC Utrecht</t>
+        </is>
+      </c>
+      <c r="D299" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E299" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="F299" t="n">
+        <v>61.3</v>
+      </c>
+      <c r="G299" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="H299" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I299" t="n">
+        <v>0</v>
+      </c>
+      <c r="J299" t="n">
+        <v>4</v>
+      </c>
+      <c r="K299" t="n">
+        <v>4</v>
+      </c>
+      <c r="L299" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>PEC Zwolle vs SC Cambuur</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>SC Cambuur</t>
+        </is>
+      </c>
+      <c r="D300" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E300" t="n">
+        <v>1.72</v>
+      </c>
+      <c r="F300" t="n">
+        <v>58</v>
+      </c>
+      <c r="G300" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H300" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I300" t="n">
+        <v>0</v>
+      </c>
+      <c r="J300" t="n">
+        <v>3</v>
+      </c>
+      <c r="K300" t="n">
+        <v>2</v>
+      </c>
+      <c r="L300" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>Benfica vs Vitória de Guimaraes</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>Benfica</t>
+        </is>
+      </c>
+      <c r="D301" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E301" t="n">
+        <v>1.14</v>
+      </c>
+      <c r="F301" t="n">
+        <v>87.40000000000001</v>
+      </c>
+      <c r="G301" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H301" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I301" t="n">
+        <v>0</v>
+      </c>
+      <c r="J301" t="n">
+        <v>6</v>
+      </c>
+      <c r="K301" t="n">
+        <v>5</v>
+      </c>
+      <c r="L301" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>Union St.-Gilloise vs OH Leuven</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>Union St.-Gilloise</t>
+        </is>
+      </c>
+      <c r="D302" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E302" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="F302" t="n">
+        <v>81.90000000000001</v>
+      </c>
+      <c r="G302" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H302" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I302" t="n">
+        <v>0</v>
+      </c>
+      <c r="J302" t="n">
+        <v>3</v>
+      </c>
+      <c r="K302" t="n">
+        <v>0</v>
+      </c>
+      <c r="L302" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>Besiktas vs Kocaelispor</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>Besiktas</t>
+        </is>
+      </c>
+      <c r="D303" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E303" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="F303" t="n">
+        <v>81.90000000000001</v>
+      </c>
+      <c r="G303" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H303" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I303" t="n">
+        <v>0</v>
+      </c>
+      <c r="J303" t="n">
+        <v>2</v>
+      </c>
+      <c r="K303" t="n">
+        <v>1</v>
+      </c>
+      <c r="L303" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>Iraklis vs Levadiakos</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>Iraklis</t>
+        </is>
+      </c>
+      <c r="D304" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E304" t="n">
+        <v>2.17</v>
+      </c>
+      <c r="F304" t="n">
+        <v>46.2</v>
+      </c>
+      <c r="G304" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H304" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I304" t="n">
+        <v>0</v>
+      </c>
+      <c r="J304" t="n">
+        <v>0</v>
+      </c>
+      <c r="K304" t="n">
+        <v>2</v>
+      </c>
+      <c r="L304" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>Aris vs Volos NFC</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>Aris</t>
+        </is>
+      </c>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E305" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="F305" t="n">
+        <v>89.40000000000001</v>
+      </c>
+      <c r="G305" t="inlineStr">
+        <is>
+          <t>3-2</t>
+        </is>
+      </c>
+      <c r="H305" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I305" t="n">
+        <v>0</v>
+      </c>
+      <c r="J305" t="n">
+        <v>2</v>
+      </c>
+      <c r="K305" t="n">
+        <v>3</v>
+      </c>
+      <c r="L305" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>Olympiacos vs Panathinaikos</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>Olympiacos</t>
+        </is>
+      </c>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E306" t="n">
+        <v>1.76</v>
+      </c>
+      <c r="F306" t="n">
+        <v>56.7</v>
+      </c>
+      <c r="G306" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H306" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I306" t="n">
+        <v>1</v>
+      </c>
+      <c r="J306" t="n">
+        <v>5</v>
+      </c>
+      <c r="K306" t="n">
+        <v>3</v>
+      </c>
+      <c r="L306" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>Atlético de San Luis vs Santos</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>Atlético de San Luis</t>
+        </is>
+      </c>
+      <c r="D307" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E307" t="n">
+        <v>2.17</v>
+      </c>
+      <c r="F307" t="n">
+        <v>46</v>
+      </c>
+      <c r="G307" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H307" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I307" t="n">
+        <v>4</v>
+      </c>
+      <c r="J307" t="n">
+        <v>0</v>
+      </c>
+      <c r="K307" t="n">
+        <v>1</v>
+      </c>
+      <c r="L307" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>Crystal Palace vs Nottingham Forest</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>Nottingham Forest</t>
+        </is>
+      </c>
+      <c r="D308" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E308" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="F308" t="n">
+        <v>76.90000000000001</v>
+      </c>
+      <c r="G308" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="H308" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I308" t="n">
+        <v>0</v>
+      </c>
+      <c r="J308" t="n">
+        <v>4</v>
+      </c>
+      <c r="K308" t="n">
+        <v>0</v>
+      </c>
+      <c r="L308" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>Liverpool vs Manchester City</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>Manchester City</t>
+        </is>
+      </c>
+      <c r="D309" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E309" t="n">
+        <v>1.49</v>
+      </c>
+      <c r="F309" t="n">
+        <v>67.09999999999999</v>
+      </c>
+      <c r="G309" t="inlineStr">
+        <is>
+          <t>0-3</t>
+        </is>
+      </c>
+      <c r="H309" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I309" t="n">
+        <v>0</v>
+      </c>
+      <c r="J309" t="n">
+        <v>0</v>
+      </c>
+      <c r="K309" t="n">
+        <v>2</v>
+      </c>
+      <c r="L309" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>Elche vs Celta Vigo</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>Celta Vigo</t>
+        </is>
+      </c>
+      <c r="D310" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E310" t="n">
+        <v>2.45</v>
+      </c>
+      <c r="F310" t="n">
+        <v>40.8</v>
+      </c>
+      <c r="G310" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H310" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I310" t="n">
+        <v>0</v>
+      </c>
+      <c r="J310" t="n">
+        <v>6</v>
+      </c>
+      <c r="K310" t="n">
+        <v>2</v>
+      </c>
+      <c r="L310" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>Real Betis vs Osasuna</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>Real Betis</t>
+        </is>
+      </c>
+      <c r="D311" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E311" t="n">
+        <v>1.21</v>
+      </c>
+      <c r="F311" t="n">
+        <v>82.59999999999999</v>
+      </c>
+      <c r="G311" t="inlineStr">
+        <is>
+          <t>5-2</t>
+        </is>
+      </c>
+      <c r="H311" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I311" t="n">
+        <v>0</v>
+      </c>
+      <c r="J311" t="n">
+        <v>2</v>
+      </c>
+      <c r="K311" t="n">
+        <v>3</v>
+      </c>
+      <c r="L311" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>Racing Santander vs Valencia</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>Racing Santander</t>
+        </is>
+      </c>
+      <c r="D312" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E312" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="F312" t="n">
+        <v>75.09999999999999</v>
+      </c>
+      <c r="G312" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="H312" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I312" t="n">
+        <v>4</v>
+      </c>
+      <c r="J312" t="n">
+        <v>4</v>
+      </c>
+      <c r="K312" t="n">
+        <v>2</v>
+      </c>
+      <c r="L312" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>Almería vs Leganés</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>Almería</t>
+        </is>
+      </c>
+      <c r="D313" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E313" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="F313" t="n">
+        <v>84.59999999999999</v>
+      </c>
+      <c r="G313" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="H313" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I313" t="n">
+        <v>0</v>
+      </c>
+      <c r="J313" t="n">
+        <v>1</v>
+      </c>
+      <c r="K313" t="n">
+        <v>1</v>
+      </c>
+      <c r="L313" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>FC Cologne vs Borussia Mönchengladbach</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>Borussia Mönchengladbach</t>
+        </is>
+      </c>
+      <c r="D314" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E314" t="n">
+        <v>2.17</v>
+      </c>
+      <c r="F314" t="n">
+        <v>46.1</v>
+      </c>
+      <c r="G314" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H314" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I314" t="n">
+        <v>0</v>
+      </c>
+      <c r="J314" t="n">
+        <v>1</v>
+      </c>
+      <c r="K314" t="n">
+        <v>0</v>
+      </c>
+      <c r="L314" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>Troyes vs Marseille</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>Troyes</t>
+        </is>
+      </c>
+      <c r="D315" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E315" t="n">
+        <v>1.39</v>
+      </c>
+      <c r="F315" t="n">
+        <v>72.09999999999999</v>
+      </c>
+      <c r="G315" t="inlineStr">
+        <is>
+          <t>0-2</t>
+        </is>
+      </c>
+      <c r="H315" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I315" t="n">
+        <v>3</v>
+      </c>
+      <c r="J315" t="n">
+        <v>0</v>
+      </c>
+      <c r="K315" t="n">
+        <v>2</v>
+      </c>
+      <c r="L315" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>Telstar vs ADO Den Haag</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>Telstar</t>
+        </is>
+      </c>
+      <c r="D316" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E316" t="n">
+        <v>2.61</v>
+      </c>
+      <c r="F316" t="n">
+        <v>38.3</v>
+      </c>
+      <c r="G316" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="H316" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I316" t="n">
+        <v>0</v>
+      </c>
+      <c r="J316" t="n">
+        <v>6</v>
+      </c>
+      <c r="K316" t="n">
+        <v>3</v>
+      </c>
+      <c r="L316" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>Arouca vs Estrela</t>
+        </is>
+      </c>
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>Arouca</t>
+        </is>
+      </c>
+      <c r="D317" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E317" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="F317" t="n">
+        <v>69</v>
+      </c>
+      <c r="G317" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H317" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I317" t="n">
+        <v>3</v>
+      </c>
+      <c r="J317" t="n">
+        <v>1</v>
+      </c>
+      <c r="K317" t="n">
+        <v>0</v>
+      </c>
+      <c r="L317" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>KV Mechelen vs Sint-Truidense</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>Sint-Truidense</t>
+        </is>
+      </c>
+      <c r="D318" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E318" t="n">
+        <v>1.53</v>
+      </c>
+      <c r="F318" t="n">
+        <v>65.2</v>
+      </c>
+      <c r="G318" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="H318" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I318" t="n">
+        <v>0</v>
+      </c>
+      <c r="J318" t="n">
+        <v>0</v>
+      </c>
+      <c r="K318" t="n">
+        <v>1</v>
+      </c>
+      <c r="L318" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>Flamengo vs Fluminense</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>Flamengo</t>
+        </is>
+      </c>
+      <c r="D319" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E319" t="n">
+        <v>1.41</v>
+      </c>
+      <c r="F319" t="n">
+        <v>71.09999999999999</v>
+      </c>
+      <c r="G319" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H319" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I319" t="n">
+        <v>3</v>
+      </c>
+      <c r="J319" t="n">
+        <v>5</v>
+      </c>
+      <c r="K319" t="n">
+        <v>5</v>
+      </c>
+      <c r="L319" t="inlineStr">
         <is>
           <t>si</t>
         </is>
@@ -15675,7 +17027,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E62"/>
+  <dimension ref="A1:E63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16814,6 +18166,25 @@
       </c>
       <c r="E62" t="n">
         <v>33</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>26</v>
+      </c>
+      <c r="C63" t="n">
+        <v>14</v>
+      </c>
+      <c r="D63" t="n">
+        <v>53.8</v>
+      </c>
+      <c r="E63" t="n">
+        <v>26</v>
       </c>
     </row>
   </sheetData>
@@ -16827,7 +18198,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E169"/>
+  <dimension ref="A1:E177"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20385,6 +21756,174 @@
         <v>0</v>
       </c>
     </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>tarjeta_roja</t>
+        </is>
+      </c>
+      <c r="C170" t="n">
+        <v>1</v>
+      </c>
+      <c r="D170" t="n">
+        <v>0</v>
+      </c>
+      <c r="E170" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>ampliacion_marcador</t>
+        </is>
+      </c>
+      <c r="C171" t="n">
+        <v>2</v>
+      </c>
+      <c r="D171" t="n">
+        <v>0</v>
+      </c>
+      <c r="E171" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>posible_victoria_favorito</t>
+        </is>
+      </c>
+      <c r="C172" t="n">
+        <v>4</v>
+      </c>
+      <c r="D172" t="n">
+        <v>2</v>
+      </c>
+      <c r="E172" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>cuidado_rival_presiona</t>
+        </is>
+      </c>
+      <c r="C173" t="n">
+        <v>5</v>
+      </c>
+      <c r="D173" t="n">
+        <v>0</v>
+      </c>
+      <c r="E173" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>gol_de_cierre</t>
+        </is>
+      </c>
+      <c r="C174" t="n">
+        <v>2</v>
+      </c>
+      <c r="D174" t="n">
+        <v>0</v>
+      </c>
+      <c r="E174" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>posible_empate</t>
+        </is>
+      </c>
+      <c r="C175" t="n">
+        <v>2</v>
+      </c>
+      <c r="D175" t="n">
+        <v>0</v>
+      </c>
+      <c r="E175" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>penal</t>
+        </is>
+      </c>
+      <c r="C176" t="n">
+        <v>1</v>
+      </c>
+      <c r="D176" t="n">
+        <v>0</v>
+      </c>
+      <c r="E176" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>alerta_1er_tiempo</t>
+        </is>
+      </c>
+      <c r="C177" t="n">
+        <v>1</v>
+      </c>
+      <c r="D177" t="n">
+        <v>0</v>
+      </c>
+      <c r="E177" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-10-13
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L319"/>
+  <dimension ref="A1:L326"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17011,6 +17011,370 @@
         <v>5</v>
       </c>
       <c r="L319" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>PAOK vs Kalamata</t>
+        </is>
+      </c>
+      <c r="C320" t="inlineStr">
+        <is>
+          <t>PAOK</t>
+        </is>
+      </c>
+      <c r="D320" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E320" t="n">
+        <v>2</v>
+      </c>
+      <c r="F320" t="n">
+        <v>50.1</v>
+      </c>
+      <c r="G320" t="inlineStr">
+        <is>
+          <t>1-3</t>
+        </is>
+      </c>
+      <c r="H320" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I320" t="n">
+        <v>0</v>
+      </c>
+      <c r="J320" t="n">
+        <v>0</v>
+      </c>
+      <c r="K320" t="n">
+        <v>2</v>
+      </c>
+      <c r="L320" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>Coritiba vs Botafogo</t>
+        </is>
+      </c>
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>Coritiba</t>
+        </is>
+      </c>
+      <c r="D321" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E321" t="n">
+        <v>2.55</v>
+      </c>
+      <c r="F321" t="n">
+        <v>39.2</v>
+      </c>
+      <c r="G321" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H321" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I321" t="n">
+        <v>0</v>
+      </c>
+      <c r="J321" t="n">
+        <v>3</v>
+      </c>
+      <c r="K321" t="n">
+        <v>1</v>
+      </c>
+      <c r="L321" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>Coventry City vs Newcastle United</t>
+        </is>
+      </c>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>Coventry City</t>
+        </is>
+      </c>
+      <c r="D322" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E322" t="n">
+        <v>1.24</v>
+      </c>
+      <c r="F322" t="n">
+        <v>80.90000000000001</v>
+      </c>
+      <c r="G322" t="inlineStr">
+        <is>
+          <t>4-1</t>
+        </is>
+      </c>
+      <c r="H322" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I322" t="n">
+        <v>0</v>
+      </c>
+      <c r="J322" t="n">
+        <v>1</v>
+      </c>
+      <c r="K322" t="n">
+        <v>1</v>
+      </c>
+      <c r="L322" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>Levante vs Sevilla</t>
+        </is>
+      </c>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>Sevilla</t>
+        </is>
+      </c>
+      <c r="D323" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E323" t="n">
+        <v>2.07</v>
+      </c>
+      <c r="F323" t="n">
+        <v>48.3</v>
+      </c>
+      <c r="G323" t="inlineStr">
+        <is>
+          <t>3-3</t>
+        </is>
+      </c>
+      <c r="H323" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I323" t="n">
+        <v>0</v>
+      </c>
+      <c r="J323" t="n">
+        <v>3</v>
+      </c>
+      <c r="K323" t="n">
+        <v>2</v>
+      </c>
+      <c r="L323" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>Burgos vs Granada</t>
+        </is>
+      </c>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>Burgos</t>
+        </is>
+      </c>
+      <c r="D324" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E324" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="F324" t="n">
+        <v>81.7</v>
+      </c>
+      <c r="G324" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H324" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I324" t="n">
+        <v>0</v>
+      </c>
+      <c r="J324" t="n">
+        <v>2</v>
+      </c>
+      <c r="K324" t="n">
+        <v>0</v>
+      </c>
+      <c r="L324" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>Real Oviedo vs Eibar</t>
+        </is>
+      </c>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>Eibar</t>
+        </is>
+      </c>
+      <c r="D325" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E325" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="F325" t="n">
+        <v>67.5</v>
+      </c>
+      <c r="G325" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="H325" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I325" t="n">
+        <v>0</v>
+      </c>
+      <c r="J325" t="n">
+        <v>3</v>
+      </c>
+      <c r="K325" t="n">
+        <v>0</v>
+      </c>
+      <c r="L325" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>FC Famalicao vs Alverca</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>FC Famalicao</t>
+        </is>
+      </c>
+      <c r="D326" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E326" t="n">
+        <v>1.52</v>
+      </c>
+      <c r="F326" t="n">
+        <v>65.8</v>
+      </c>
+      <c r="G326" t="inlineStr">
+        <is>
+          <t>1-4</t>
+        </is>
+      </c>
+      <c r="H326" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I326" t="n">
+        <v>0</v>
+      </c>
+      <c r="J326" t="n">
+        <v>1</v>
+      </c>
+      <c r="K326" t="n">
+        <v>1</v>
+      </c>
+      <c r="L326" t="inlineStr">
         <is>
           <t>si</t>
         </is>
@@ -17027,7 +17391,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E63"/>
+  <dimension ref="A1:E64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18185,6 +18549,25 @@
       </c>
       <c r="E63" t="n">
         <v>26</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>7</v>
+      </c>
+      <c r="C64" t="n">
+        <v>1</v>
+      </c>
+      <c r="D64" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="E64" t="n">
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-10-14
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L326"/>
+  <dimension ref="A1:L334"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17375,6 +17375,422 @@
         <v>1</v>
       </c>
       <c r="L326" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>Arsenal vs Lille</t>
+        </is>
+      </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>Arsenal</t>
+        </is>
+      </c>
+      <c r="D327" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E327" t="n">
+        <v>1.26</v>
+      </c>
+      <c r="F327" t="n">
+        <v>79.59999999999999</v>
+      </c>
+      <c r="G327" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="H327" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I327" t="n">
+        <v>1</v>
+      </c>
+      <c r="J327" t="n">
+        <v>4</v>
+      </c>
+      <c r="K327" t="n">
+        <v>1</v>
+      </c>
+      <c r="L327" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>Galatasaray vs Barcelona</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>Barcelona</t>
+        </is>
+      </c>
+      <c r="D328" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E328" t="n">
+        <v>1.88</v>
+      </c>
+      <c r="F328" t="n">
+        <v>53.1</v>
+      </c>
+      <c r="G328" t="inlineStr">
+        <is>
+          <t>1-4</t>
+        </is>
+      </c>
+      <c r="H328" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I328" t="n">
+        <v>1</v>
+      </c>
+      <c r="J328" t="n">
+        <v>5</v>
+      </c>
+      <c r="K328" t="n">
+        <v>9</v>
+      </c>
+      <c r="L328" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>Viking FK vs Bayern Munich</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>Bayern Munich</t>
+        </is>
+      </c>
+      <c r="D329" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E329" t="n">
+        <v>1.34</v>
+      </c>
+      <c r="F329" t="n">
+        <v>74.5</v>
+      </c>
+      <c r="G329" t="inlineStr">
+        <is>
+          <t>3-3</t>
+        </is>
+      </c>
+      <c r="H329" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I329" t="n">
+        <v>1</v>
+      </c>
+      <c r="J329" t="n">
+        <v>0</v>
+      </c>
+      <c r="K329" t="n">
+        <v>5</v>
+      </c>
+      <c r="L329" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>Cardiff City vs Watford</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>Cardiff City</t>
+        </is>
+      </c>
+      <c r="D330" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E330" t="n">
+        <v>1.13</v>
+      </c>
+      <c r="F330" t="n">
+        <v>88.5</v>
+      </c>
+      <c r="G330" t="inlineStr">
+        <is>
+          <t>5-1</t>
+        </is>
+      </c>
+      <c r="H330" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I330" t="n">
+        <v>0</v>
+      </c>
+      <c r="J330" t="n">
+        <v>4</v>
+      </c>
+      <c r="K330" t="n">
+        <v>6</v>
+      </c>
+      <c r="L330" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>Wolverhampton Wanderers vs Bolton Wanderers</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>Bolton Wanderers</t>
+        </is>
+      </c>
+      <c r="D331" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E331" t="n">
+        <v>2.49</v>
+      </c>
+      <c r="F331" t="n">
+        <v>40.1</v>
+      </c>
+      <c r="G331" t="inlineStr">
+        <is>
+          <t>1-3</t>
+        </is>
+      </c>
+      <c r="H331" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I331" t="n">
+        <v>0</v>
+      </c>
+      <c r="J331" t="n">
+        <v>3</v>
+      </c>
+      <c r="K331" t="n">
+        <v>0</v>
+      </c>
+      <c r="L331" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>Stoke City vs Middlesbrough</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>Middlesbrough</t>
+        </is>
+      </c>
+      <c r="D332" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E332" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="F332" t="n">
+        <v>74</v>
+      </c>
+      <c r="G332" t="inlineStr">
+        <is>
+          <t>2-3</t>
+        </is>
+      </c>
+      <c r="H332" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I332" t="n">
+        <v>1</v>
+      </c>
+      <c r="J332" t="n">
+        <v>1</v>
+      </c>
+      <c r="K332" t="n">
+        <v>2</v>
+      </c>
+      <c r="L332" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>Internazionale vs Club Brugge</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>Club Brugge</t>
+        </is>
+      </c>
+      <c r="D333" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E333" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="F333" t="n">
+        <v>62.5</v>
+      </c>
+      <c r="G333" t="inlineStr">
+        <is>
+          <t>3-4</t>
+        </is>
+      </c>
+      <c r="H333" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I333" t="n">
+        <v>2</v>
+      </c>
+      <c r="J333" t="n">
+        <v>3</v>
+      </c>
+      <c r="K333" t="n">
+        <v>5</v>
+      </c>
+      <c r="L333" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>RB Leipzig vs PSV Eindhoven</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>PSV Eindhoven</t>
+        </is>
+      </c>
+      <c r="D334" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E334" t="n">
+        <v>1.28</v>
+      </c>
+      <c r="F334" t="n">
+        <v>78.40000000000001</v>
+      </c>
+      <c r="G334" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H334" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I334" t="n">
+        <v>1</v>
+      </c>
+      <c r="J334" t="n">
+        <v>3</v>
+      </c>
+      <c r="K334" t="n">
+        <v>6</v>
+      </c>
+      <c r="L334" t="inlineStr">
         <is>
           <t>si</t>
         </is>
@@ -17391,7 +17807,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E64"/>
+  <dimension ref="A1:E65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18568,6 +18984,25 @@
       </c>
       <c r="E64" t="n">
         <v>7</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>8</v>
+      </c>
+      <c r="C65" t="n">
+        <v>6</v>
+      </c>
+      <c r="D65" t="n">
+        <v>75</v>
+      </c>
+      <c r="E65" t="n">
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -18581,7 +19016,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E177"/>
+  <dimension ref="A1:E181"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22307,6 +22742,90 @@
         <v>0</v>
       </c>
     </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>partido_resuelto</t>
+        </is>
+      </c>
+      <c r="C178" t="n">
+        <v>2</v>
+      </c>
+      <c r="D178" t="n">
+        <v>0</v>
+      </c>
+      <c r="E178" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>tarjeta_roja</t>
+        </is>
+      </c>
+      <c r="C179" t="n">
+        <v>1</v>
+      </c>
+      <c r="D179" t="n">
+        <v>0</v>
+      </c>
+      <c r="E179" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>ampliacion_marcador</t>
+        </is>
+      </c>
+      <c r="C180" t="n">
+        <v>2</v>
+      </c>
+      <c r="D180" t="n">
+        <v>0</v>
+      </c>
+      <c r="E180" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>penal</t>
+        </is>
+      </c>
+      <c r="C181" t="n">
+        <v>2</v>
+      </c>
+      <c r="D181" t="n">
+        <v>0</v>
+      </c>
+      <c r="E181" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-10-15
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L334"/>
+  <dimension ref="A1:L341"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17791,6 +17791,370 @@
         <v>6</v>
       </c>
       <c r="L334" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>Nashville SC vs Sporting Kansas City</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>Nashville SC</t>
+        </is>
+      </c>
+      <c r="D335" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E335" t="n">
+        <v>1.41</v>
+      </c>
+      <c r="F335" t="n">
+        <v>71</v>
+      </c>
+      <c r="G335" t="inlineStr">
+        <is>
+          <t>4-0</t>
+        </is>
+      </c>
+      <c r="H335" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I335" t="n">
+        <v>1</v>
+      </c>
+      <c r="J335" t="n">
+        <v>2</v>
+      </c>
+      <c r="K335" t="n">
+        <v>3</v>
+      </c>
+      <c r="L335" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>Atlético-MG vs Montevideo City Torque</t>
+        </is>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>Atlético-MG</t>
+        </is>
+      </c>
+      <c r="D336" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E336" t="n">
+        <v>2.29</v>
+      </c>
+      <c r="F336" t="n">
+        <v>43.7</v>
+      </c>
+      <c r="G336" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="H336" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I336" t="n">
+        <v>5</v>
+      </c>
+      <c r="J336" t="n">
+        <v>1</v>
+      </c>
+      <c r="K336" t="n">
+        <v>0</v>
+      </c>
+      <c r="L336" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>Slovan Bratislava vs VfB Stuttgart</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>VfB Stuttgart</t>
+        </is>
+      </c>
+      <c r="D337" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E337" t="n">
+        <v>1.93</v>
+      </c>
+      <c r="F337" t="n">
+        <v>51.7</v>
+      </c>
+      <c r="G337" t="inlineStr">
+        <is>
+          <t>0-3</t>
+        </is>
+      </c>
+      <c r="H337" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I337" t="n">
+        <v>3</v>
+      </c>
+      <c r="J337" t="n">
+        <v>1</v>
+      </c>
+      <c r="K337" t="n">
+        <v>1</v>
+      </c>
+      <c r="L337" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>Toronto FC vs Orlando City SC</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>Orlando City SC</t>
+        </is>
+      </c>
+      <c r="D338" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E338" t="n">
+        <v>1.31</v>
+      </c>
+      <c r="F338" t="n">
+        <v>76.5</v>
+      </c>
+      <c r="G338" t="inlineStr">
+        <is>
+          <t>3-3</t>
+        </is>
+      </c>
+      <c r="H338" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I338" t="n">
+        <v>3</v>
+      </c>
+      <c r="J338" t="n">
+        <v>2</v>
+      </c>
+      <c r="K338" t="n">
+        <v>3</v>
+      </c>
+      <c r="L338" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>Fluminense vs Palmeiras</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>Palmeiras</t>
+        </is>
+      </c>
+      <c r="D339" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E339" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="F339" t="n">
+        <v>72.59999999999999</v>
+      </c>
+      <c r="G339" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H339" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I339" t="n">
+        <v>0</v>
+      </c>
+      <c r="J339" t="n">
+        <v>6</v>
+      </c>
+      <c r="K339" t="n">
+        <v>4</v>
+      </c>
+      <c r="L339" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>LASK Linz vs Liverpool</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>LASK Linz</t>
+        </is>
+      </c>
+      <c r="D340" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E340" t="n">
+        <v>2.24</v>
+      </c>
+      <c r="F340" t="n">
+        <v>44.7</v>
+      </c>
+      <c r="G340" t="inlineStr">
+        <is>
+          <t>3-6</t>
+        </is>
+      </c>
+      <c r="H340" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I340" t="n">
+        <v>0</v>
+      </c>
+      <c r="J340" t="n">
+        <v>0</v>
+      </c>
+      <c r="K340" t="n">
+        <v>1</v>
+      </c>
+      <c r="L340" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>Manchester City vs Paris Saint-Germain</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>Manchester City</t>
+        </is>
+      </c>
+      <c r="D341" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E341" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="F341" t="n">
+        <v>67.3</v>
+      </c>
+      <c r="G341" t="inlineStr">
+        <is>
+          <t>2-4</t>
+        </is>
+      </c>
+      <c r="H341" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I341" t="n">
+        <v>4</v>
+      </c>
+      <c r="J341" t="n">
+        <v>3</v>
+      </c>
+      <c r="K341" t="n">
+        <v>5</v>
+      </c>
+      <c r="L341" t="inlineStr">
         <is>
           <t>si</t>
         </is>
@@ -17807,7 +18171,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E65"/>
+  <dimension ref="A1:E66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19003,6 +19367,25 @@
       </c>
       <c r="E65" t="n">
         <v>8</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>7</v>
+      </c>
+      <c r="C66" t="n">
+        <v>4</v>
+      </c>
+      <c r="D66" t="n">
+        <v>57.1</v>
+      </c>
+      <c r="E66" t="n">
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -19016,7 +19399,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E181"/>
+  <dimension ref="A1:E189"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22826,6 +23209,174 @@
         <v>0</v>
       </c>
     </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>ampliacion_marcador</t>
+        </is>
+      </c>
+      <c r="C182" t="n">
+        <v>5</v>
+      </c>
+      <c r="D182" t="n">
+        <v>1</v>
+      </c>
+      <c r="E182" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>posible_victoria_favorito</t>
+        </is>
+      </c>
+      <c r="C183" t="n">
+        <v>1</v>
+      </c>
+      <c r="D183" t="n">
+        <v>1</v>
+      </c>
+      <c r="E183" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>alerta_1er_tiempo</t>
+        </is>
+      </c>
+      <c r="C184" t="n">
+        <v>1</v>
+      </c>
+      <c r="D184" t="n">
+        <v>1</v>
+      </c>
+      <c r="E184" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>partido_resuelto</t>
+        </is>
+      </c>
+      <c r="C185" t="n">
+        <v>3</v>
+      </c>
+      <c r="D185" t="n">
+        <v>0</v>
+      </c>
+      <c r="E185" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>cuidado_rival_presiona</t>
+        </is>
+      </c>
+      <c r="C186" t="n">
+        <v>2</v>
+      </c>
+      <c r="D186" t="n">
+        <v>1</v>
+      </c>
+      <c r="E186" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>penal</t>
+        </is>
+      </c>
+      <c r="C187" t="n">
+        <v>2</v>
+      </c>
+      <c r="D187" t="n">
+        <v>0</v>
+      </c>
+      <c r="E187" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>posible_empate</t>
+        </is>
+      </c>
+      <c r="C188" t="n">
+        <v>1</v>
+      </c>
+      <c r="D188" t="n">
+        <v>0</v>
+      </c>
+      <c r="E188" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>gol_de_cierre</t>
+        </is>
+      </c>
+      <c r="C189" t="n">
+        <v>1</v>
+      </c>
+      <c r="D189" t="n">
+        <v>0</v>
+      </c>
+      <c r="E189" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-10-16
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L341"/>
+  <dimension ref="A1:L349"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18155,6 +18155,422 @@
         <v>5</v>
       </c>
       <c r="L341" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>AZ Alkmaar vs Hapoel Be'er</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>AZ Alkmaar</t>
+        </is>
+      </c>
+      <c r="D342" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E342" t="n">
+        <v>1.72</v>
+      </c>
+      <c r="F342" t="n">
+        <v>58</v>
+      </c>
+      <c r="G342" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H342" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I342" t="n">
+        <v>0</v>
+      </c>
+      <c r="J342" t="n">
+        <v>4</v>
+      </c>
+      <c r="K342" t="n">
+        <v>0</v>
+      </c>
+      <c r="L342" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>AFC Bournemouth vs SK Sturm Graz</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>AFC Bournemouth</t>
+        </is>
+      </c>
+      <c r="D343" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E343" t="n">
+        <v>2.02</v>
+      </c>
+      <c r="F343" t="n">
+        <v>49.6</v>
+      </c>
+      <c r="G343" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="H343" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I343" t="n">
+        <v>4</v>
+      </c>
+      <c r="J343" t="n">
+        <v>1</v>
+      </c>
+      <c r="K343" t="n">
+        <v>0</v>
+      </c>
+      <c r="L343" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>Benfica vs Celtic</t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t>Benfica</t>
+        </is>
+      </c>
+      <c r="D344" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E344" t="n">
+        <v>1.46</v>
+      </c>
+      <c r="F344" t="n">
+        <v>68.5</v>
+      </c>
+      <c r="G344" t="inlineStr">
+        <is>
+          <t>4-1</t>
+        </is>
+      </c>
+      <c r="H344" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I344" t="n">
+        <v>4</v>
+      </c>
+      <c r="J344" t="n">
+        <v>7</v>
+      </c>
+      <c r="K344" t="n">
+        <v>0</v>
+      </c>
+      <c r="L344" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>Jagiellonia Bialystok vs Ararat-Armenia</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>Jagiellonia Bialystok</t>
+        </is>
+      </c>
+      <c r="D345" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E345" t="n">
+        <v>2.52</v>
+      </c>
+      <c r="F345" t="n">
+        <v>39.7</v>
+      </c>
+      <c r="G345" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="H345" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I345" t="n">
+        <v>3</v>
+      </c>
+      <c r="J345" t="n">
+        <v>1</v>
+      </c>
+      <c r="K345" t="n">
+        <v>0</v>
+      </c>
+      <c r="L345" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>Stade Rennais vs OFI Crete</t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t>Stade Rennais</t>
+        </is>
+      </c>
+      <c r="D346" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E346" t="n">
+        <v>1.83</v>
+      </c>
+      <c r="F346" t="n">
+        <v>54.7</v>
+      </c>
+      <c r="G346" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H346" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I346" t="n">
+        <v>5</v>
+      </c>
+      <c r="J346" t="n">
+        <v>2</v>
+      </c>
+      <c r="K346" t="n">
+        <v>5</v>
+      </c>
+      <c r="L346" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>Lyon vs Crystal Palace</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>Lyon</t>
+        </is>
+      </c>
+      <c r="D347" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E347" t="n">
+        <v>1.37</v>
+      </c>
+      <c r="F347" t="n">
+        <v>73</v>
+      </c>
+      <c r="G347" t="inlineStr">
+        <is>
+          <t>3-2</t>
+        </is>
+      </c>
+      <c r="H347" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I347" t="n">
+        <v>0</v>
+      </c>
+      <c r="J347" t="n">
+        <v>0</v>
+      </c>
+      <c r="K347" t="n">
+        <v>5</v>
+      </c>
+      <c r="L347" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>Torreense vs Sunderland</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>Torreense</t>
+        </is>
+      </c>
+      <c r="D348" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E348" t="n">
+        <v>2.31</v>
+      </c>
+      <c r="F348" t="n">
+        <v>43.3</v>
+      </c>
+      <c r="G348" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H348" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I348" t="n">
+        <v>0</v>
+      </c>
+      <c r="J348" t="n">
+        <v>0</v>
+      </c>
+      <c r="K348" t="n">
+        <v>3</v>
+      </c>
+      <c r="L348" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>Union St.-Gilloise vs Real Sociedad</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>Union St.-Gilloise</t>
+        </is>
+      </c>
+      <c r="D349" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E349" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="F349" t="n">
+        <v>71.59999999999999</v>
+      </c>
+      <c r="G349" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H349" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I349" t="n">
+        <v>0</v>
+      </c>
+      <c r="J349" t="n">
+        <v>4</v>
+      </c>
+      <c r="K349" t="n">
+        <v>1</v>
+      </c>
+      <c r="L349" t="inlineStr">
         <is>
           <t>si</t>
         </is>
@@ -18171,7 +18587,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E66"/>
+  <dimension ref="A1:E67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19386,6 +19802,25 @@
       </c>
       <c r="E66" t="n">
         <v>7</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>8</v>
+      </c>
+      <c r="C67" t="n">
+        <v>6</v>
+      </c>
+      <c r="D67" t="n">
+        <v>75</v>
+      </c>
+      <c r="E67" t="n">
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -19399,7 +19834,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E189"/>
+  <dimension ref="A1:E197"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23377,6 +23812,174 @@
         <v>0</v>
       </c>
     </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>alerta_1er_tiempo</t>
+        </is>
+      </c>
+      <c r="C190" t="n">
+        <v>1</v>
+      </c>
+      <c r="D190" t="n">
+        <v>0</v>
+      </c>
+      <c r="E190" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>posible_victoria_favorito</t>
+        </is>
+      </c>
+      <c r="C191" t="n">
+        <v>1</v>
+      </c>
+      <c r="D191" t="n">
+        <v>1</v>
+      </c>
+      <c r="E191" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>ampliacion_marcador</t>
+        </is>
+      </c>
+      <c r="C192" t="n">
+        <v>6</v>
+      </c>
+      <c r="D192" t="n">
+        <v>2</v>
+      </c>
+      <c r="E192" t="n">
+        <v>33.3</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>partido_resuelto</t>
+        </is>
+      </c>
+      <c r="C193" t="n">
+        <v>2</v>
+      </c>
+      <c r="D193" t="n">
+        <v>0</v>
+      </c>
+      <c r="E193" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>penal</t>
+        </is>
+      </c>
+      <c r="C194" t="n">
+        <v>1</v>
+      </c>
+      <c r="D194" t="n">
+        <v>1</v>
+      </c>
+      <c r="E194" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>cuidado_rival_presiona</t>
+        </is>
+      </c>
+      <c r="C195" t="n">
+        <v>1</v>
+      </c>
+      <c r="D195" t="n">
+        <v>0</v>
+      </c>
+      <c r="E195" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>posible_empate</t>
+        </is>
+      </c>
+      <c r="C196" t="n">
+        <v>3</v>
+      </c>
+      <c r="D196" t="n">
+        <v>1</v>
+      </c>
+      <c r="E196" t="n">
+        <v>33.3</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>gol_de_cierre</t>
+        </is>
+      </c>
+      <c r="C197" t="n">
+        <v>1</v>
+      </c>
+      <c r="D197" t="n">
+        <v>1</v>
+      </c>
+      <c r="E197" t="n">
+        <v>100</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-10-17
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L349"/>
+  <dimension ref="A1:L352"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18571,6 +18571,162 @@
         <v>1</v>
       </c>
       <c r="L349" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>Necaxa vs Atlas</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>Necaxa</t>
+        </is>
+      </c>
+      <c r="D350" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E350" t="n">
+        <v>2.46</v>
+      </c>
+      <c r="F350" t="n">
+        <v>40.6</v>
+      </c>
+      <c r="G350" t="inlineStr">
+        <is>
+          <t>0-2</t>
+        </is>
+      </c>
+      <c r="H350" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I350" t="n">
+        <v>0</v>
+      </c>
+      <c r="J350" t="n">
+        <v>0</v>
+      </c>
+      <c r="K350" t="n">
+        <v>1</v>
+      </c>
+      <c r="L350" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>Tijuana vs Puebla</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>Tijuana</t>
+        </is>
+      </c>
+      <c r="D351" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E351" t="n">
+        <v>2.06</v>
+      </c>
+      <c r="F351" t="n">
+        <v>48.4</v>
+      </c>
+      <c r="G351" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H351" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I351" t="n">
+        <v>0</v>
+      </c>
+      <c r="J351" t="n">
+        <v>0</v>
+      </c>
+      <c r="K351" t="n">
+        <v>1</v>
+      </c>
+      <c r="L351" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>Le Mans vs Toulouse</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>Le Mans</t>
+        </is>
+      </c>
+      <c r="D352" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E352" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="F352" t="n">
+        <v>75</v>
+      </c>
+      <c r="G352" t="inlineStr">
+        <is>
+          <t>0-3</t>
+        </is>
+      </c>
+      <c r="H352" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I352" t="n">
+        <v>4</v>
+      </c>
+      <c r="J352" t="n">
+        <v>4</v>
+      </c>
+      <c r="K352" t="n">
+        <v>0</v>
+      </c>
+      <c r="L352" t="inlineStr">
         <is>
           <t>si</t>
         </is>
@@ -18587,7 +18743,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E67"/>
+  <dimension ref="A1:E68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19821,6 +19977,25 @@
       </c>
       <c r="E67" t="n">
         <v>8</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>3</v>
+      </c>
+      <c r="C68" t="n">
+        <v>0</v>
+      </c>
+      <c r="D68" t="n">
+        <v>0</v>
+      </c>
+      <c r="E68" t="n">
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -19834,7 +20009,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E197"/>
+  <dimension ref="A1:E200"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23980,6 +24155,69 @@
         <v>100</v>
       </c>
     </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>cuidado_rival_presiona</t>
+        </is>
+      </c>
+      <c r="C198" t="n">
+        <v>2</v>
+      </c>
+      <c r="D198" t="n">
+        <v>2</v>
+      </c>
+      <c r="E198" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>partido_resuelto</t>
+        </is>
+      </c>
+      <c r="C199" t="n">
+        <v>1</v>
+      </c>
+      <c r="D199" t="n">
+        <v>0</v>
+      </c>
+      <c r="E199" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>gol_de_cierre</t>
+        </is>
+      </c>
+      <c r="C200" t="n">
+        <v>1</v>
+      </c>
+      <c r="D200" t="n">
+        <v>0</v>
+      </c>
+      <c r="E200" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-10-18
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L352"/>
+  <dimension ref="A1:L381"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18727,6 +18727,1514 @@
         <v>0</v>
       </c>
       <c r="L352" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>Everton vs Chelsea</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>Everton</t>
+        </is>
+      </c>
+      <c r="D353" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E353" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="F353" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="G353" t="inlineStr">
+        <is>
+          <t>0-2</t>
+        </is>
+      </c>
+      <c r="H353" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I353" t="n">
+        <v>0</v>
+      </c>
+      <c r="J353" t="n">
+        <v>2</v>
+      </c>
+      <c r="K353" t="n">
+        <v>4</v>
+      </c>
+      <c r="L353" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>Manchester City vs Ipswich Town</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>Manchester City</t>
+        </is>
+      </c>
+      <c r="D354" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E354" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="F354" t="n">
+        <v>67.59999999999999</v>
+      </c>
+      <c r="G354" t="inlineStr">
+        <is>
+          <t>3-2</t>
+        </is>
+      </c>
+      <c r="H354" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I354" t="n">
+        <v>0</v>
+      </c>
+      <c r="J354" t="n">
+        <v>4</v>
+      </c>
+      <c r="K354" t="n">
+        <v>3</v>
+      </c>
+      <c r="L354" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>Southampton vs Bolton Wanderers</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>Southampton</t>
+        </is>
+      </c>
+      <c r="D355" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E355" t="n">
+        <v>1.86</v>
+      </c>
+      <c r="F355" t="n">
+        <v>53.8</v>
+      </c>
+      <c r="G355" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H355" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I355" t="n">
+        <v>0</v>
+      </c>
+      <c r="J355" t="n">
+        <v>1</v>
+      </c>
+      <c r="K355" t="n">
+        <v>1</v>
+      </c>
+      <c r="L355" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>Villarreal vs Elche</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>Villarreal</t>
+        </is>
+      </c>
+      <c r="D356" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E356" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="F356" t="n">
+        <v>77.09999999999999</v>
+      </c>
+      <c r="G356" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H356" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I356" t="n">
+        <v>0</v>
+      </c>
+      <c r="J356" t="n">
+        <v>4</v>
+      </c>
+      <c r="K356" t="n">
+        <v>7</v>
+      </c>
+      <c r="L356" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>Real Betis vs Barcelona</t>
+        </is>
+      </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>Barcelona</t>
+        </is>
+      </c>
+      <c r="D357" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E357" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="F357" t="n">
+        <v>67.8</v>
+      </c>
+      <c r="G357" t="inlineStr">
+        <is>
+          <t>2-5</t>
+        </is>
+      </c>
+      <c r="H357" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I357" t="n">
+        <v>1</v>
+      </c>
+      <c r="J357" t="n">
+        <v>3</v>
+      </c>
+      <c r="K357" t="n">
+        <v>10</v>
+      </c>
+      <c r="L357" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>Bayern Munich vs RB Leipzig</t>
+        </is>
+      </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>Bayern Munich</t>
+        </is>
+      </c>
+      <c r="D358" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E358" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="F358" t="n">
+        <v>78.40000000000001</v>
+      </c>
+      <c r="G358" t="inlineStr">
+        <is>
+          <t>6-1</t>
+        </is>
+      </c>
+      <c r="H358" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I358" t="n">
+        <v>1</v>
+      </c>
+      <c r="J358" t="n">
+        <v>6</v>
+      </c>
+      <c r="K358" t="n">
+        <v>4</v>
+      </c>
+      <c r="L358" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>Strasbourg vs Paris Saint-Germain</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>Paris Saint-Germain</t>
+        </is>
+      </c>
+      <c r="D359" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E359" t="n">
+        <v>1.64</v>
+      </c>
+      <c r="F359" t="n">
+        <v>60.9</v>
+      </c>
+      <c r="G359" t="inlineStr">
+        <is>
+          <t>1-3</t>
+        </is>
+      </c>
+      <c r="H359" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I359" t="n">
+        <v>0</v>
+      </c>
+      <c r="J359" t="n">
+        <v>2</v>
+      </c>
+      <c r="K359" t="n">
+        <v>6</v>
+      </c>
+      <c r="L359" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>ADO Den Haag vs PSV Eindhoven</t>
+        </is>
+      </c>
+      <c r="C360" t="inlineStr">
+        <is>
+          <t>PSV Eindhoven</t>
+        </is>
+      </c>
+      <c r="D360" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E360" t="n">
+        <v>1.26</v>
+      </c>
+      <c r="F360" t="n">
+        <v>79.59999999999999</v>
+      </c>
+      <c r="G360" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H360" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I360" t="n">
+        <v>0</v>
+      </c>
+      <c r="J360" t="n">
+        <v>4</v>
+      </c>
+      <c r="K360" t="n">
+        <v>7</v>
+      </c>
+      <c r="L360" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>Telstar vs Feyenoord Rotterdam</t>
+        </is>
+      </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>Feyenoord Rotterdam</t>
+        </is>
+      </c>
+      <c r="D361" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E361" t="n">
+        <v>1.31</v>
+      </c>
+      <c r="F361" t="n">
+        <v>76.09999999999999</v>
+      </c>
+      <c r="G361" t="inlineStr">
+        <is>
+          <t>3-4</t>
+        </is>
+      </c>
+      <c r="H361" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I361" t="n">
+        <v>3</v>
+      </c>
+      <c r="J361" t="n">
+        <v>7</v>
+      </c>
+      <c r="K361" t="n">
+        <v>5</v>
+      </c>
+      <c r="L361" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>Sparta Rotterdam vs Willem II</t>
+        </is>
+      </c>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>Willem II</t>
+        </is>
+      </c>
+      <c r="D362" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E362" t="n">
+        <v>2.23</v>
+      </c>
+      <c r="F362" t="n">
+        <v>44.8</v>
+      </c>
+      <c r="G362" t="inlineStr">
+        <is>
+          <t>3-2</t>
+        </is>
+      </c>
+      <c r="H362" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I362" t="n">
+        <v>3</v>
+      </c>
+      <c r="J362" t="n">
+        <v>6</v>
+      </c>
+      <c r="K362" t="n">
+        <v>5</v>
+      </c>
+      <c r="L362" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>Genclerbirligi vs Galatasaray</t>
+        </is>
+      </c>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>Galatasaray</t>
+        </is>
+      </c>
+      <c r="D363" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E363" t="n">
+        <v>1.44</v>
+      </c>
+      <c r="F363" t="n">
+        <v>69.5</v>
+      </c>
+      <c r="G363" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H363" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I363" t="n">
+        <v>0</v>
+      </c>
+      <c r="J363" t="n">
+        <v>0</v>
+      </c>
+      <c r="K363" t="n">
+        <v>6</v>
+      </c>
+      <c r="L363" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>Botafogo vs Chapecoense</t>
+        </is>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>Botafogo</t>
+        </is>
+      </c>
+      <c r="D364" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E364" t="n">
+        <v>1.77</v>
+      </c>
+      <c r="F364" t="n">
+        <v>56.6</v>
+      </c>
+      <c r="G364" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H364" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I364" t="n">
+        <v>5</v>
+      </c>
+      <c r="J364" t="n">
+        <v>2</v>
+      </c>
+      <c r="K364" t="n">
+        <v>2</v>
+      </c>
+      <c r="L364" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>Toluca vs Atlético de San Luis</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>Toluca</t>
+        </is>
+      </c>
+      <c r="D365" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E365" t="n">
+        <v>1.79</v>
+      </c>
+      <c r="F365" t="n">
+        <v>55.8</v>
+      </c>
+      <c r="G365" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H365" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I365" t="n">
+        <v>0</v>
+      </c>
+      <c r="J365" t="n">
+        <v>5</v>
+      </c>
+      <c r="K365" t="n">
+        <v>1</v>
+      </c>
+      <c r="L365" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>Cruz Azul vs FC Juárez</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>Cruz Azul</t>
+        </is>
+      </c>
+      <c r="D366" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E366" t="n">
+        <v>2.03</v>
+      </c>
+      <c r="F366" t="n">
+        <v>49.3</v>
+      </c>
+      <c r="G366" t="inlineStr">
+        <is>
+          <t>5-0</t>
+        </is>
+      </c>
+      <c r="H366" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I366" t="n">
+        <v>0</v>
+      </c>
+      <c r="J366" t="n">
+        <v>0</v>
+      </c>
+      <c r="K366" t="n">
+        <v>1</v>
+      </c>
+      <c r="L366" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>Philadelphia Union vs Charlotte FC</t>
+        </is>
+      </c>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>Philadelphia Union</t>
+        </is>
+      </c>
+      <c r="D367" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E367" t="n">
+        <v>1.62</v>
+      </c>
+      <c r="F367" t="n">
+        <v>61.8</v>
+      </c>
+      <c r="G367" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="H367" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I367" t="n">
+        <v>5</v>
+      </c>
+      <c r="J367" t="n">
+        <v>2</v>
+      </c>
+      <c r="K367" t="n">
+        <v>0</v>
+      </c>
+      <c r="L367" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>Seattle Sounders FC vs CF Montréal</t>
+        </is>
+      </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>Seattle Sounders FC</t>
+        </is>
+      </c>
+      <c r="D368" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E368" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="F368" t="n">
+        <v>55.6</v>
+      </c>
+      <c r="G368" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H368" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I368" t="n">
+        <v>0</v>
+      </c>
+      <c r="J368" t="n">
+        <v>3</v>
+      </c>
+      <c r="K368" t="n">
+        <v>0</v>
+      </c>
+      <c r="L368" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>Middlesbrough vs Cardiff City</t>
+        </is>
+      </c>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t>Middlesbrough</t>
+        </is>
+      </c>
+      <c r="D369" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E369" t="n">
+        <v>2.36</v>
+      </c>
+      <c r="F369" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="G369" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="H369" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I369" t="n">
+        <v>0</v>
+      </c>
+      <c r="J369" t="n">
+        <v>3</v>
+      </c>
+      <c r="K369" t="n">
+        <v>5</v>
+      </c>
+      <c r="L369" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>Millwall vs Lincoln City</t>
+        </is>
+      </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>Millwall</t>
+        </is>
+      </c>
+      <c r="D370" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E370" t="n">
+        <v>1.51</v>
+      </c>
+      <c r="F370" t="n">
+        <v>66.2</v>
+      </c>
+      <c r="G370" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="H370" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I370" t="n">
+        <v>0</v>
+      </c>
+      <c r="J370" t="n">
+        <v>3</v>
+      </c>
+      <c r="K370" t="n">
+        <v>1</v>
+      </c>
+      <c r="L370" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>Watford vs Charlton Athletic</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>Charlton Athletic</t>
+        </is>
+      </c>
+      <c r="D371" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E371" t="n">
+        <v>1.23</v>
+      </c>
+      <c r="F371" t="n">
+        <v>81.09999999999999</v>
+      </c>
+      <c r="G371" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H371" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I371" t="n">
+        <v>0</v>
+      </c>
+      <c r="J371" t="n">
+        <v>7</v>
+      </c>
+      <c r="K371" t="n">
+        <v>1</v>
+      </c>
+      <c r="L371" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>Swansea City vs West Ham United</t>
+        </is>
+      </c>
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>Swansea City</t>
+        </is>
+      </c>
+      <c r="D372" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E372" t="n">
+        <v>1.46</v>
+      </c>
+      <c r="F372" t="n">
+        <v>68.59999999999999</v>
+      </c>
+      <c r="G372" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H372" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I372" t="n">
+        <v>0</v>
+      </c>
+      <c r="J372" t="n">
+        <v>3</v>
+      </c>
+      <c r="K372" t="n">
+        <v>5</v>
+      </c>
+      <c r="L372" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>West Bromwich Albion vs Blackburn Rovers</t>
+        </is>
+      </c>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>West Bromwich Albion</t>
+        </is>
+      </c>
+      <c r="D373" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E373" t="n">
+        <v>1.47</v>
+      </c>
+      <c r="F373" t="n">
+        <v>68.09999999999999</v>
+      </c>
+      <c r="G373" t="inlineStr">
+        <is>
+          <t>3-2</t>
+        </is>
+      </c>
+      <c r="H373" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I373" t="n">
+        <v>0</v>
+      </c>
+      <c r="J373" t="n">
+        <v>1</v>
+      </c>
+      <c r="K373" t="n">
+        <v>3</v>
+      </c>
+      <c r="L373" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>Espanyol vs Atlético Madrid</t>
+        </is>
+      </c>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>Atlético Madrid</t>
+        </is>
+      </c>
+      <c r="D374" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E374" t="n">
+        <v>1.82</v>
+      </c>
+      <c r="F374" t="n">
+        <v>55.1</v>
+      </c>
+      <c r="G374" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H374" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I374" t="n">
+        <v>0</v>
+      </c>
+      <c r="J374" t="n">
+        <v>2</v>
+      </c>
+      <c r="K374" t="n">
+        <v>2</v>
+      </c>
+      <c r="L374" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>AS Roma vs Genoa</t>
+        </is>
+      </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>AS Roma</t>
+        </is>
+      </c>
+      <c r="D375" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E375" t="n">
+        <v>1.14</v>
+      </c>
+      <c r="F375" t="n">
+        <v>88.09999999999999</v>
+      </c>
+      <c r="G375" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H375" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I375" t="n">
+        <v>5</v>
+      </c>
+      <c r="J375" t="n">
+        <v>1</v>
+      </c>
+      <c r="K375" t="n">
+        <v>2</v>
+      </c>
+      <c r="L375" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>Hamburg SV vs VfB Stuttgart</t>
+        </is>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>VfB Stuttgart</t>
+        </is>
+      </c>
+      <c r="D376" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E376" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="F376" t="n">
+        <v>71.59999999999999</v>
+      </c>
+      <c r="G376" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H376" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I376" t="n">
+        <v>0</v>
+      </c>
+      <c r="J376" t="n">
+        <v>3</v>
+      </c>
+      <c r="K376" t="n">
+        <v>2</v>
+      </c>
+      <c r="L376" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>Schalke 04 vs Mainz</t>
+        </is>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>Schalke 04</t>
+        </is>
+      </c>
+      <c r="D377" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E377" t="n">
+        <v>1.46</v>
+      </c>
+      <c r="F377" t="n">
+        <v>68.5</v>
+      </c>
+      <c r="G377" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H377" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I377" t="n">
+        <v>0</v>
+      </c>
+      <c r="J377" t="n">
+        <v>3</v>
+      </c>
+      <c r="K377" t="n">
+        <v>0</v>
+      </c>
+      <c r="L377" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>SV Elversberg vs FC Augsburg</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>SV Elversberg</t>
+        </is>
+      </c>
+      <c r="D378" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E378" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F378" t="n">
+        <v>66.90000000000001</v>
+      </c>
+      <c r="G378" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="H378" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I378" t="n">
+        <v>0</v>
+      </c>
+      <c r="J378" t="n">
+        <v>1</v>
+      </c>
+      <c r="K378" t="n">
+        <v>3</v>
+      </c>
+      <c r="L378" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>Lille vs Brest</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>Lille</t>
+        </is>
+      </c>
+      <c r="D379" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E379" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="F379" t="n">
+        <v>81.90000000000001</v>
+      </c>
+      <c r="G379" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H379" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I379" t="n">
+        <v>5</v>
+      </c>
+      <c r="J379" t="n">
+        <v>2</v>
+      </c>
+      <c r="K379" t="n">
+        <v>2</v>
+      </c>
+      <c r="L379" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>Levadiakos vs Volos NFC</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>Levadiakos</t>
+        </is>
+      </c>
+      <c r="D380" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E380" t="n">
+        <v>1.19</v>
+      </c>
+      <c r="F380" t="n">
+        <v>84</v>
+      </c>
+      <c r="G380" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H380" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I380" t="n">
+        <v>0</v>
+      </c>
+      <c r="J380" t="n">
+        <v>3</v>
+      </c>
+      <c r="K380" t="n">
+        <v>4</v>
+      </c>
+      <c r="L380" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>Atromitos vs AEK Athens</t>
+        </is>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>AEK Athens</t>
+        </is>
+      </c>
+      <c r="D381" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E381" t="n">
+        <v>2.09</v>
+      </c>
+      <c r="F381" t="n">
+        <v>47.9</v>
+      </c>
+      <c r="G381" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H381" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I381" t="n">
+        <v>0</v>
+      </c>
+      <c r="J381" t="n">
+        <v>2</v>
+      </c>
+      <c r="K381" t="n">
+        <v>5</v>
+      </c>
+      <c r="L381" t="inlineStr">
         <is>
           <t>si</t>
         </is>
@@ -18743,7 +20251,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E68"/>
+  <dimension ref="A1:E69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19996,6 +21504,25 @@
       </c>
       <c r="E68" t="n">
         <v>3</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>29</v>
+      </c>
+      <c r="C69" t="n">
+        <v>12</v>
+      </c>
+      <c r="D69" t="n">
+        <v>41.4</v>
+      </c>
+      <c r="E69" t="n">
+        <v>29</v>
       </c>
     </row>
   </sheetData>
@@ -20009,7 +21536,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E200"/>
+  <dimension ref="A1:E209"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24218,6 +25745,195 @@
         <v>0</v>
       </c>
     </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>tarjeta_roja</t>
+        </is>
+      </c>
+      <c r="C201" t="n">
+        <v>1</v>
+      </c>
+      <c r="D201" t="n">
+        <v>0</v>
+      </c>
+      <c r="E201" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>partido_resuelto</t>
+        </is>
+      </c>
+      <c r="C202" t="n">
+        <v>1</v>
+      </c>
+      <c r="D202" t="n">
+        <v>0</v>
+      </c>
+      <c r="E202" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>penal</t>
+        </is>
+      </c>
+      <c r="C203" t="n">
+        <v>3</v>
+      </c>
+      <c r="D203" t="n">
+        <v>1</v>
+      </c>
+      <c r="E203" t="n">
+        <v>33.3</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>cuidado_rival_presiona</t>
+        </is>
+      </c>
+      <c r="C204" t="n">
+        <v>4</v>
+      </c>
+      <c r="D204" t="n">
+        <v>3</v>
+      </c>
+      <c r="E204" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>ampliacion_marcador</t>
+        </is>
+      </c>
+      <c r="C205" t="n">
+        <v>10</v>
+      </c>
+      <c r="D205" t="n">
+        <v>1</v>
+      </c>
+      <c r="E205" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>posible_victoria_favorito</t>
+        </is>
+      </c>
+      <c r="C206" t="n">
+        <v>6</v>
+      </c>
+      <c r="D206" t="n">
+        <v>2</v>
+      </c>
+      <c r="E206" t="n">
+        <v>33.3</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>alerta_1er_tiempo</t>
+        </is>
+      </c>
+      <c r="C207" t="n">
+        <v>1</v>
+      </c>
+      <c r="D207" t="n">
+        <v>0</v>
+      </c>
+      <c r="E207" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>posible_empate</t>
+        </is>
+      </c>
+      <c r="C208" t="n">
+        <v>1</v>
+      </c>
+      <c r="D208" t="n">
+        <v>1</v>
+      </c>
+      <c r="E208" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>gol_de_cierre</t>
+        </is>
+      </c>
+      <c r="C209" t="n">
+        <v>1</v>
+      </c>
+      <c r="D209" t="n">
+        <v>0</v>
+      </c>
+      <c r="E209" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-10-19
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L381"/>
+  <dimension ref="A1:L402"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20235,6 +20235,1098 @@
         <v>5</v>
       </c>
       <c r="L381" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>Brighton &amp; Hove Albion vs Crystal Palace</t>
+        </is>
+      </c>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t>Brighton &amp; Hove Albion</t>
+        </is>
+      </c>
+      <c r="D382" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E382" t="n">
+        <v>1.41</v>
+      </c>
+      <c r="F382" t="n">
+        <v>70.8</v>
+      </c>
+      <c r="G382" t="inlineStr">
+        <is>
+          <t>5-0</t>
+        </is>
+      </c>
+      <c r="H382" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I382" t="n">
+        <v>0</v>
+      </c>
+      <c r="J382" t="n">
+        <v>3</v>
+      </c>
+      <c r="K382" t="n">
+        <v>6</v>
+      </c>
+      <c r="L382" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>Real Madrid vs Sevilla</t>
+        </is>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>Real Madrid</t>
+        </is>
+      </c>
+      <c r="D383" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E383" t="n">
+        <v>1.24</v>
+      </c>
+      <c r="F383" t="n">
+        <v>80.7</v>
+      </c>
+      <c r="G383" t="inlineStr">
+        <is>
+          <t>4-1</t>
+        </is>
+      </c>
+      <c r="H383" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I383" t="n">
+        <v>6</v>
+      </c>
+      <c r="J383" t="n">
+        <v>6</v>
+      </c>
+      <c r="K383" t="n">
+        <v>3</v>
+      </c>
+      <c r="L383" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>Borussia Mönchengladbach vs TSG Hoffenheim</t>
+        </is>
+      </c>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t>Borussia Mönchengladbach</t>
+        </is>
+      </c>
+      <c r="D384" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E384" t="n">
+        <v>1.86</v>
+      </c>
+      <c r="F384" t="n">
+        <v>53.7</v>
+      </c>
+      <c r="G384" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H384" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I384" t="n">
+        <v>0</v>
+      </c>
+      <c r="J384" t="n">
+        <v>1</v>
+      </c>
+      <c r="K384" t="n">
+        <v>3</v>
+      </c>
+      <c r="L384" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>Lyon vs Nice</t>
+        </is>
+      </c>
+      <c r="C385" t="inlineStr">
+        <is>
+          <t>Lyon</t>
+        </is>
+      </c>
+      <c r="D385" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E385" t="n">
+        <v>1.39</v>
+      </c>
+      <c r="F385" t="n">
+        <v>72.2</v>
+      </c>
+      <c r="G385" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H385" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I385" t="n">
+        <v>6</v>
+      </c>
+      <c r="J385" t="n">
+        <v>1</v>
+      </c>
+      <c r="K385" t="n">
+        <v>5</v>
+      </c>
+      <c r="L385" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>SC Cambuur vs AZ Alkmaar</t>
+        </is>
+      </c>
+      <c r="C386" t="inlineStr">
+        <is>
+          <t>AZ Alkmaar</t>
+        </is>
+      </c>
+      <c r="D386" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E386" t="n">
+        <v>2</v>
+      </c>
+      <c r="F386" t="n">
+        <v>50.1</v>
+      </c>
+      <c r="G386" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="H386" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I386" t="n">
+        <v>0</v>
+      </c>
+      <c r="J386" t="n">
+        <v>3</v>
+      </c>
+      <c r="K386" t="n">
+        <v>5</v>
+      </c>
+      <c r="L386" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>FC Twente vs FC Utrecht</t>
+        </is>
+      </c>
+      <c r="C387" t="inlineStr">
+        <is>
+          <t>FC Twente</t>
+        </is>
+      </c>
+      <c r="D387" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E387" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="F387" t="n">
+        <v>55.4</v>
+      </c>
+      <c r="G387" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H387" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I387" t="n">
+        <v>2</v>
+      </c>
+      <c r="J387" t="n">
+        <v>5</v>
+      </c>
+      <c r="K387" t="n">
+        <v>5</v>
+      </c>
+      <c r="L387" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>Kalamata vs OFI Crete</t>
+        </is>
+      </c>
+      <c r="C388" t="inlineStr">
+        <is>
+          <t>Kalamata</t>
+        </is>
+      </c>
+      <c r="D388" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E388" t="n">
+        <v>1.77</v>
+      </c>
+      <c r="F388" t="n">
+        <v>56.7</v>
+      </c>
+      <c r="G388" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="H388" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I388" t="n">
+        <v>0</v>
+      </c>
+      <c r="J388" t="n">
+        <v>3</v>
+      </c>
+      <c r="K388" t="n">
+        <v>6</v>
+      </c>
+      <c r="L388" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>Panetolikos vs Olympiacos</t>
+        </is>
+      </c>
+      <c r="C389" t="inlineStr">
+        <is>
+          <t>Olympiacos</t>
+        </is>
+      </c>
+      <c r="D389" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E389" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="F389" t="n">
+        <v>70.09999999999999</v>
+      </c>
+      <c r="G389" t="inlineStr">
+        <is>
+          <t>0-2</t>
+        </is>
+      </c>
+      <c r="H389" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I389" t="n">
+        <v>0</v>
+      </c>
+      <c r="J389" t="n">
+        <v>1</v>
+      </c>
+      <c r="K389" t="n">
+        <v>6</v>
+      </c>
+      <c r="L389" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>Panathinaikos vs Asteras Tripoli</t>
+        </is>
+      </c>
+      <c r="C390" t="inlineStr">
+        <is>
+          <t>Panathinaikos</t>
+        </is>
+      </c>
+      <c r="D390" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E390" t="n">
+        <v>2.32</v>
+      </c>
+      <c r="F390" t="n">
+        <v>43.1</v>
+      </c>
+      <c r="G390" t="inlineStr">
+        <is>
+          <t>5-1</t>
+        </is>
+      </c>
+      <c r="H390" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I390" t="n">
+        <v>0</v>
+      </c>
+      <c r="J390" t="n">
+        <v>4</v>
+      </c>
+      <c r="K390" t="n">
+        <v>3</v>
+      </c>
+      <c r="L390" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>PAOK vs Iraklis</t>
+        </is>
+      </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t>PAOK</t>
+        </is>
+      </c>
+      <c r="D391" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E391" t="n">
+        <v>2.29</v>
+      </c>
+      <c r="F391" t="n">
+        <v>43.7</v>
+      </c>
+      <c r="G391" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H391" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I391" t="n">
+        <v>4</v>
+      </c>
+      <c r="J391" t="n">
+        <v>1</v>
+      </c>
+      <c r="K391" t="n">
+        <v>1</v>
+      </c>
+      <c r="L391" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>Grêmio vs Cruzeiro</t>
+        </is>
+      </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>Grêmio</t>
+        </is>
+      </c>
+      <c r="D392" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E392" t="n">
+        <v>2.62</v>
+      </c>
+      <c r="F392" t="n">
+        <v>38.2</v>
+      </c>
+      <c r="G392" t="inlineStr">
+        <is>
+          <t>2-4</t>
+        </is>
+      </c>
+      <c r="H392" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I392" t="n">
+        <v>5</v>
+      </c>
+      <c r="J392" t="n">
+        <v>0</v>
+      </c>
+      <c r="K392" t="n">
+        <v>1</v>
+      </c>
+      <c r="L392" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>AFC Bournemouth vs Sunderland</t>
+        </is>
+      </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>AFC Bournemouth</t>
+        </is>
+      </c>
+      <c r="D393" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E393" t="n">
+        <v>1.51</v>
+      </c>
+      <c r="F393" t="n">
+        <v>66.09999999999999</v>
+      </c>
+      <c r="G393" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H393" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I393" t="n">
+        <v>0</v>
+      </c>
+      <c r="J393" t="n">
+        <v>2</v>
+      </c>
+      <c r="K393" t="n">
+        <v>4</v>
+      </c>
+      <c r="L393" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>Nottingham Forest vs Arsenal</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>Arsenal</t>
+        </is>
+      </c>
+      <c r="D394" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E394" t="n">
+        <v>1.84</v>
+      </c>
+      <c r="F394" t="n">
+        <v>54.4</v>
+      </c>
+      <c r="G394" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H394" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I394" t="n">
+        <v>0</v>
+      </c>
+      <c r="J394" t="n">
+        <v>1</v>
+      </c>
+      <c r="K394" t="n">
+        <v>5</v>
+      </c>
+      <c r="L394" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>Osasuna vs Racing Santander</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>Racing Santander</t>
+        </is>
+      </c>
+      <c r="D395" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E395" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="F395" t="n">
+        <v>76.90000000000001</v>
+      </c>
+      <c r="G395" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H395" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I395" t="n">
+        <v>0</v>
+      </c>
+      <c r="J395" t="n">
+        <v>4</v>
+      </c>
+      <c r="K395" t="n">
+        <v>5</v>
+      </c>
+      <c r="L395" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>Fiorentina vs Como</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>Como</t>
+        </is>
+      </c>
+      <c r="D396" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E396" t="n">
+        <v>1.24</v>
+      </c>
+      <c r="F396" t="n">
+        <v>80.59999999999999</v>
+      </c>
+      <c r="G396" t="inlineStr">
+        <is>
+          <t>1-3</t>
+        </is>
+      </c>
+      <c r="H396" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I396" t="n">
+        <v>0</v>
+      </c>
+      <c r="J396" t="n">
+        <v>1</v>
+      </c>
+      <c r="K396" t="n">
+        <v>3</v>
+      </c>
+      <c r="L396" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>Bayer Leverkusen vs SC Freiburg</t>
+        </is>
+      </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t>Bayer Leverkusen</t>
+        </is>
+      </c>
+      <c r="D397" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E397" t="n">
+        <v>1.78</v>
+      </c>
+      <c r="F397" t="n">
+        <v>56.1</v>
+      </c>
+      <c r="G397" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H397" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I397" t="n">
+        <v>0</v>
+      </c>
+      <c r="J397" t="n">
+        <v>0</v>
+      </c>
+      <c r="K397" t="n">
+        <v>1</v>
+      </c>
+      <c r="L397" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>PEC Zwolle vs Go Ahead Eagles</t>
+        </is>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>Go Ahead Eagles</t>
+        </is>
+      </c>
+      <c r="D398" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E398" t="n">
+        <v>1.19</v>
+      </c>
+      <c r="F398" t="n">
+        <v>84.40000000000001</v>
+      </c>
+      <c r="G398" t="inlineStr">
+        <is>
+          <t>4-1</t>
+        </is>
+      </c>
+      <c r="H398" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I398" t="n">
+        <v>0</v>
+      </c>
+      <c r="J398" t="n">
+        <v>4</v>
+      </c>
+      <c r="K398" t="n">
+        <v>2</v>
+      </c>
+      <c r="L398" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>NEC Nijmegen vs Fortuna Sittard</t>
+        </is>
+      </c>
+      <c r="C399" t="inlineStr">
+        <is>
+          <t>NEC Nijmegen</t>
+        </is>
+      </c>
+      <c r="D399" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E399" t="n">
+        <v>1.42</v>
+      </c>
+      <c r="F399" t="n">
+        <v>70.2</v>
+      </c>
+      <c r="G399" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="H399" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I399" t="n">
+        <v>7</v>
+      </c>
+      <c r="J399" t="n">
+        <v>4</v>
+      </c>
+      <c r="K399" t="n">
+        <v>3</v>
+      </c>
+      <c r="L399" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>Kifisia vs Aris</t>
+        </is>
+      </c>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t>Aris</t>
+        </is>
+      </c>
+      <c r="D400" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E400" t="n">
+        <v>1.46</v>
+      </c>
+      <c r="F400" t="n">
+        <v>68.7</v>
+      </c>
+      <c r="G400" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H400" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I400" t="n">
+        <v>4</v>
+      </c>
+      <c r="J400" t="n">
+        <v>5</v>
+      </c>
+      <c r="K400" t="n">
+        <v>3</v>
+      </c>
+      <c r="L400" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>Celtic vs Heart of Midlothian</t>
+        </is>
+      </c>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t>Celtic</t>
+        </is>
+      </c>
+      <c r="D401" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E401" t="n">
+        <v>1.53</v>
+      </c>
+      <c r="F401" t="n">
+        <v>65.3</v>
+      </c>
+      <c r="G401" t="inlineStr">
+        <is>
+          <t>7-1</t>
+        </is>
+      </c>
+      <c r="H401" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I401" t="n">
+        <v>0</v>
+      </c>
+      <c r="J401" t="n">
+        <v>1</v>
+      </c>
+      <c r="K401" t="n">
+        <v>0</v>
+      </c>
+      <c r="L401" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>Bahia vs Flamengo</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>Flamengo</t>
+        </is>
+      </c>
+      <c r="D402" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E402" t="n">
+        <v>2.07</v>
+      </c>
+      <c r="F402" t="n">
+        <v>48.3</v>
+      </c>
+      <c r="G402" t="inlineStr">
+        <is>
+          <t>0-3</t>
+        </is>
+      </c>
+      <c r="H402" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I402" t="n">
+        <v>7</v>
+      </c>
+      <c r="J402" t="n">
+        <v>1</v>
+      </c>
+      <c r="K402" t="n">
+        <v>6</v>
+      </c>
+      <c r="L402" t="inlineStr">
         <is>
           <t>si</t>
         </is>
@@ -20251,7 +21343,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E69"/>
+  <dimension ref="A1:E70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21523,6 +22615,25 @@
       </c>
       <c r="E69" t="n">
         <v>29</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>21</v>
+      </c>
+      <c r="C70" t="n">
+        <v>14</v>
+      </c>
+      <c r="D70" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="E70" t="n">
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -21536,7 +22647,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E209"/>
+  <dimension ref="A1:E218"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -25934,6 +27045,195 @@
         <v>0</v>
       </c>
     </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>alerta_1er_tiempo</t>
+        </is>
+      </c>
+      <c r="C210" t="n">
+        <v>3</v>
+      </c>
+      <c r="D210" t="n">
+        <v>1</v>
+      </c>
+      <c r="E210" t="n">
+        <v>33.3</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>posible_victoria_favorito</t>
+        </is>
+      </c>
+      <c r="C211" t="n">
+        <v>8</v>
+      </c>
+      <c r="D211" t="n">
+        <v>2</v>
+      </c>
+      <c r="E211" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>ampliacion_marcador</t>
+        </is>
+      </c>
+      <c r="C212" t="n">
+        <v>4</v>
+      </c>
+      <c r="D212" t="n">
+        <v>2</v>
+      </c>
+      <c r="E212" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>cuidado_rival_presiona</t>
+        </is>
+      </c>
+      <c r="C213" t="n">
+        <v>13</v>
+      </c>
+      <c r="D213" t="n">
+        <v>3</v>
+      </c>
+      <c r="E213" t="n">
+        <v>23.1</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>partido_resuelto</t>
+        </is>
+      </c>
+      <c r="C214" t="n">
+        <v>2</v>
+      </c>
+      <c r="D214" t="n">
+        <v>0</v>
+      </c>
+      <c r="E214" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>tarjeta_roja</t>
+        </is>
+      </c>
+      <c r="C215" t="n">
+        <v>3</v>
+      </c>
+      <c r="D215" t="n">
+        <v>0</v>
+      </c>
+      <c r="E215" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>gol_de_cierre</t>
+        </is>
+      </c>
+      <c r="C216" t="n">
+        <v>3</v>
+      </c>
+      <c r="D216" t="n">
+        <v>0</v>
+      </c>
+      <c r="E216" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>penal</t>
+        </is>
+      </c>
+      <c r="C217" t="n">
+        <v>3</v>
+      </c>
+      <c r="D217" t="n">
+        <v>2</v>
+      </c>
+      <c r="E217" t="n">
+        <v>66.7</v>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>posible_empate</t>
+        </is>
+      </c>
+      <c r="C218" t="n">
+        <v>2</v>
+      </c>
+      <c r="D218" t="n">
+        <v>0</v>
+      </c>
+      <c r="E218" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-10-20
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L402"/>
+  <dimension ref="A1:L405"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21327,6 +21327,162 @@
         <v>6</v>
       </c>
       <c r="L402" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>Monza vs Cagliari</t>
+        </is>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>Monza</t>
+        </is>
+      </c>
+      <c r="D403" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E403" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="F403" t="n">
+        <v>80</v>
+      </c>
+      <c r="G403" t="inlineStr">
+        <is>
+          <t>4-0</t>
+        </is>
+      </c>
+      <c r="H403" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I403" t="n">
+        <v>0</v>
+      </c>
+      <c r="J403" t="n">
+        <v>0</v>
+      </c>
+      <c r="K403" t="n">
+        <v>1</v>
+      </c>
+      <c r="L403" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>Braga vs Gil Vicente</t>
+        </is>
+      </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>Braga</t>
+        </is>
+      </c>
+      <c r="D404" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E404" t="n">
+        <v>1.34</v>
+      </c>
+      <c r="F404" t="n">
+        <v>74.59999999999999</v>
+      </c>
+      <c r="G404" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H404" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I404" t="n">
+        <v>2</v>
+      </c>
+      <c r="J404" t="n">
+        <v>2</v>
+      </c>
+      <c r="K404" t="n">
+        <v>2</v>
+      </c>
+      <c r="L404" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>Trabzonspor vs Besiktas</t>
+        </is>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>Besiktas</t>
+        </is>
+      </c>
+      <c r="D405" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E405" t="n">
+        <v>1.83</v>
+      </c>
+      <c r="F405" t="n">
+        <v>54.5</v>
+      </c>
+      <c r="G405" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H405" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I405" t="n">
+        <v>0</v>
+      </c>
+      <c r="J405" t="n">
+        <v>0</v>
+      </c>
+      <c r="K405" t="n">
+        <v>3</v>
+      </c>
+      <c r="L405" t="inlineStr">
         <is>
           <t>si</t>
         </is>
@@ -21343,7 +21499,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E70"/>
+  <dimension ref="A1:E71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22634,6 +22790,25 @@
       </c>
       <c r="E70" t="n">
         <v>21</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>3</v>
+      </c>
+      <c r="C71" t="n">
+        <v>1</v>
+      </c>
+      <c r="D71" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="E71" t="n">
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -22647,7 +22822,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E218"/>
+  <dimension ref="A1:E219"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27234,6 +27409,27 @@
         <v>0</v>
       </c>
     </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>posible_empate</t>
+        </is>
+      </c>
+      <c r="C219" t="n">
+        <v>2</v>
+      </c>
+      <c r="D219" t="n">
+        <v>0</v>
+      </c>
+      <c r="E219" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-10-21
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L405"/>
+  <dimension ref="A1:L411"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21483,6 +21483,318 @@
         <v>3</v>
       </c>
       <c r="L405" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>Guadalajara vs Necaxa</t>
+        </is>
+      </c>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t>Guadalajara</t>
+        </is>
+      </c>
+      <c r="D406" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E406" t="n">
+        <v>1.39</v>
+      </c>
+      <c r="F406" t="n">
+        <v>71.90000000000001</v>
+      </c>
+      <c r="G406" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H406" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I406" t="n">
+        <v>2</v>
+      </c>
+      <c r="J406" t="n">
+        <v>0</v>
+      </c>
+      <c r="K406" t="n">
+        <v>1</v>
+      </c>
+      <c r="L406" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>Sabah FK vs Borussia Dortmund</t>
+        </is>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>Borussia Dortmund</t>
+        </is>
+      </c>
+      <c r="D407" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E407" t="n">
+        <v>2.06</v>
+      </c>
+      <c r="F407" t="n">
+        <v>48.6</v>
+      </c>
+      <c r="G407" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H407" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I407" t="n">
+        <v>0</v>
+      </c>
+      <c r="J407" t="n">
+        <v>1</v>
+      </c>
+      <c r="K407" t="n">
+        <v>1</v>
+      </c>
+      <c r="L407" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>AS Roma vs Slovan Bratislava</t>
+        </is>
+      </c>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t>AS Roma</t>
+        </is>
+      </c>
+      <c r="D408" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E408" t="n">
+        <v>1.24</v>
+      </c>
+      <c r="F408" t="n">
+        <v>80.5</v>
+      </c>
+      <c r="G408" t="inlineStr">
+        <is>
+          <t>4-0</t>
+        </is>
+      </c>
+      <c r="H408" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I408" t="n">
+        <v>2</v>
+      </c>
+      <c r="J408" t="n">
+        <v>2</v>
+      </c>
+      <c r="K408" t="n">
+        <v>2</v>
+      </c>
+      <c r="L408" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>Manchester City vs AEK Athens</t>
+        </is>
+      </c>
+      <c r="C409" t="inlineStr">
+        <is>
+          <t>Manchester City</t>
+        </is>
+      </c>
+      <c r="D409" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E409" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="F409" t="n">
+        <v>69.2</v>
+      </c>
+      <c r="G409" t="inlineStr">
+        <is>
+          <t>5-1</t>
+        </is>
+      </c>
+      <c r="H409" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I409" t="n">
+        <v>4</v>
+      </c>
+      <c r="J409" t="n">
+        <v>5</v>
+      </c>
+      <c r="K409" t="n">
+        <v>6</v>
+      </c>
+      <c r="L409" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>Wolverhampton Wanderers vs Portsmouth</t>
+        </is>
+      </c>
+      <c r="C410" t="inlineStr">
+        <is>
+          <t>Portsmouth</t>
+        </is>
+      </c>
+      <c r="D410" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E410" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="F410" t="n">
+        <v>45.4</v>
+      </c>
+      <c r="G410" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H410" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I410" t="n">
+        <v>3</v>
+      </c>
+      <c r="J410" t="n">
+        <v>4</v>
+      </c>
+      <c r="K410" t="n">
+        <v>0</v>
+      </c>
+      <c r="L410" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>Paris Saint-Germain vs Barcelona</t>
+        </is>
+      </c>
+      <c r="C411" t="inlineStr">
+        <is>
+          <t>Barcelona</t>
+        </is>
+      </c>
+      <c r="D411" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E411" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F411" t="n">
+        <v>66.5</v>
+      </c>
+      <c r="G411" t="inlineStr">
+        <is>
+          <t>4-2</t>
+        </is>
+      </c>
+      <c r="H411" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I411" t="n">
+        <v>2</v>
+      </c>
+      <c r="J411" t="n">
+        <v>7</v>
+      </c>
+      <c r="K411" t="n">
+        <v>11</v>
+      </c>
+      <c r="L411" t="inlineStr">
         <is>
           <t>si</t>
         </is>
@@ -21499,7 +21811,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E71"/>
+  <dimension ref="A1:E72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22809,6 +23121,25 @@
       </c>
       <c r="E71" t="n">
         <v>3</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>6</v>
+      </c>
+      <c r="C72" t="n">
+        <v>4</v>
+      </c>
+      <c r="D72" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="E72" t="n">
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -22822,7 +23153,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E219"/>
+  <dimension ref="A1:E224"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27430,6 +27761,111 @@
         <v>0</v>
       </c>
     </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>alerta_1er_tiempo</t>
+        </is>
+      </c>
+      <c r="C220" t="n">
+        <v>1</v>
+      </c>
+      <c r="D220" t="n">
+        <v>0</v>
+      </c>
+      <c r="E220" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>posible_victoria_favorito</t>
+        </is>
+      </c>
+      <c r="C221" t="n">
+        <v>2</v>
+      </c>
+      <c r="D221" t="n">
+        <v>0</v>
+      </c>
+      <c r="E221" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>ampliacion_marcador</t>
+        </is>
+      </c>
+      <c r="C222" t="n">
+        <v>4</v>
+      </c>
+      <c r="D222" t="n">
+        <v>3</v>
+      </c>
+      <c r="E222" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>partido_resuelto</t>
+        </is>
+      </c>
+      <c r="C223" t="n">
+        <v>2</v>
+      </c>
+      <c r="D223" t="n">
+        <v>0</v>
+      </c>
+      <c r="E223" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>cuidado_rival_presiona</t>
+        </is>
+      </c>
+      <c r="C224" t="n">
+        <v>4</v>
+      </c>
+      <c r="D224" t="n">
+        <v>2</v>
+      </c>
+      <c r="E224" t="n">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-10-22
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L411"/>
+  <dimension ref="A1:L420"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21795,6 +21795,474 @@
         <v>11</v>
       </c>
       <c r="L411" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>Toluca vs Tijuana</t>
+        </is>
+      </c>
+      <c r="C412" t="inlineStr">
+        <is>
+          <t>Toluca</t>
+        </is>
+      </c>
+      <c r="D412" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E412" t="n">
+        <v>1.86</v>
+      </c>
+      <c r="F412" t="n">
+        <v>53.8</v>
+      </c>
+      <c r="G412" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="H412" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I412" t="n">
+        <v>0</v>
+      </c>
+      <c r="J412" t="n">
+        <v>6</v>
+      </c>
+      <c r="K412" t="n">
+        <v>1</v>
+      </c>
+      <c r="L412" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>Aston Villa vs Viking FK</t>
+        </is>
+      </c>
+      <c r="C413" t="inlineStr">
+        <is>
+          <t>Aston Villa</t>
+        </is>
+      </c>
+      <c r="D413" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E413" t="n">
+        <v>2.08</v>
+      </c>
+      <c r="F413" t="n">
+        <v>48.1</v>
+      </c>
+      <c r="G413" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="H413" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I413" t="n">
+        <v>3</v>
+      </c>
+      <c r="J413" t="n">
+        <v>0</v>
+      </c>
+      <c r="K413" t="n">
+        <v>1</v>
+      </c>
+      <c r="L413" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>Internazionale vs Shakhtar Donetsk</t>
+        </is>
+      </c>
+      <c r="C414" t="inlineStr">
+        <is>
+          <t>Internazionale</t>
+        </is>
+      </c>
+      <c r="D414" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E414" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="F414" t="n">
+        <v>54.1</v>
+      </c>
+      <c r="G414" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H414" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I414" t="n">
+        <v>5</v>
+      </c>
+      <c r="J414" t="n">
+        <v>4</v>
+      </c>
+      <c r="K414" t="n">
+        <v>1</v>
+      </c>
+      <c r="L414" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>Real Madrid vs RB Leipzig</t>
+        </is>
+      </c>
+      <c r="C415" t="inlineStr">
+        <is>
+          <t>Real Madrid</t>
+        </is>
+      </c>
+      <c r="D415" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E415" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="F415" t="n">
+        <v>76.8</v>
+      </c>
+      <c r="G415" t="inlineStr">
+        <is>
+          <t>4-1</t>
+        </is>
+      </c>
+      <c r="H415" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I415" t="n">
+        <v>3</v>
+      </c>
+      <c r="J415" t="n">
+        <v>7</v>
+      </c>
+      <c r="K415" t="n">
+        <v>5</v>
+      </c>
+      <c r="L415" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>Sporting CP vs LASK Linz</t>
+        </is>
+      </c>
+      <c r="C416" t="inlineStr">
+        <is>
+          <t>Sporting CP</t>
+        </is>
+      </c>
+      <c r="D416" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E416" t="n">
+        <v>1.49</v>
+      </c>
+      <c r="F416" t="n">
+        <v>67.09999999999999</v>
+      </c>
+      <c r="G416" t="inlineStr">
+        <is>
+          <t>2-3</t>
+        </is>
+      </c>
+      <c r="H416" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I416" t="n">
+        <v>3</v>
+      </c>
+      <c r="J416" t="n">
+        <v>5</v>
+      </c>
+      <c r="K416" t="n">
+        <v>1</v>
+      </c>
+      <c r="L416" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>Palmeiras vs Fluminense</t>
+        </is>
+      </c>
+      <c r="C417" t="inlineStr">
+        <is>
+          <t>Palmeiras</t>
+        </is>
+      </c>
+      <c r="D417" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E417" t="n">
+        <v>1.13</v>
+      </c>
+      <c r="F417" t="n">
+        <v>88.40000000000001</v>
+      </c>
+      <c r="G417" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H417" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I417" t="n">
+        <v>0</v>
+      </c>
+      <c r="J417" t="n">
+        <v>5</v>
+      </c>
+      <c r="K417" t="n">
+        <v>7</v>
+      </c>
+      <c r="L417" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>Lille vs Galatasaray</t>
+        </is>
+      </c>
+      <c r="C418" t="inlineStr">
+        <is>
+          <t>Galatasaray</t>
+        </is>
+      </c>
+      <c r="D418" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E418" t="n">
+        <v>1.52</v>
+      </c>
+      <c r="F418" t="n">
+        <v>66</v>
+      </c>
+      <c r="G418" t="inlineStr">
+        <is>
+          <t>2-4</t>
+        </is>
+      </c>
+      <c r="H418" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I418" t="n">
+        <v>0</v>
+      </c>
+      <c r="J418" t="n">
+        <v>3</v>
+      </c>
+      <c r="K418" t="n">
+        <v>7</v>
+      </c>
+      <c r="L418" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>Bayern Munich vs Arsenal</t>
+        </is>
+      </c>
+      <c r="C419" t="inlineStr">
+        <is>
+          <t>Bayern Munich</t>
+        </is>
+      </c>
+      <c r="D419" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E419" t="n">
+        <v>1.46</v>
+      </c>
+      <c r="F419" t="n">
+        <v>68.40000000000001</v>
+      </c>
+      <c r="G419" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="H419" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I419" t="n">
+        <v>3</v>
+      </c>
+      <c r="J419" t="n">
+        <v>7</v>
+      </c>
+      <c r="K419" t="n">
+        <v>6</v>
+      </c>
+      <c r="L419" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>Club Brugge vs Lens</t>
+        </is>
+      </c>
+      <c r="C420" t="inlineStr">
+        <is>
+          <t>Club Brugge</t>
+        </is>
+      </c>
+      <c r="D420" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E420" t="n">
+        <v>1.21</v>
+      </c>
+      <c r="F420" t="n">
+        <v>82.59999999999999</v>
+      </c>
+      <c r="G420" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="H420" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I420" t="n">
+        <v>2</v>
+      </c>
+      <c r="J420" t="n">
+        <v>6</v>
+      </c>
+      <c r="K420" t="n">
+        <v>0</v>
+      </c>
+      <c r="L420" t="inlineStr">
         <is>
           <t>si</t>
         </is>
@@ -21811,7 +22279,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E72"/>
+  <dimension ref="A1:E73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23140,6 +23608,25 @@
       </c>
       <c r="E72" t="n">
         <v>6</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B73" t="n">
+        <v>9</v>
+      </c>
+      <c r="C73" t="n">
+        <v>5</v>
+      </c>
+      <c r="D73" t="n">
+        <v>55.6</v>
+      </c>
+      <c r="E73" t="n">
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -23153,7 +23640,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E224"/>
+  <dimension ref="A1:E231"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27866,6 +28353,153 @@
         <v>50</v>
       </c>
     </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>ampliacion_marcador</t>
+        </is>
+      </c>
+      <c r="C225" t="n">
+        <v>6</v>
+      </c>
+      <c r="D225" t="n">
+        <v>2</v>
+      </c>
+      <c r="E225" t="n">
+        <v>33.3</v>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>penal</t>
+        </is>
+      </c>
+      <c r="C226" t="n">
+        <v>3</v>
+      </c>
+      <c r="D226" t="n">
+        <v>0</v>
+      </c>
+      <c r="E226" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>partido_resuelto</t>
+        </is>
+      </c>
+      <c r="C227" t="n">
+        <v>3</v>
+      </c>
+      <c r="D227" t="n">
+        <v>0</v>
+      </c>
+      <c r="E227" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>cuidado_rival_presiona</t>
+        </is>
+      </c>
+      <c r="C228" t="n">
+        <v>4</v>
+      </c>
+      <c r="D228" t="n">
+        <v>1</v>
+      </c>
+      <c r="E228" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>tarjeta_roja</t>
+        </is>
+      </c>
+      <c r="C229" t="n">
+        <v>1</v>
+      </c>
+      <c r="D229" t="n">
+        <v>0</v>
+      </c>
+      <c r="E229" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>gol_de_cierre</t>
+        </is>
+      </c>
+      <c r="C230" t="n">
+        <v>1</v>
+      </c>
+      <c r="D230" t="n">
+        <v>1</v>
+      </c>
+      <c r="E230" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>posible_victoria_favorito</t>
+        </is>
+      </c>
+      <c r="C231" t="n">
+        <v>1</v>
+      </c>
+      <c r="D231" t="n">
+        <v>0</v>
+      </c>
+      <c r="E231" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-10-23
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L420"/>
+  <dimension ref="A1:L432"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22265,6 +22265,630 @@
       <c r="L420" t="inlineStr">
         <is>
           <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>Flamengo vs Estudiantes de La Plata</t>
+        </is>
+      </c>
+      <c r="C421" t="inlineStr">
+        <is>
+          <t>Flamengo</t>
+        </is>
+      </c>
+      <c r="D421" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E421" t="n">
+        <v>1.47</v>
+      </c>
+      <c r="F421" t="n">
+        <v>68.3</v>
+      </c>
+      <c r="G421" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H421" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I421" t="n">
+        <v>0</v>
+      </c>
+      <c r="J421" t="n">
+        <v>7</v>
+      </c>
+      <c r="K421" t="n">
+        <v>0</v>
+      </c>
+      <c r="L421" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>Ararat-Armenia vs AZ Alkmaar</t>
+        </is>
+      </c>
+      <c r="C422" t="inlineStr">
+        <is>
+          <t>AZ Alkmaar</t>
+        </is>
+      </c>
+      <c r="D422" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E422" t="n">
+        <v>1.98</v>
+      </c>
+      <c r="F422" t="n">
+        <v>50.5</v>
+      </c>
+      <c r="G422" t="inlineStr">
+        <is>
+          <t>0-4</t>
+        </is>
+      </c>
+      <c r="H422" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I422" t="n">
+        <v>0</v>
+      </c>
+      <c r="J422" t="n">
+        <v>1</v>
+      </c>
+      <c r="K422" t="n">
+        <v>6</v>
+      </c>
+      <c r="L422" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>Dinamo Zagreb vs NEC Nijmegen</t>
+        </is>
+      </c>
+      <c r="C423" t="inlineStr">
+        <is>
+          <t>Dinamo Zagreb</t>
+        </is>
+      </c>
+      <c r="D423" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E423" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="F423" t="n">
+        <v>39.4</v>
+      </c>
+      <c r="G423" t="inlineStr">
+        <is>
+          <t>2-4</t>
+        </is>
+      </c>
+      <c r="H423" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I423" t="n">
+        <v>0</v>
+      </c>
+      <c r="J423" t="n">
+        <v>0</v>
+      </c>
+      <c r="K423" t="n">
+        <v>5</v>
+      </c>
+      <c r="L423" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>Ferencvaros vs Torreense</t>
+        </is>
+      </c>
+      <c r="C424" t="inlineStr">
+        <is>
+          <t>Ferencvaros</t>
+        </is>
+      </c>
+      <c r="D424" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E424" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="F424" t="n">
+        <v>58.8</v>
+      </c>
+      <c r="G424" t="inlineStr">
+        <is>
+          <t>4-1</t>
+        </is>
+      </c>
+      <c r="H424" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I424" t="n">
+        <v>0</v>
+      </c>
+      <c r="J424" t="n">
+        <v>0</v>
+      </c>
+      <c r="K424" t="n">
+        <v>1</v>
+      </c>
+      <c r="L424" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>OFI Crete vs Bayer Leverkusen</t>
+        </is>
+      </c>
+      <c r="C425" t="inlineStr">
+        <is>
+          <t>Bayer Leverkusen</t>
+        </is>
+      </c>
+      <c r="D425" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E425" t="n">
+        <v>1.89</v>
+      </c>
+      <c r="F425" t="n">
+        <v>52.9</v>
+      </c>
+      <c r="G425" t="inlineStr">
+        <is>
+          <t>0-2</t>
+        </is>
+      </c>
+      <c r="H425" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I425" t="n">
+        <v>0</v>
+      </c>
+      <c r="J425" t="n">
+        <v>7</v>
+      </c>
+      <c r="K425" t="n">
+        <v>1</v>
+      </c>
+      <c r="L425" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B426" t="inlineStr">
+        <is>
+          <t>Union St.-Gilloise vs Hapoel Be'er</t>
+        </is>
+      </c>
+      <c r="C426" t="inlineStr">
+        <is>
+          <t>Union St.-Gilloise</t>
+        </is>
+      </c>
+      <c r="D426" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E426" t="n">
+        <v>1.37</v>
+      </c>
+      <c r="F426" t="n">
+        <v>72.90000000000001</v>
+      </c>
+      <c r="G426" t="inlineStr">
+        <is>
+          <t>4-0</t>
+        </is>
+      </c>
+      <c r="H426" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I426" t="n">
+        <v>0</v>
+      </c>
+      <c r="J426" t="n">
+        <v>5</v>
+      </c>
+      <c r="K426" t="n">
+        <v>1</v>
+      </c>
+      <c r="L426" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>Omonia Nicosia vs Benfica</t>
+        </is>
+      </c>
+      <c r="C427" t="inlineStr">
+        <is>
+          <t>Benfica</t>
+        </is>
+      </c>
+      <c r="D427" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E427" t="n">
+        <v>1.29</v>
+      </c>
+      <c r="F427" t="n">
+        <v>77.40000000000001</v>
+      </c>
+      <c r="G427" t="inlineStr">
+        <is>
+          <t>1-4</t>
+        </is>
+      </c>
+      <c r="H427" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I427" t="n">
+        <v>5</v>
+      </c>
+      <c r="J427" t="n">
+        <v>0</v>
+      </c>
+      <c r="K427" t="n">
+        <v>8</v>
+      </c>
+      <c r="L427" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>Juventus vs Stade Rennais</t>
+        </is>
+      </c>
+      <c r="C428" t="inlineStr">
+        <is>
+          <t>Stade Rennais</t>
+        </is>
+      </c>
+      <c r="D428" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E428" t="n">
+        <v>2.66</v>
+      </c>
+      <c r="F428" t="n">
+        <v>37.6</v>
+      </c>
+      <c r="G428" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="H428" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I428" t="n">
+        <v>0</v>
+      </c>
+      <c r="J428" t="n">
+        <v>1</v>
+      </c>
+      <c r="K428" t="n">
+        <v>3</v>
+      </c>
+      <c r="L428" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>Besiktas vs Crystal Palace</t>
+        </is>
+      </c>
+      <c r="C429" t="inlineStr">
+        <is>
+          <t>Besiktas</t>
+        </is>
+      </c>
+      <c r="D429" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E429" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="F429" t="n">
+        <v>87.09999999999999</v>
+      </c>
+      <c r="G429" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="H429" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I429" t="n">
+        <v>3</v>
+      </c>
+      <c r="J429" t="n">
+        <v>4</v>
+      </c>
+      <c r="K429" t="n">
+        <v>7</v>
+      </c>
+      <c r="L429" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>Celtic vs Celta Vigo</t>
+        </is>
+      </c>
+      <c r="C430" t="inlineStr">
+        <is>
+          <t>Celtic</t>
+        </is>
+      </c>
+      <c r="D430" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E430" t="n">
+        <v>1.28</v>
+      </c>
+      <c r="F430" t="n">
+        <v>78</v>
+      </c>
+      <c r="G430" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H430" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I430" t="n">
+        <v>2</v>
+      </c>
+      <c r="J430" t="n">
+        <v>2</v>
+      </c>
+      <c r="K430" t="n">
+        <v>3</v>
+      </c>
+      <c r="L430" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>Lillestrom vs Real Sociedad</t>
+        </is>
+      </c>
+      <c r="C431" t="inlineStr">
+        <is>
+          <t>Lillestrom</t>
+        </is>
+      </c>
+      <c r="D431" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E431" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="F431" t="n">
+        <v>58.7</v>
+      </c>
+      <c r="G431" t="inlineStr">
+        <is>
+          <t>0-6</t>
+        </is>
+      </c>
+      <c r="H431" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I431" t="n">
+        <v>2</v>
+      </c>
+      <c r="J431" t="n">
+        <v>0</v>
+      </c>
+      <c r="K431" t="n">
+        <v>2</v>
+      </c>
+      <c r="L431" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>Olympiacos vs Sparta Prague</t>
+        </is>
+      </c>
+      <c r="C432" t="inlineStr">
+        <is>
+          <t>Olympiacos</t>
+        </is>
+      </c>
+      <c r="D432" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E432" t="n">
+        <v>1.44</v>
+      </c>
+      <c r="F432" t="n">
+        <v>69.3</v>
+      </c>
+      <c r="G432" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H432" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I432" t="n">
+        <v>5</v>
+      </c>
+      <c r="J432" t="n">
+        <v>7</v>
+      </c>
+      <c r="K432" t="n">
+        <v>0</v>
+      </c>
+      <c r="L432" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -22279,7 +22903,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E73"/>
+  <dimension ref="A1:E74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23627,6 +24251,25 @@
       </c>
       <c r="E73" t="n">
         <v>9</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B74" t="n">
+        <v>12</v>
+      </c>
+      <c r="C74" t="n">
+        <v>6</v>
+      </c>
+      <c r="D74" t="n">
+        <v>50</v>
+      </c>
+      <c r="E74" t="n">
+        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -23640,7 +24283,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E231"/>
+  <dimension ref="A1:E237"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28500,6 +29143,132 @@
         <v>0</v>
       </c>
     </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>cuidado_rival_presiona</t>
+        </is>
+      </c>
+      <c r="C232" t="n">
+        <v>6</v>
+      </c>
+      <c r="D232" t="n">
+        <v>1</v>
+      </c>
+      <c r="E232" t="n">
+        <v>16.7</v>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>ampliacion_marcador</t>
+        </is>
+      </c>
+      <c r="C233" t="n">
+        <v>4</v>
+      </c>
+      <c r="D233" t="n">
+        <v>2</v>
+      </c>
+      <c r="E233" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>partido_resuelto</t>
+        </is>
+      </c>
+      <c r="C234" t="n">
+        <v>2</v>
+      </c>
+      <c r="D234" t="n">
+        <v>0</v>
+      </c>
+      <c r="E234" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>tarjeta_roja</t>
+        </is>
+      </c>
+      <c r="C235" t="n">
+        <v>1</v>
+      </c>
+      <c r="D235" t="n">
+        <v>0</v>
+      </c>
+      <c r="E235" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>alerta_1er_tiempo</t>
+        </is>
+      </c>
+      <c r="C236" t="n">
+        <v>1</v>
+      </c>
+      <c r="D236" t="n">
+        <v>0</v>
+      </c>
+      <c r="E236" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>posible_victoria_favorito</t>
+        </is>
+      </c>
+      <c r="C237" t="n">
+        <v>3</v>
+      </c>
+      <c r="D237" t="n">
+        <v>1</v>
+      </c>
+      <c r="E237" t="n">
+        <v>33.3</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-10-24
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L432"/>
+  <dimension ref="A1:L437"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22889,6 +22889,266 @@
       <c r="L432" t="inlineStr">
         <is>
           <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>VfB Stuttgart vs Borussia Mönchengladbach</t>
+        </is>
+      </c>
+      <c r="C433" t="inlineStr">
+        <is>
+          <t>VfB Stuttgart</t>
+        </is>
+      </c>
+      <c r="D433" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E433" t="n">
+        <v>1.32</v>
+      </c>
+      <c r="F433" t="n">
+        <v>75.5</v>
+      </c>
+      <c r="G433" t="inlineStr">
+        <is>
+          <t>2-3</t>
+        </is>
+      </c>
+      <c r="H433" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I433" t="n">
+        <v>1</v>
+      </c>
+      <c r="J433" t="n">
+        <v>3</v>
+      </c>
+      <c r="K433" t="n">
+        <v>2</v>
+      </c>
+      <c r="L433" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B434" t="inlineStr">
+        <is>
+          <t>Cruzeiro vs Remo</t>
+        </is>
+      </c>
+      <c r="C434" t="inlineStr">
+        <is>
+          <t>Cruzeiro</t>
+        </is>
+      </c>
+      <c r="D434" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E434" t="n">
+        <v>1.73</v>
+      </c>
+      <c r="F434" t="n">
+        <v>57.8</v>
+      </c>
+      <c r="G434" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H434" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I434" t="n">
+        <v>1</v>
+      </c>
+      <c r="J434" t="n">
+        <v>2</v>
+      </c>
+      <c r="K434" t="n">
+        <v>5</v>
+      </c>
+      <c r="L434" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B435" t="inlineStr">
+        <is>
+          <t>Bolton Wanderers vs Middlesbrough</t>
+        </is>
+      </c>
+      <c r="C435" t="inlineStr">
+        <is>
+          <t>Middlesbrough</t>
+        </is>
+      </c>
+      <c r="D435" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E435" t="n">
+        <v>2.14</v>
+      </c>
+      <c r="F435" t="n">
+        <v>46.8</v>
+      </c>
+      <c r="G435" t="inlineStr">
+        <is>
+          <t>1-5</t>
+        </is>
+      </c>
+      <c r="H435" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I435" t="n">
+        <v>4</v>
+      </c>
+      <c r="J435" t="n">
+        <v>2</v>
+      </c>
+      <c r="K435" t="n">
+        <v>4</v>
+      </c>
+      <c r="L435" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B436" t="inlineStr">
+        <is>
+          <t>Alavés vs Málaga</t>
+        </is>
+      </c>
+      <c r="C436" t="inlineStr">
+        <is>
+          <t>Málaga</t>
+        </is>
+      </c>
+      <c r="D436" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E436" t="n">
+        <v>2.04</v>
+      </c>
+      <c r="F436" t="n">
+        <v>49</v>
+      </c>
+      <c r="G436" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H436" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I436" t="n">
+        <v>1</v>
+      </c>
+      <c r="J436" t="n">
+        <v>1</v>
+      </c>
+      <c r="K436" t="n">
+        <v>6</v>
+      </c>
+      <c r="L436" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B437" t="inlineStr">
+        <is>
+          <t>Torino vs Monza</t>
+        </is>
+      </c>
+      <c r="C437" t="inlineStr">
+        <is>
+          <t>Monza</t>
+        </is>
+      </c>
+      <c r="D437" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E437" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F437" t="n">
+        <v>66.59999999999999</v>
+      </c>
+      <c r="G437" t="inlineStr">
+        <is>
+          <t>3-2</t>
+        </is>
+      </c>
+      <c r="H437" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I437" t="n">
+        <v>1</v>
+      </c>
+      <c r="J437" t="n">
+        <v>0</v>
+      </c>
+      <c r="K437" t="n">
+        <v>1</v>
+      </c>
+      <c r="L437" t="inlineStr">
+        <is>
+          <t>si</t>
         </is>
       </c>
     </row>
@@ -22903,7 +23163,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E74"/>
+  <dimension ref="A1:E75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24270,6 +24530,25 @@
       </c>
       <c r="E74" t="n">
         <v>12</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B75" t="n">
+        <v>5</v>
+      </c>
+      <c r="C75" t="n">
+        <v>2</v>
+      </c>
+      <c r="D75" t="n">
+        <v>40</v>
+      </c>
+      <c r="E75" t="n">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -24283,7 +24562,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E237"/>
+  <dimension ref="A1:E240"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -29269,6 +29548,69 @@
         <v>33.3</v>
       </c>
     </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>cuidado_rival_presiona</t>
+        </is>
+      </c>
+      <c r="C238" t="n">
+        <v>3</v>
+      </c>
+      <c r="D238" t="n">
+        <v>0</v>
+      </c>
+      <c r="E238" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>ampliacion_marcador</t>
+        </is>
+      </c>
+      <c r="C239" t="n">
+        <v>4</v>
+      </c>
+      <c r="D239" t="n">
+        <v>2</v>
+      </c>
+      <c r="E239" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>partido_resuelto</t>
+        </is>
+      </c>
+      <c r="C240" t="n">
+        <v>1</v>
+      </c>
+      <c r="D240" t="n">
+        <v>0</v>
+      </c>
+      <c r="E240" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-10-25
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L437"/>
+  <dimension ref="A1:L466"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23147,6 +23147,1514 @@
         <v>1</v>
       </c>
       <c r="L437" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B438" t="inlineStr">
+        <is>
+          <t>Arsenal vs Everton</t>
+        </is>
+      </c>
+      <c r="C438" t="inlineStr">
+        <is>
+          <t>Arsenal</t>
+        </is>
+      </c>
+      <c r="D438" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E438" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="F438" t="n">
+        <v>89.40000000000001</v>
+      </c>
+      <c r="G438" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H438" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I438" t="n">
+        <v>0</v>
+      </c>
+      <c r="J438" t="n">
+        <v>7</v>
+      </c>
+      <c r="K438" t="n">
+        <v>3</v>
+      </c>
+      <c r="L438" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B439" t="inlineStr">
+        <is>
+          <t>Charlton Athletic vs Norwich City</t>
+        </is>
+      </c>
+      <c r="C439" t="inlineStr">
+        <is>
+          <t>Norwich City</t>
+        </is>
+      </c>
+      <c r="D439" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E439" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="F439" t="n">
+        <v>62.4</v>
+      </c>
+      <c r="G439" t="inlineStr">
+        <is>
+          <t>1-3</t>
+        </is>
+      </c>
+      <c r="H439" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I439" t="n">
+        <v>0</v>
+      </c>
+      <c r="J439" t="n">
+        <v>2</v>
+      </c>
+      <c r="K439" t="n">
+        <v>0</v>
+      </c>
+      <c r="L439" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B440" t="inlineStr">
+        <is>
+          <t>Wolverhampton Wanderers vs Watford</t>
+        </is>
+      </c>
+      <c r="C440" t="inlineStr">
+        <is>
+          <t>Wolverhampton Wanderers</t>
+        </is>
+      </c>
+      <c r="D440" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E440" t="n">
+        <v>1.29</v>
+      </c>
+      <c r="F440" t="n">
+        <v>77.5</v>
+      </c>
+      <c r="G440" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H440" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I440" t="n">
+        <v>0</v>
+      </c>
+      <c r="J440" t="n">
+        <v>5</v>
+      </c>
+      <c r="K440" t="n">
+        <v>8</v>
+      </c>
+      <c r="L440" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>Atlético Madrid vs Deportivo</t>
+        </is>
+      </c>
+      <c r="C441" t="inlineStr">
+        <is>
+          <t>Atlético Madrid</t>
+        </is>
+      </c>
+      <c r="D441" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E441" t="n">
+        <v>1.51</v>
+      </c>
+      <c r="F441" t="n">
+        <v>66.09999999999999</v>
+      </c>
+      <c r="G441" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H441" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I441" t="n">
+        <v>5</v>
+      </c>
+      <c r="J441" t="n">
+        <v>3</v>
+      </c>
+      <c r="K441" t="n">
+        <v>6</v>
+      </c>
+      <c r="L441" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B442" t="inlineStr">
+        <is>
+          <t>Como vs Sassuolo</t>
+        </is>
+      </c>
+      <c r="C442" t="inlineStr">
+        <is>
+          <t>Como</t>
+        </is>
+      </c>
+      <c r="D442" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E442" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="F442" t="n">
+        <v>83.09999999999999</v>
+      </c>
+      <c r="G442" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H442" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I442" t="n">
+        <v>0</v>
+      </c>
+      <c r="J442" t="n">
+        <v>4</v>
+      </c>
+      <c r="K442" t="n">
+        <v>0</v>
+      </c>
+      <c r="L442" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>Borussia Dortmund vs Eintracht Frankfurt</t>
+        </is>
+      </c>
+      <c r="C443" t="inlineStr">
+        <is>
+          <t>Borussia Dortmund</t>
+        </is>
+      </c>
+      <c r="D443" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E443" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="F443" t="n">
+        <v>78.7</v>
+      </c>
+      <c r="G443" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H443" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I443" t="n">
+        <v>0</v>
+      </c>
+      <c r="J443" t="n">
+        <v>2</v>
+      </c>
+      <c r="K443" t="n">
+        <v>0</v>
+      </c>
+      <c r="L443" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B444" t="inlineStr">
+        <is>
+          <t>Gil Vicente vs FC Porto</t>
+        </is>
+      </c>
+      <c r="C444" t="inlineStr">
+        <is>
+          <t>FC Porto</t>
+        </is>
+      </c>
+      <c r="D444" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E444" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="F444" t="n">
+        <v>72.7</v>
+      </c>
+      <c r="G444" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H444" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I444" t="n">
+        <v>4</v>
+      </c>
+      <c r="J444" t="n">
+        <v>3</v>
+      </c>
+      <c r="K444" t="n">
+        <v>2</v>
+      </c>
+      <c r="L444" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B445" t="inlineStr">
+        <is>
+          <t>Asteras Tripoli vs Levadiakos</t>
+        </is>
+      </c>
+      <c r="C445" t="inlineStr">
+        <is>
+          <t>Asteras Tripoli</t>
+        </is>
+      </c>
+      <c r="D445" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E445" t="n">
+        <v>2.03</v>
+      </c>
+      <c r="F445" t="n">
+        <v>49.4</v>
+      </c>
+      <c r="G445" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H445" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I445" t="n">
+        <v>0</v>
+      </c>
+      <c r="J445" t="n">
+        <v>4</v>
+      </c>
+      <c r="K445" t="n">
+        <v>4</v>
+      </c>
+      <c r="L445" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B446" t="inlineStr">
+        <is>
+          <t>AEK Athens vs Panetolikos</t>
+        </is>
+      </c>
+      <c r="C446" t="inlineStr">
+        <is>
+          <t>AEK Athens</t>
+        </is>
+      </c>
+      <c r="D446" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E446" t="n">
+        <v>1.49</v>
+      </c>
+      <c r="F446" t="n">
+        <v>67.09999999999999</v>
+      </c>
+      <c r="G446" t="inlineStr">
+        <is>
+          <t>5-0</t>
+        </is>
+      </c>
+      <c r="H446" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I446" t="n">
+        <v>1</v>
+      </c>
+      <c r="J446" t="n">
+        <v>7</v>
+      </c>
+      <c r="K446" t="n">
+        <v>2</v>
+      </c>
+      <c r="L446" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B447" t="inlineStr">
+        <is>
+          <t>Chapecoense vs Fluminense</t>
+        </is>
+      </c>
+      <c r="C447" t="inlineStr">
+        <is>
+          <t>Chapecoense</t>
+        </is>
+      </c>
+      <c r="D447" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E447" t="n">
+        <v>2.31</v>
+      </c>
+      <c r="F447" t="n">
+        <v>43.3</v>
+      </c>
+      <c r="G447" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H447" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I447" t="n">
+        <v>2</v>
+      </c>
+      <c r="J447" t="n">
+        <v>3</v>
+      </c>
+      <c r="K447" t="n">
+        <v>8</v>
+      </c>
+      <c r="L447" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B448" t="inlineStr">
+        <is>
+          <t>Red Bull New York vs Inter Miami CF</t>
+        </is>
+      </c>
+      <c r="C448" t="inlineStr">
+        <is>
+          <t>Red Bull New York</t>
+        </is>
+      </c>
+      <c r="D448" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E448" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F448" t="n">
+        <v>40</v>
+      </c>
+      <c r="G448" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H448" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I448" t="n">
+        <v>5</v>
+      </c>
+      <c r="J448" t="n">
+        <v>0</v>
+      </c>
+      <c r="K448" t="n">
+        <v>1</v>
+      </c>
+      <c r="L448" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B449" t="inlineStr">
+        <is>
+          <t>Colorado Rapids vs Vancouver Whitecaps</t>
+        </is>
+      </c>
+      <c r="C449" t="inlineStr">
+        <is>
+          <t>Colorado Rapids</t>
+        </is>
+      </c>
+      <c r="D449" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E449" t="n">
+        <v>2.59</v>
+      </c>
+      <c r="F449" t="n">
+        <v>38.6</v>
+      </c>
+      <c r="G449" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H449" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I449" t="n">
+        <v>0</v>
+      </c>
+      <c r="J449" t="n">
+        <v>0</v>
+      </c>
+      <c r="K449" t="n">
+        <v>7</v>
+      </c>
+      <c r="L449" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B450" t="inlineStr">
+        <is>
+          <t>Aston Villa vs Manchester City</t>
+        </is>
+      </c>
+      <c r="C450" t="inlineStr">
+        <is>
+          <t>Manchester City</t>
+        </is>
+      </c>
+      <c r="D450" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E450" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="F450" t="n">
+        <v>67.40000000000001</v>
+      </c>
+      <c r="G450" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H450" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I450" t="n">
+        <v>0</v>
+      </c>
+      <c r="J450" t="n">
+        <v>1</v>
+      </c>
+      <c r="K450" t="n">
+        <v>6</v>
+      </c>
+      <c r="L450" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B451" t="inlineStr">
+        <is>
+          <t>Coventry City vs Fulham</t>
+        </is>
+      </c>
+      <c r="C451" t="inlineStr">
+        <is>
+          <t>Coventry City</t>
+        </is>
+      </c>
+      <c r="D451" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E451" t="n">
+        <v>1.13</v>
+      </c>
+      <c r="F451" t="n">
+        <v>88.5</v>
+      </c>
+      <c r="G451" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H451" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I451" t="n">
+        <v>0</v>
+      </c>
+      <c r="J451" t="n">
+        <v>2</v>
+      </c>
+      <c r="K451" t="n">
+        <v>4</v>
+      </c>
+      <c r="L451" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B452" t="inlineStr">
+        <is>
+          <t>Lincoln City vs Burnley</t>
+        </is>
+      </c>
+      <c r="C452" t="inlineStr">
+        <is>
+          <t>Lincoln City</t>
+        </is>
+      </c>
+      <c r="D452" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E452" t="n">
+        <v>1.41</v>
+      </c>
+      <c r="F452" t="n">
+        <v>71</v>
+      </c>
+      <c r="G452" t="inlineStr">
+        <is>
+          <t>4-1</t>
+        </is>
+      </c>
+      <c r="H452" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I452" t="n">
+        <v>0</v>
+      </c>
+      <c r="J452" t="n">
+        <v>2</v>
+      </c>
+      <c r="K452" t="n">
+        <v>2</v>
+      </c>
+      <c r="L452" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B453" t="inlineStr">
+        <is>
+          <t>Rayo Vallecano vs Elche</t>
+        </is>
+      </c>
+      <c r="C453" t="inlineStr">
+        <is>
+          <t>Rayo Vallecano</t>
+        </is>
+      </c>
+      <c r="D453" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E453" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="F453" t="n">
+        <v>68.90000000000001</v>
+      </c>
+      <c r="G453" t="inlineStr">
+        <is>
+          <t>0-3</t>
+        </is>
+      </c>
+      <c r="H453" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I453" t="n">
+        <v>0</v>
+      </c>
+      <c r="J453" t="n">
+        <v>3</v>
+      </c>
+      <c r="K453" t="n">
+        <v>8</v>
+      </c>
+      <c r="L453" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B454" t="inlineStr">
+        <is>
+          <t>Racing Santander vs Espanyol</t>
+        </is>
+      </c>
+      <c r="C454" t="inlineStr">
+        <is>
+          <t>Racing Santander</t>
+        </is>
+      </c>
+      <c r="D454" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E454" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="F454" t="n">
+        <v>76.7</v>
+      </c>
+      <c r="G454" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H454" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I454" t="n">
+        <v>0</v>
+      </c>
+      <c r="J454" t="n">
+        <v>6</v>
+      </c>
+      <c r="K454" t="n">
+        <v>3</v>
+      </c>
+      <c r="L454" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B455" t="inlineStr">
+        <is>
+          <t>Almería vs Real Oviedo</t>
+        </is>
+      </c>
+      <c r="C455" t="inlineStr">
+        <is>
+          <t>Almería</t>
+        </is>
+      </c>
+      <c r="D455" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E455" t="n">
+        <v>1.17</v>
+      </c>
+      <c r="F455" t="n">
+        <v>85.59999999999999</v>
+      </c>
+      <c r="G455" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="H455" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I455" t="n">
+        <v>7</v>
+      </c>
+      <c r="J455" t="n">
+        <v>2</v>
+      </c>
+      <c r="K455" t="n">
+        <v>4</v>
+      </c>
+      <c r="L455" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B456" t="inlineStr">
+        <is>
+          <t>Napoli vs AS Roma</t>
+        </is>
+      </c>
+      <c r="C456" t="inlineStr">
+        <is>
+          <t>AS Roma</t>
+        </is>
+      </c>
+      <c r="D456" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E456" t="n">
+        <v>1.74</v>
+      </c>
+      <c r="F456" t="n">
+        <v>57.5</v>
+      </c>
+      <c r="G456" t="inlineStr">
+        <is>
+          <t>3-3</t>
+        </is>
+      </c>
+      <c r="H456" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I456" t="n">
+        <v>0</v>
+      </c>
+      <c r="J456" t="n">
+        <v>0</v>
+      </c>
+      <c r="K456" t="n">
+        <v>3</v>
+      </c>
+      <c r="L456" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B457" t="inlineStr">
+        <is>
+          <t>FC Utrecht vs PEC Zwolle</t>
+        </is>
+      </c>
+      <c r="C457" t="inlineStr">
+        <is>
+          <t>FC Utrecht</t>
+        </is>
+      </c>
+      <c r="D457" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E457" t="n">
+        <v>1.13</v>
+      </c>
+      <c r="F457" t="n">
+        <v>88.40000000000001</v>
+      </c>
+      <c r="G457" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H457" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I457" t="n">
+        <v>0</v>
+      </c>
+      <c r="J457" t="n">
+        <v>6</v>
+      </c>
+      <c r="K457" t="n">
+        <v>5</v>
+      </c>
+      <c r="L457" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B458" t="inlineStr">
+        <is>
+          <t>Willem II vs SC Cambuur</t>
+        </is>
+      </c>
+      <c r="C458" t="inlineStr">
+        <is>
+          <t>SC Cambuur</t>
+        </is>
+      </c>
+      <c r="D458" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E458" t="n">
+        <v>2.52</v>
+      </c>
+      <c r="F458" t="n">
+        <v>39.7</v>
+      </c>
+      <c r="G458" t="inlineStr">
+        <is>
+          <t>1-6</t>
+        </is>
+      </c>
+      <c r="H458" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I458" t="n">
+        <v>1</v>
+      </c>
+      <c r="J458" t="n">
+        <v>6</v>
+      </c>
+      <c r="K458" t="n">
+        <v>4</v>
+      </c>
+      <c r="L458" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B459" t="inlineStr">
+        <is>
+          <t>Estrela vs Casa Pia</t>
+        </is>
+      </c>
+      <c r="C459" t="inlineStr">
+        <is>
+          <t>Estrela</t>
+        </is>
+      </c>
+      <c r="D459" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E459" t="n">
+        <v>1.94</v>
+      </c>
+      <c r="F459" t="n">
+        <v>51.5</v>
+      </c>
+      <c r="G459" t="inlineStr">
+        <is>
+          <t>0-2</t>
+        </is>
+      </c>
+      <c r="H459" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I459" t="n">
+        <v>0</v>
+      </c>
+      <c r="J459" t="n">
+        <v>1</v>
+      </c>
+      <c r="K459" t="n">
+        <v>3</v>
+      </c>
+      <c r="L459" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B460" t="inlineStr">
+        <is>
+          <t>Antwerp vs Royal Charleroi SC</t>
+        </is>
+      </c>
+      <c r="C460" t="inlineStr">
+        <is>
+          <t>Royal Charleroi SC</t>
+        </is>
+      </c>
+      <c r="D460" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E460" t="n">
+        <v>1.39</v>
+      </c>
+      <c r="F460" t="n">
+        <v>72</v>
+      </c>
+      <c r="G460" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="H460" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I460" t="n">
+        <v>0</v>
+      </c>
+      <c r="J460" t="n">
+        <v>2</v>
+      </c>
+      <c r="K460" t="n">
+        <v>0</v>
+      </c>
+      <c r="L460" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B461" t="inlineStr">
+        <is>
+          <t>RAAL La Louvière vs Zulte-Waregem</t>
+        </is>
+      </c>
+      <c r="C461" t="inlineStr">
+        <is>
+          <t>Zulte-Waregem</t>
+        </is>
+      </c>
+      <c r="D461" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E461" t="n">
+        <v>1.39</v>
+      </c>
+      <c r="F461" t="n">
+        <v>71.7</v>
+      </c>
+      <c r="G461" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="H461" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I461" t="n">
+        <v>6</v>
+      </c>
+      <c r="J461" t="n">
+        <v>1</v>
+      </c>
+      <c r="K461" t="n">
+        <v>3</v>
+      </c>
+      <c r="L461" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B462" t="inlineStr">
+        <is>
+          <t>Eyupspor vs Kasimpasa</t>
+        </is>
+      </c>
+      <c r="C462" t="inlineStr">
+        <is>
+          <t>Eyupspor</t>
+        </is>
+      </c>
+      <c r="D462" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E462" t="n">
+        <v>1.34</v>
+      </c>
+      <c r="F462" t="n">
+        <v>74.7</v>
+      </c>
+      <c r="G462" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H462" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I462" t="n">
+        <v>0</v>
+      </c>
+      <c r="J462" t="n">
+        <v>0</v>
+      </c>
+      <c r="K462" t="n">
+        <v>1</v>
+      </c>
+      <c r="L462" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B463" t="inlineStr">
+        <is>
+          <t>Iraklis vs Kifisia</t>
+        </is>
+      </c>
+      <c r="C463" t="inlineStr">
+        <is>
+          <t>Iraklis</t>
+        </is>
+      </c>
+      <c r="D463" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E463" t="n">
+        <v>1.86</v>
+      </c>
+      <c r="F463" t="n">
+        <v>53.7</v>
+      </c>
+      <c r="G463" t="inlineStr">
+        <is>
+          <t>2-3</t>
+        </is>
+      </c>
+      <c r="H463" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I463" t="n">
+        <v>0</v>
+      </c>
+      <c r="J463" t="n">
+        <v>2</v>
+      </c>
+      <c r="K463" t="n">
+        <v>6</v>
+      </c>
+      <c r="L463" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B464" t="inlineStr">
+        <is>
+          <t>Mirassol vs São Paulo</t>
+        </is>
+      </c>
+      <c r="C464" t="inlineStr">
+        <is>
+          <t>Mirassol</t>
+        </is>
+      </c>
+      <c r="D464" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E464" t="n">
+        <v>1.19</v>
+      </c>
+      <c r="F464" t="n">
+        <v>84.3</v>
+      </c>
+      <c r="G464" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H464" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I464" t="n">
+        <v>4</v>
+      </c>
+      <c r="J464" t="n">
+        <v>0</v>
+      </c>
+      <c r="K464" t="n">
+        <v>6</v>
+      </c>
+      <c r="L464" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B465" t="inlineStr">
+        <is>
+          <t>Banfield vs Lanús</t>
+        </is>
+      </c>
+      <c r="C465" t="inlineStr">
+        <is>
+          <t>Lanús</t>
+        </is>
+      </c>
+      <c r="D465" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E465" t="n">
+        <v>2.39</v>
+      </c>
+      <c r="F465" t="n">
+        <v>41.9</v>
+      </c>
+      <c r="G465" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H465" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I465" t="n">
+        <v>2</v>
+      </c>
+      <c r="J465" t="n">
+        <v>1</v>
+      </c>
+      <c r="K465" t="n">
+        <v>2</v>
+      </c>
+      <c r="L465" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B466" t="inlineStr">
+        <is>
+          <t>Houston Dynamo FC vs Minnesota United FC</t>
+        </is>
+      </c>
+      <c r="C466" t="inlineStr">
+        <is>
+          <t>Minnesota United FC</t>
+        </is>
+      </c>
+      <c r="D466" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E466" t="n">
+        <v>2.59</v>
+      </c>
+      <c r="F466" t="n">
+        <v>38.7</v>
+      </c>
+      <c r="G466" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H466" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I466" t="n">
+        <v>0</v>
+      </c>
+      <c r="J466" t="n">
+        <v>0</v>
+      </c>
+      <c r="K466" t="n">
+        <v>3</v>
+      </c>
+      <c r="L466" t="inlineStr">
         <is>
           <t>si</t>
         </is>
@@ -23163,7 +24671,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E75"/>
+  <dimension ref="A1:E76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24549,6 +26057,25 @@
       </c>
       <c r="E75" t="n">
         <v>5</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B76" t="n">
+        <v>29</v>
+      </c>
+      <c r="C76" t="n">
+        <v>14</v>
+      </c>
+      <c r="D76" t="n">
+        <v>48.3</v>
+      </c>
+      <c r="E76" t="n">
+        <v>29</v>
       </c>
     </row>
   </sheetData>
@@ -24562,7 +26089,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E240"/>
+  <dimension ref="A1:E247"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -29611,6 +31138,153 @@
         <v>0</v>
       </c>
     </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>cuidado_rival_presiona</t>
+        </is>
+      </c>
+      <c r="C241" t="n">
+        <v>11</v>
+      </c>
+      <c r="D241" t="n">
+        <v>0</v>
+      </c>
+      <c r="E241" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>ampliacion_marcador</t>
+        </is>
+      </c>
+      <c r="C242" t="n">
+        <v>13</v>
+      </c>
+      <c r="D242" t="n">
+        <v>1</v>
+      </c>
+      <c r="E242" t="n">
+        <v>7.7</v>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>alerta_1er_tiempo</t>
+        </is>
+      </c>
+      <c r="C243" t="n">
+        <v>2</v>
+      </c>
+      <c r="D243" t="n">
+        <v>0</v>
+      </c>
+      <c r="E243" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>posible_victoria_favorito</t>
+        </is>
+      </c>
+      <c r="C244" t="n">
+        <v>5</v>
+      </c>
+      <c r="D244" t="n">
+        <v>0</v>
+      </c>
+      <c r="E244" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>tarjeta_roja</t>
+        </is>
+      </c>
+      <c r="C245" t="n">
+        <v>2</v>
+      </c>
+      <c r="D245" t="n">
+        <v>0</v>
+      </c>
+      <c r="E245" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>partido_resuelto</t>
+        </is>
+      </c>
+      <c r="C246" t="n">
+        <v>3</v>
+      </c>
+      <c r="D246" t="n">
+        <v>0</v>
+      </c>
+      <c r="E246" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>posible_empate</t>
+        </is>
+      </c>
+      <c r="C247" t="n">
+        <v>1</v>
+      </c>
+      <c r="D247" t="n">
+        <v>0</v>
+      </c>
+      <c r="E247" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-10-26
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L466"/>
+  <dimension ref="A1:L490"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24655,6 +24655,1254 @@
         <v>3</v>
       </c>
       <c r="L466" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B467" t="inlineStr">
+        <is>
+          <t>Hull City vs Brentford</t>
+        </is>
+      </c>
+      <c r="C467" t="inlineStr">
+        <is>
+          <t>Hull City</t>
+        </is>
+      </c>
+      <c r="D467" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E467" t="n">
+        <v>2.18</v>
+      </c>
+      <c r="F467" t="n">
+        <v>45.9</v>
+      </c>
+      <c r="G467" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H467" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I467" t="n">
+        <v>0</v>
+      </c>
+      <c r="J467" t="n">
+        <v>2</v>
+      </c>
+      <c r="K467" t="n">
+        <v>1</v>
+      </c>
+      <c r="L467" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B468" t="inlineStr">
+        <is>
+          <t>Athletic Club vs Getafe</t>
+        </is>
+      </c>
+      <c r="C468" t="inlineStr">
+        <is>
+          <t>Athletic Club</t>
+        </is>
+      </c>
+      <c r="D468" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E468" t="n">
+        <v>2.27</v>
+      </c>
+      <c r="F468" t="n">
+        <v>44.1</v>
+      </c>
+      <c r="G468" t="inlineStr">
+        <is>
+          <t>4-0</t>
+        </is>
+      </c>
+      <c r="H468" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I468" t="n">
+        <v>0</v>
+      </c>
+      <c r="J468" t="n">
+        <v>2</v>
+      </c>
+      <c r="K468" t="n">
+        <v>3</v>
+      </c>
+      <c r="L468" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B469" t="inlineStr">
+        <is>
+          <t>Genoa vs Venezia</t>
+        </is>
+      </c>
+      <c r="C469" t="inlineStr">
+        <is>
+          <t>Venezia</t>
+        </is>
+      </c>
+      <c r="D469" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E469" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="F469" t="n">
+        <v>84.59999999999999</v>
+      </c>
+      <c r="G469" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H469" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I469" t="n">
+        <v>0</v>
+      </c>
+      <c r="J469" t="n">
+        <v>3</v>
+      </c>
+      <c r="K469" t="n">
+        <v>0</v>
+      </c>
+      <c r="L469" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B470" t="inlineStr">
+        <is>
+          <t>PSV Eindhoven vs Feyenoord Rotterdam</t>
+        </is>
+      </c>
+      <c r="C470" t="inlineStr">
+        <is>
+          <t>PSV Eindhoven</t>
+        </is>
+      </c>
+      <c r="D470" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E470" t="n">
+        <v>1.58</v>
+      </c>
+      <c r="F470" t="n">
+        <v>63.4</v>
+      </c>
+      <c r="G470" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H470" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I470" t="n">
+        <v>0</v>
+      </c>
+      <c r="J470" t="n">
+        <v>8</v>
+      </c>
+      <c r="K470" t="n">
+        <v>6</v>
+      </c>
+      <c r="L470" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B471" t="inlineStr">
+        <is>
+          <t>Sparta Rotterdam vs Ajax Amsterdam</t>
+        </is>
+      </c>
+      <c r="C471" t="inlineStr">
+        <is>
+          <t>Ajax Amsterdam</t>
+        </is>
+      </c>
+      <c r="D471" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E471" t="n">
+        <v>1.67</v>
+      </c>
+      <c r="F471" t="n">
+        <v>60</v>
+      </c>
+      <c r="G471" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H471" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I471" t="n">
+        <v>0</v>
+      </c>
+      <c r="J471" t="n">
+        <v>7</v>
+      </c>
+      <c r="K471" t="n">
+        <v>6</v>
+      </c>
+      <c r="L471" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B472" t="inlineStr">
+        <is>
+          <t>C.D. Nacional vs Braga</t>
+        </is>
+      </c>
+      <c r="C472" t="inlineStr">
+        <is>
+          <t>Braga</t>
+        </is>
+      </c>
+      <c r="D472" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E472" t="n">
+        <v>2.29</v>
+      </c>
+      <c r="F472" t="n">
+        <v>43.6</v>
+      </c>
+      <c r="G472" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H472" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I472" t="n">
+        <v>2</v>
+      </c>
+      <c r="J472" t="n">
+        <v>1</v>
+      </c>
+      <c r="K472" t="n">
+        <v>3</v>
+      </c>
+      <c r="L472" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B473" t="inlineStr">
+        <is>
+          <t>Sporting CP vs Académico de Viseu</t>
+        </is>
+      </c>
+      <c r="C473" t="inlineStr">
+        <is>
+          <t>Sporting CP</t>
+        </is>
+      </c>
+      <c r="D473" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E473" t="n">
+        <v>2.09</v>
+      </c>
+      <c r="F473" t="n">
+        <v>48</v>
+      </c>
+      <c r="G473" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H473" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I473" t="n">
+        <v>7</v>
+      </c>
+      <c r="J473" t="n">
+        <v>6</v>
+      </c>
+      <c r="K473" t="n">
+        <v>2</v>
+      </c>
+      <c r="L473" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B474" t="inlineStr">
+        <is>
+          <t>Racing Genk vs Standard Liege</t>
+        </is>
+      </c>
+      <c r="C474" t="inlineStr">
+        <is>
+          <t>Racing Genk</t>
+        </is>
+      </c>
+      <c r="D474" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E474" t="n">
+        <v>2.51</v>
+      </c>
+      <c r="F474" t="n">
+        <v>39.9</v>
+      </c>
+      <c r="G474" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H474" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I474" t="n">
+        <v>0</v>
+      </c>
+      <c r="J474" t="n">
+        <v>2</v>
+      </c>
+      <c r="K474" t="n">
+        <v>1</v>
+      </c>
+      <c r="L474" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>Club Brugge vs Sint-Truidense</t>
+        </is>
+      </c>
+      <c r="C475" t="inlineStr">
+        <is>
+          <t>Club Brugge</t>
+        </is>
+      </c>
+      <c r="D475" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E475" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="F475" t="n">
+        <v>87.2</v>
+      </c>
+      <c r="G475" t="inlineStr">
+        <is>
+          <t>3-2</t>
+        </is>
+      </c>
+      <c r="H475" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I475" t="n">
+        <v>0</v>
+      </c>
+      <c r="J475" t="n">
+        <v>7</v>
+      </c>
+      <c r="K475" t="n">
+        <v>2</v>
+      </c>
+      <c r="L475" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B476" t="inlineStr">
+        <is>
+          <t>Union St.-Gilloise vs Cercle Brugge KSV</t>
+        </is>
+      </c>
+      <c r="C476" t="inlineStr">
+        <is>
+          <t>Union St.-Gilloise</t>
+        </is>
+      </c>
+      <c r="D476" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E476" t="n">
+        <v>1.41</v>
+      </c>
+      <c r="F476" t="n">
+        <v>70.7</v>
+      </c>
+      <c r="G476" t="inlineStr">
+        <is>
+          <t>5-2</t>
+        </is>
+      </c>
+      <c r="H476" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I476" t="n">
+        <v>8</v>
+      </c>
+      <c r="J476" t="n">
+        <v>6</v>
+      </c>
+      <c r="K476" t="n">
+        <v>1</v>
+      </c>
+      <c r="L476" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B477" t="inlineStr">
+        <is>
+          <t>Goztepe vs Çorum FK</t>
+        </is>
+      </c>
+      <c r="C477" t="inlineStr">
+        <is>
+          <t>Goztepe</t>
+        </is>
+      </c>
+      <c r="D477" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E477" t="n">
+        <v>2.06</v>
+      </c>
+      <c r="F477" t="n">
+        <v>48.6</v>
+      </c>
+      <c r="G477" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H477" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I477" t="n">
+        <v>0</v>
+      </c>
+      <c r="J477" t="n">
+        <v>1</v>
+      </c>
+      <c r="K477" t="n">
+        <v>2</v>
+      </c>
+      <c r="L477" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B478" t="inlineStr">
+        <is>
+          <t>Olympiacos vs Kalamata</t>
+        </is>
+      </c>
+      <c r="C478" t="inlineStr">
+        <is>
+          <t>Olympiacos</t>
+        </is>
+      </c>
+      <c r="D478" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E478" t="n">
+        <v>1.59</v>
+      </c>
+      <c r="F478" t="n">
+        <v>63.1</v>
+      </c>
+      <c r="G478" t="inlineStr">
+        <is>
+          <t>5-0</t>
+        </is>
+      </c>
+      <c r="H478" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I478" t="n">
+        <v>0</v>
+      </c>
+      <c r="J478" t="n">
+        <v>8</v>
+      </c>
+      <c r="K478" t="n">
+        <v>4</v>
+      </c>
+      <c r="L478" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B479" t="inlineStr">
+        <is>
+          <t>Volos NFC vs Panathinaikos</t>
+        </is>
+      </c>
+      <c r="C479" t="inlineStr">
+        <is>
+          <t>Panathinaikos</t>
+        </is>
+      </c>
+      <c r="D479" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E479" t="n">
+        <v>1.17</v>
+      </c>
+      <c r="F479" t="n">
+        <v>85.40000000000001</v>
+      </c>
+      <c r="G479" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H479" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I479" t="n">
+        <v>0</v>
+      </c>
+      <c r="J479" t="n">
+        <v>5</v>
+      </c>
+      <c r="K479" t="n">
+        <v>5</v>
+      </c>
+      <c r="L479" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B480" t="inlineStr">
+        <is>
+          <t>River Plate vs Racing Club</t>
+        </is>
+      </c>
+      <c r="C480" t="inlineStr">
+        <is>
+          <t>River Plate</t>
+        </is>
+      </c>
+      <c r="D480" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E480" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="F480" t="n">
+        <v>44.4</v>
+      </c>
+      <c r="G480" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H480" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I480" t="n">
+        <v>3</v>
+      </c>
+      <c r="J480" t="n">
+        <v>1</v>
+      </c>
+      <c r="K480" t="n">
+        <v>1</v>
+      </c>
+      <c r="L480" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B481" t="inlineStr">
+        <is>
+          <t>Celta Vigo vs Real Betis</t>
+        </is>
+      </c>
+      <c r="C481" t="inlineStr">
+        <is>
+          <t>Real Betis</t>
+        </is>
+      </c>
+      <c r="D481" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E481" t="n">
+        <v>2.01</v>
+      </c>
+      <c r="F481" t="n">
+        <v>49.9</v>
+      </c>
+      <c r="G481" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H481" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I481" t="n">
+        <v>0</v>
+      </c>
+      <c r="J481" t="n">
+        <v>4</v>
+      </c>
+      <c r="K481" t="n">
+        <v>4</v>
+      </c>
+      <c r="L481" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B482" t="inlineStr">
+        <is>
+          <t>Barcelona vs Real Madrid</t>
+        </is>
+      </c>
+      <c r="C482" t="inlineStr">
+        <is>
+          <t>Barcelona</t>
+        </is>
+      </c>
+      <c r="D482" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E482" t="n">
+        <v>1.54</v>
+      </c>
+      <c r="F482" t="n">
+        <v>65.09999999999999</v>
+      </c>
+      <c r="G482" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H482" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I482" t="n">
+        <v>3</v>
+      </c>
+      <c r="J482" t="n">
+        <v>12</v>
+      </c>
+      <c r="K482" t="n">
+        <v>8</v>
+      </c>
+      <c r="L482" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>Internazionale vs Fiorentina</t>
+        </is>
+      </c>
+      <c r="C483" t="inlineStr">
+        <is>
+          <t>Internazionale</t>
+        </is>
+      </c>
+      <c r="D483" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E483" t="n">
+        <v>1.32</v>
+      </c>
+      <c r="F483" t="n">
+        <v>75.90000000000001</v>
+      </c>
+      <c r="G483" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H483" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I483" t="n">
+        <v>0</v>
+      </c>
+      <c r="J483" t="n">
+        <v>5</v>
+      </c>
+      <c r="K483" t="n">
+        <v>2</v>
+      </c>
+      <c r="L483" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B484" t="inlineStr">
+        <is>
+          <t>SC Freiburg vs Bayern Munich</t>
+        </is>
+      </c>
+      <c r="C484" t="inlineStr">
+        <is>
+          <t>Bayern Munich</t>
+        </is>
+      </c>
+      <c r="D484" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E484" t="n">
+        <v>1.24</v>
+      </c>
+      <c r="F484" t="n">
+        <v>80.5</v>
+      </c>
+      <c r="G484" t="inlineStr">
+        <is>
+          <t>1-3</t>
+        </is>
+      </c>
+      <c r="H484" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I484" t="n">
+        <v>0</v>
+      </c>
+      <c r="J484" t="n">
+        <v>2</v>
+      </c>
+      <c r="K484" t="n">
+        <v>8</v>
+      </c>
+      <c r="L484" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>Angers vs Lorient</t>
+        </is>
+      </c>
+      <c r="C485" t="inlineStr">
+        <is>
+          <t>Lorient</t>
+        </is>
+      </c>
+      <c r="D485" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E485" t="n">
+        <v>2.07</v>
+      </c>
+      <c r="F485" t="n">
+        <v>48.3</v>
+      </c>
+      <c r="G485" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H485" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I485" t="n">
+        <v>0</v>
+      </c>
+      <c r="J485" t="n">
+        <v>0</v>
+      </c>
+      <c r="K485" t="n">
+        <v>1</v>
+      </c>
+      <c r="L485" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>Marseille vs Le Havre AC</t>
+        </is>
+      </c>
+      <c r="C486" t="inlineStr">
+        <is>
+          <t>Marseille</t>
+        </is>
+      </c>
+      <c r="D486" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E486" t="n">
+        <v>2.04</v>
+      </c>
+      <c r="F486" t="n">
+        <v>49.1</v>
+      </c>
+      <c r="G486" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="H486" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I486" t="n">
+        <v>0</v>
+      </c>
+      <c r="J486" t="n">
+        <v>3</v>
+      </c>
+      <c r="K486" t="n">
+        <v>0</v>
+      </c>
+      <c r="L486" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>Stade Rennais vs Strasbourg</t>
+        </is>
+      </c>
+      <c r="C487" t="inlineStr">
+        <is>
+          <t>Stade Rennais</t>
+        </is>
+      </c>
+      <c r="D487" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E487" t="n">
+        <v>1.32</v>
+      </c>
+      <c r="F487" t="n">
+        <v>75.8</v>
+      </c>
+      <c r="G487" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="H487" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I487" t="n">
+        <v>0</v>
+      </c>
+      <c r="J487" t="n">
+        <v>4</v>
+      </c>
+      <c r="K487" t="n">
+        <v>3</v>
+      </c>
+      <c r="L487" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B488" t="inlineStr">
+        <is>
+          <t>Fortuna Sittard vs Excelsior</t>
+        </is>
+      </c>
+      <c r="C488" t="inlineStr">
+        <is>
+          <t>Excelsior</t>
+        </is>
+      </c>
+      <c r="D488" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E488" t="n">
+        <v>1.67</v>
+      </c>
+      <c r="F488" t="n">
+        <v>59.7</v>
+      </c>
+      <c r="G488" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H488" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I488" t="n">
+        <v>0</v>
+      </c>
+      <c r="J488" t="n">
+        <v>4</v>
+      </c>
+      <c r="K488" t="n">
+        <v>5</v>
+      </c>
+      <c r="L488" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B489" t="inlineStr">
+        <is>
+          <t>Estoril vs Moreirense</t>
+        </is>
+      </c>
+      <c r="C489" t="inlineStr">
+        <is>
+          <t>Moreirense</t>
+        </is>
+      </c>
+      <c r="D489" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E489" t="n">
+        <v>2.55</v>
+      </c>
+      <c r="F489" t="n">
+        <v>39.3</v>
+      </c>
+      <c r="G489" t="inlineStr">
+        <is>
+          <t>1-3</t>
+        </is>
+      </c>
+      <c r="H489" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I489" t="n">
+        <v>0</v>
+      </c>
+      <c r="J489" t="n">
+        <v>3</v>
+      </c>
+      <c r="K489" t="n">
+        <v>2</v>
+      </c>
+      <c r="L489" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B490" t="inlineStr">
+        <is>
+          <t>Aris vs Atromitos</t>
+        </is>
+      </c>
+      <c r="C490" t="inlineStr">
+        <is>
+          <t>Aris</t>
+        </is>
+      </c>
+      <c r="D490" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E490" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F490" t="n">
+        <v>66.59999999999999</v>
+      </c>
+      <c r="G490" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="H490" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I490" t="n">
+        <v>2</v>
+      </c>
+      <c r="J490" t="n">
+        <v>4</v>
+      </c>
+      <c r="K490" t="n">
+        <v>3</v>
+      </c>
+      <c r="L490" t="inlineStr">
         <is>
           <t>si</t>
         </is>
@@ -24671,7 +25919,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E76"/>
+  <dimension ref="A1:E77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26076,6 +27324,25 @@
       </c>
       <c r="E76" t="n">
         <v>29</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B77" t="n">
+        <v>24</v>
+      </c>
+      <c r="C77" t="n">
+        <v>15</v>
+      </c>
+      <c r="D77" t="n">
+        <v>62.5</v>
+      </c>
+      <c r="E77" t="n">
+        <v>24</v>
       </c>
     </row>
   </sheetData>
@@ -26089,7 +27356,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E247"/>
+  <dimension ref="A1:E254"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -31285,6 +32552,153 @@
         <v>0</v>
       </c>
     </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>posible_empate</t>
+        </is>
+      </c>
+      <c r="C248" t="n">
+        <v>7</v>
+      </c>
+      <c r="D248" t="n">
+        <v>2</v>
+      </c>
+      <c r="E248" t="n">
+        <v>28.6</v>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>cuidado_rival_presiona</t>
+        </is>
+      </c>
+      <c r="C249" t="n">
+        <v>4</v>
+      </c>
+      <c r="D249" t="n">
+        <v>0</v>
+      </c>
+      <c r="E249" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>posible_victoria_favorito</t>
+        </is>
+      </c>
+      <c r="C250" t="n">
+        <v>7</v>
+      </c>
+      <c r="D250" t="n">
+        <v>1</v>
+      </c>
+      <c r="E250" t="n">
+        <v>14.3</v>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>gol_de_cierre</t>
+        </is>
+      </c>
+      <c r="C251" t="n">
+        <v>2</v>
+      </c>
+      <c r="D251" t="n">
+        <v>1</v>
+      </c>
+      <c r="E251" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>tarjeta_roja</t>
+        </is>
+      </c>
+      <c r="C252" t="n">
+        <v>1</v>
+      </c>
+      <c r="D252" t="n">
+        <v>0</v>
+      </c>
+      <c r="E252" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>ampliacion_marcador</t>
+        </is>
+      </c>
+      <c r="C253" t="n">
+        <v>3</v>
+      </c>
+      <c r="D253" t="n">
+        <v>1</v>
+      </c>
+      <c r="E253" t="n">
+        <v>33.3</v>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>partido_resuelto</t>
+        </is>
+      </c>
+      <c r="C254" t="n">
+        <v>1</v>
+      </c>
+      <c r="D254" t="n">
+        <v>0</v>
+      </c>
+      <c r="E254" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-10-27
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L490"/>
+  <dimension ref="A1:L496"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -25903,6 +25903,318 @@
         <v>3</v>
       </c>
       <c r="L490" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B491" t="inlineStr">
+        <is>
+          <t>Paris Saint-Germain vs Lyon</t>
+        </is>
+      </c>
+      <c r="C491" t="inlineStr">
+        <is>
+          <t>Paris Saint-Germain</t>
+        </is>
+      </c>
+      <c r="D491" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E491" t="n">
+        <v>1.67</v>
+      </c>
+      <c r="F491" t="n">
+        <v>59.9</v>
+      </c>
+      <c r="G491" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H491" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I491" t="n">
+        <v>3</v>
+      </c>
+      <c r="J491" t="n">
+        <v>8</v>
+      </c>
+      <c r="K491" t="n">
+        <v>2</v>
+      </c>
+      <c r="L491" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B492" t="inlineStr">
+        <is>
+          <t>Santa Clara vs Benfica</t>
+        </is>
+      </c>
+      <c r="C492" t="inlineStr">
+        <is>
+          <t>Benfica</t>
+        </is>
+      </c>
+      <c r="D492" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E492" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="F492" t="n">
+        <v>89.2</v>
+      </c>
+      <c r="G492" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H492" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I492" t="n">
+        <v>1</v>
+      </c>
+      <c r="J492" t="n">
+        <v>0</v>
+      </c>
+      <c r="K492" t="n">
+        <v>9</v>
+      </c>
+      <c r="L492" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B493" t="inlineStr">
+        <is>
+          <t>Besiktas vs Istanbul Basaksehir</t>
+        </is>
+      </c>
+      <c r="C493" t="inlineStr">
+        <is>
+          <t>Besiktas</t>
+        </is>
+      </c>
+      <c r="D493" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E493" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="F493" t="n">
+        <v>58.9</v>
+      </c>
+      <c r="G493" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H493" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I493" t="n">
+        <v>0</v>
+      </c>
+      <c r="J493" t="n">
+        <v>5</v>
+      </c>
+      <c r="K493" t="n">
+        <v>0</v>
+      </c>
+      <c r="L493" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B494" t="inlineStr">
+        <is>
+          <t>Galatasaray vs Fenerbahce</t>
+        </is>
+      </c>
+      <c r="C494" t="inlineStr">
+        <is>
+          <t>Galatasaray</t>
+        </is>
+      </c>
+      <c r="D494" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E494" t="n">
+        <v>1.82</v>
+      </c>
+      <c r="F494" t="n">
+        <v>54.9</v>
+      </c>
+      <c r="G494" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H494" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I494" t="n">
+        <v>0</v>
+      </c>
+      <c r="J494" t="n">
+        <v>8</v>
+      </c>
+      <c r="K494" t="n">
+        <v>0</v>
+      </c>
+      <c r="L494" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B495" t="inlineStr">
+        <is>
+          <t>Flamengo vs Atlético-MG</t>
+        </is>
+      </c>
+      <c r="C495" t="inlineStr">
+        <is>
+          <t>Flamengo</t>
+        </is>
+      </c>
+      <c r="D495" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E495" t="n">
+        <v>1.56</v>
+      </c>
+      <c r="F495" t="n">
+        <v>64.2</v>
+      </c>
+      <c r="G495" t="inlineStr">
+        <is>
+          <t>3-2</t>
+        </is>
+      </c>
+      <c r="H495" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I495" t="n">
+        <v>7</v>
+      </c>
+      <c r="J495" t="n">
+        <v>8</v>
+      </c>
+      <c r="K495" t="n">
+        <v>2</v>
+      </c>
+      <c r="L495" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B496" t="inlineStr">
+        <is>
+          <t>Caykur Rizespor vs Trabzonspor</t>
+        </is>
+      </c>
+      <c r="C496" t="inlineStr">
+        <is>
+          <t>Trabzonspor</t>
+        </is>
+      </c>
+      <c r="D496" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E496" t="n">
+        <v>2.06</v>
+      </c>
+      <c r="F496" t="n">
+        <v>48.6</v>
+      </c>
+      <c r="G496" t="inlineStr">
+        <is>
+          <t>3-4</t>
+        </is>
+      </c>
+      <c r="H496" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I496" t="n">
+        <v>0</v>
+      </c>
+      <c r="J496" t="n">
+        <v>0</v>
+      </c>
+      <c r="K496" t="n">
+        <v>1</v>
+      </c>
+      <c r="L496" t="inlineStr">
         <is>
           <t>si</t>
         </is>
@@ -25919,7 +26231,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E77"/>
+  <dimension ref="A1:E78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27343,6 +27655,25 @@
       </c>
       <c r="E77" t="n">
         <v>24</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B78" t="n">
+        <v>6</v>
+      </c>
+      <c r="C78" t="n">
+        <v>6</v>
+      </c>
+      <c r="D78" t="n">
+        <v>100</v>
+      </c>
+      <c r="E78" t="n">
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -27356,7 +27687,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E254"/>
+  <dimension ref="A1:E258"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -32699,6 +33030,90 @@
         <v>0</v>
       </c>
     </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>posible_victoria_favorito</t>
+        </is>
+      </c>
+      <c r="C255" t="n">
+        <v>4</v>
+      </c>
+      <c r="D255" t="n">
+        <v>2</v>
+      </c>
+      <c r="E255" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>ampliacion_marcador</t>
+        </is>
+      </c>
+      <c r="C256" t="n">
+        <v>4</v>
+      </c>
+      <c r="D256" t="n">
+        <v>1</v>
+      </c>
+      <c r="E256" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>penal</t>
+        </is>
+      </c>
+      <c r="C257" t="n">
+        <v>2</v>
+      </c>
+      <c r="D257" t="n">
+        <v>0</v>
+      </c>
+      <c r="E257" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>posible_empate</t>
+        </is>
+      </c>
+      <c r="C258" t="n">
+        <v>1</v>
+      </c>
+      <c r="D258" t="n">
+        <v>1</v>
+      </c>
+      <c r="E258" t="n">
+        <v>100</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-10-28
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L496"/>
+  <dimension ref="A1:L499"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26215,6 +26215,162 @@
         <v>1</v>
       </c>
       <c r="L496" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B497" t="inlineStr">
+        <is>
+          <t>AS Roma vs Cagliari</t>
+        </is>
+      </c>
+      <c r="C497" t="inlineStr">
+        <is>
+          <t>AS Roma</t>
+        </is>
+      </c>
+      <c r="D497" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E497" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="F497" t="n">
+        <v>89.40000000000001</v>
+      </c>
+      <c r="G497" t="inlineStr">
+        <is>
+          <t>4-2</t>
+        </is>
+      </c>
+      <c r="H497" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I497" t="n">
+        <v>4</v>
+      </c>
+      <c r="J497" t="n">
+        <v>4</v>
+      </c>
+      <c r="K497" t="n">
+        <v>2</v>
+      </c>
+      <c r="L497" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B498" t="inlineStr">
+        <is>
+          <t>Argentinos Juniors vs Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="C498" t="inlineStr">
+        <is>
+          <t>Argentinos Juniors</t>
+        </is>
+      </c>
+      <c r="D498" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E498" t="n">
+        <v>2.31</v>
+      </c>
+      <c r="F498" t="n">
+        <v>43.2</v>
+      </c>
+      <c r="G498" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H498" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I498" t="n">
+        <v>3</v>
+      </c>
+      <c r="J498" t="n">
+        <v>2</v>
+      </c>
+      <c r="K498" t="n">
+        <v>2</v>
+      </c>
+      <c r="L498" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B499" t="inlineStr">
+        <is>
+          <t>Torino vs Como</t>
+        </is>
+      </c>
+      <c r="C499" t="inlineStr">
+        <is>
+          <t>Como</t>
+        </is>
+      </c>
+      <c r="D499" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E499" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="F499" t="n">
+        <v>76.90000000000001</v>
+      </c>
+      <c r="G499" t="inlineStr">
+        <is>
+          <t>1-3</t>
+        </is>
+      </c>
+      <c r="H499" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I499" t="n">
+        <v>3</v>
+      </c>
+      <c r="J499" t="n">
+        <v>1</v>
+      </c>
+      <c r="K499" t="n">
+        <v>5</v>
+      </c>
+      <c r="L499" t="inlineStr">
         <is>
           <t>si</t>
         </is>
@@ -26231,7 +26387,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E78"/>
+  <dimension ref="A1:E79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27674,6 +27830,25 @@
       </c>
       <c r="E78" t="n">
         <v>6</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B79" t="n">
+        <v>3</v>
+      </c>
+      <c r="C79" t="n">
+        <v>3</v>
+      </c>
+      <c r="D79" t="n">
+        <v>100</v>
+      </c>
+      <c r="E79" t="n">
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -27687,7 +27862,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E258"/>
+  <dimension ref="A1:E263"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -33114,6 +33289,111 @@
         <v>100</v>
       </c>
     </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>penal</t>
+        </is>
+      </c>
+      <c r="C259" t="n">
+        <v>1</v>
+      </c>
+      <c r="D259" t="n">
+        <v>0</v>
+      </c>
+      <c r="E259" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>ampliacion_marcador</t>
+        </is>
+      </c>
+      <c r="C260" t="n">
+        <v>3</v>
+      </c>
+      <c r="D260" t="n">
+        <v>0</v>
+      </c>
+      <c r="E260" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>cuidado_rival_presiona</t>
+        </is>
+      </c>
+      <c r="C261" t="n">
+        <v>4</v>
+      </c>
+      <c r="D261" t="n">
+        <v>1</v>
+      </c>
+      <c r="E261" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>posible_victoria_favorito</t>
+        </is>
+      </c>
+      <c r="C262" t="n">
+        <v>1</v>
+      </c>
+      <c r="D262" t="n">
+        <v>1</v>
+      </c>
+      <c r="E262" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>posible_empate</t>
+        </is>
+      </c>
+      <c r="C263" t="n">
+        <v>1</v>
+      </c>
+      <c r="D263" t="n">
+        <v>0</v>
+      </c>
+      <c r="E263" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-10-29
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L499"/>
+  <dimension ref="A1:L510"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26371,6 +26371,578 @@
         <v>5</v>
       </c>
       <c r="L499" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B500" t="inlineStr">
+        <is>
+          <t>Celtic vs Dundee United</t>
+        </is>
+      </c>
+      <c r="C500" t="inlineStr">
+        <is>
+          <t>Celtic</t>
+        </is>
+      </c>
+      <c r="D500" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E500" t="n">
+        <v>1.28</v>
+      </c>
+      <c r="F500" t="n">
+        <v>78.09999999999999</v>
+      </c>
+      <c r="G500" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="H500" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I500" t="n">
+        <v>4</v>
+      </c>
+      <c r="J500" t="n">
+        <v>3</v>
+      </c>
+      <c r="K500" t="n">
+        <v>0</v>
+      </c>
+      <c r="L500" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B501" t="inlineStr">
+        <is>
+          <t>Red Bull Bragantino vs Chapecoense</t>
+        </is>
+      </c>
+      <c r="C501" t="inlineStr">
+        <is>
+          <t>Red Bull Bragantino</t>
+        </is>
+      </c>
+      <c r="D501" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E501" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="F501" t="n">
+        <v>57</v>
+      </c>
+      <c r="G501" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="H501" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I501" t="n">
+        <v>5</v>
+      </c>
+      <c r="J501" t="n">
+        <v>1</v>
+      </c>
+      <c r="K501" t="n">
+        <v>4</v>
+      </c>
+      <c r="L501" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B502" t="inlineStr">
+        <is>
+          <t>América vs Tijuana</t>
+        </is>
+      </c>
+      <c r="C502" t="inlineStr">
+        <is>
+          <t>América</t>
+        </is>
+      </c>
+      <c r="D502" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E502" t="n">
+        <v>1.93</v>
+      </c>
+      <c r="F502" t="n">
+        <v>51.8</v>
+      </c>
+      <c r="G502" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H502" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I502" t="n">
+        <v>0</v>
+      </c>
+      <c r="J502" t="n">
+        <v>0</v>
+      </c>
+      <c r="K502" t="n">
+        <v>2</v>
+      </c>
+      <c r="L502" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B503" t="inlineStr">
+        <is>
+          <t>Inter Miami CF vs FC Cincinnati</t>
+        </is>
+      </c>
+      <c r="C503" t="inlineStr">
+        <is>
+          <t>Inter Miami CF</t>
+        </is>
+      </c>
+      <c r="D503" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E503" t="n">
+        <v>2.17</v>
+      </c>
+      <c r="F503" t="n">
+        <v>46.2</v>
+      </c>
+      <c r="G503" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="H503" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I503" t="n">
+        <v>3</v>
+      </c>
+      <c r="J503" t="n">
+        <v>2</v>
+      </c>
+      <c r="K503" t="n">
+        <v>3</v>
+      </c>
+      <c r="L503" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B504" t="inlineStr">
+        <is>
+          <t>Minnesota United FC vs Sporting Kansas City</t>
+        </is>
+      </c>
+      <c r="C504" t="inlineStr">
+        <is>
+          <t>Minnesota United FC</t>
+        </is>
+      </c>
+      <c r="D504" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E504" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="F504" t="n">
+        <v>70</v>
+      </c>
+      <c r="G504" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="H504" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I504" t="n">
+        <v>3</v>
+      </c>
+      <c r="J504" t="n">
+        <v>4</v>
+      </c>
+      <c r="K504" t="n">
+        <v>4</v>
+      </c>
+      <c r="L504" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B505" t="inlineStr">
+        <is>
+          <t>Nashville SC vs Philadelphia Union</t>
+        </is>
+      </c>
+      <c r="C505" t="inlineStr">
+        <is>
+          <t>Nashville SC</t>
+        </is>
+      </c>
+      <c r="D505" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E505" t="n">
+        <v>2.03</v>
+      </c>
+      <c r="F505" t="n">
+        <v>49.4</v>
+      </c>
+      <c r="G505" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H505" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I505" t="n">
+        <v>1</v>
+      </c>
+      <c r="J505" t="n">
+        <v>3</v>
+      </c>
+      <c r="K505" t="n">
+        <v>3</v>
+      </c>
+      <c r="L505" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B506" t="inlineStr">
+        <is>
+          <t>Vancouver Whitecaps vs San Diego FC</t>
+        </is>
+      </c>
+      <c r="C506" t="inlineStr">
+        <is>
+          <t>Vancouver Whitecaps</t>
+        </is>
+      </c>
+      <c r="D506" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E506" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="F506" t="n">
+        <v>47.7</v>
+      </c>
+      <c r="G506" t="inlineStr">
+        <is>
+          <t>4-1</t>
+        </is>
+      </c>
+      <c r="H506" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I506" t="n">
+        <v>0</v>
+      </c>
+      <c r="J506" t="n">
+        <v>8</v>
+      </c>
+      <c r="K506" t="n">
+        <v>0</v>
+      </c>
+      <c r="L506" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B507" t="inlineStr">
+        <is>
+          <t>Venezia vs Internazionale</t>
+        </is>
+      </c>
+      <c r="C507" t="inlineStr">
+        <is>
+          <t>Venezia</t>
+        </is>
+      </c>
+      <c r="D507" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E507" t="n">
+        <v>2.19</v>
+      </c>
+      <c r="F507" t="n">
+        <v>45.7</v>
+      </c>
+      <c r="G507" t="inlineStr">
+        <is>
+          <t>0-2</t>
+        </is>
+      </c>
+      <c r="H507" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I507" t="n">
+        <v>0</v>
+      </c>
+      <c r="J507" t="n">
+        <v>1</v>
+      </c>
+      <c r="K507" t="n">
+        <v>6</v>
+      </c>
+      <c r="L507" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B508" t="inlineStr">
+        <is>
+          <t>Santos vs Palmeiras</t>
+        </is>
+      </c>
+      <c r="C508" t="inlineStr">
+        <is>
+          <t>Palmeiras</t>
+        </is>
+      </c>
+      <c r="D508" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E508" t="n">
+        <v>1.89</v>
+      </c>
+      <c r="F508" t="n">
+        <v>53</v>
+      </c>
+      <c r="G508" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H508" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I508" t="n">
+        <v>3</v>
+      </c>
+      <c r="J508" t="n">
+        <v>1</v>
+      </c>
+      <c r="K508" t="n">
+        <v>6</v>
+      </c>
+      <c r="L508" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B509" t="inlineStr">
+        <is>
+          <t>Bahia vs São Paulo</t>
+        </is>
+      </c>
+      <c r="C509" t="inlineStr">
+        <is>
+          <t>Bahia</t>
+        </is>
+      </c>
+      <c r="D509" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E509" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="F509" t="n">
+        <v>83.2</v>
+      </c>
+      <c r="G509" t="inlineStr">
+        <is>
+          <t>3-2</t>
+        </is>
+      </c>
+      <c r="H509" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I509" t="n">
+        <v>1</v>
+      </c>
+      <c r="J509" t="n">
+        <v>2</v>
+      </c>
+      <c r="K509" t="n">
+        <v>7</v>
+      </c>
+      <c r="L509" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B510" t="inlineStr">
+        <is>
+          <t>Toronto FC vs D.C. United</t>
+        </is>
+      </c>
+      <c r="C510" t="inlineStr">
+        <is>
+          <t>D.C. United</t>
+        </is>
+      </c>
+      <c r="D510" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E510" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="F510" t="n">
+        <v>72.40000000000001</v>
+      </c>
+      <c r="G510" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H510" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I510" t="n">
+        <v>1</v>
+      </c>
+      <c r="J510" t="n">
+        <v>3</v>
+      </c>
+      <c r="K510" t="n">
+        <v>2</v>
+      </c>
+      <c r="L510" t="inlineStr">
         <is>
           <t>si</t>
         </is>
@@ -26387,7 +26959,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E79"/>
+  <dimension ref="A1:E80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27849,6 +28421,25 @@
       </c>
       <c r="E79" t="n">
         <v>3</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B80" t="n">
+        <v>11</v>
+      </c>
+      <c r="C80" t="n">
+        <v>4</v>
+      </c>
+      <c r="D80" t="n">
+        <v>36.4</v>
+      </c>
+      <c r="E80" t="n">
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -27862,7 +28453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E263"/>
+  <dimension ref="A1:E270"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -33394,6 +33985,153 @@
         <v>0</v>
       </c>
     </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>posible_empate</t>
+        </is>
+      </c>
+      <c r="C264" t="n">
+        <v>2</v>
+      </c>
+      <c r="D264" t="n">
+        <v>1</v>
+      </c>
+      <c r="E264" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>posible_victoria_favorito</t>
+        </is>
+      </c>
+      <c r="C265" t="n">
+        <v>5</v>
+      </c>
+      <c r="D265" t="n">
+        <v>1</v>
+      </c>
+      <c r="E265" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>gol_de_cierre</t>
+        </is>
+      </c>
+      <c r="C266" t="n">
+        <v>1</v>
+      </c>
+      <c r="D266" t="n">
+        <v>0</v>
+      </c>
+      <c r="E266" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>alerta_1er_tiempo</t>
+        </is>
+      </c>
+      <c r="C267" t="n">
+        <v>2</v>
+      </c>
+      <c r="D267" t="n">
+        <v>0</v>
+      </c>
+      <c r="E267" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>ampliacion_marcador</t>
+        </is>
+      </c>
+      <c r="C268" t="n">
+        <v>3</v>
+      </c>
+      <c r="D268" t="n">
+        <v>0</v>
+      </c>
+      <c r="E268" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>partido_resuelto</t>
+        </is>
+      </c>
+      <c r="C269" t="n">
+        <v>1</v>
+      </c>
+      <c r="D269" t="n">
+        <v>0</v>
+      </c>
+      <c r="E269" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>cuidado_rival_presiona</t>
+        </is>
+      </c>
+      <c r="C270" t="n">
+        <v>7</v>
+      </c>
+      <c r="D270" t="n">
+        <v>1</v>
+      </c>
+      <c r="E270" t="n">
+        <v>14.3</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-10-30
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L510"/>
+  <dimension ref="A1:L512"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26943,6 +26943,110 @@
         <v>2</v>
       </c>
       <c r="L510" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B511" t="inlineStr">
+        <is>
+          <t>Frosinone vs Lecce</t>
+        </is>
+      </c>
+      <c r="C511" t="inlineStr">
+        <is>
+          <t>Frosinone</t>
+        </is>
+      </c>
+      <c r="D511" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E511" t="n">
+        <v>1.13</v>
+      </c>
+      <c r="F511" t="n">
+        <v>88.5</v>
+      </c>
+      <c r="G511" t="inlineStr">
+        <is>
+          <t>5-1</t>
+        </is>
+      </c>
+      <c r="H511" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I511" t="n">
+        <v>0</v>
+      </c>
+      <c r="J511" t="n">
+        <v>0</v>
+      </c>
+      <c r="K511" t="n">
+        <v>1</v>
+      </c>
+      <c r="L511" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B512" t="inlineStr">
+        <is>
+          <t>Vasco da Gama vs Flamengo</t>
+        </is>
+      </c>
+      <c r="C512" t="inlineStr">
+        <is>
+          <t>Flamengo</t>
+        </is>
+      </c>
+      <c r="D512" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E512" t="n">
+        <v>2.11</v>
+      </c>
+      <c r="F512" t="n">
+        <v>47.4</v>
+      </c>
+      <c r="G512" t="inlineStr">
+        <is>
+          <t>1-4</t>
+        </is>
+      </c>
+      <c r="H512" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I512" t="n">
+        <v>5</v>
+      </c>
+      <c r="J512" t="n">
+        <v>3</v>
+      </c>
+      <c r="K512" t="n">
+        <v>9</v>
+      </c>
+      <c r="L512" t="inlineStr">
         <is>
           <t>si</t>
         </is>
@@ -26959,7 +27063,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E80"/>
+  <dimension ref="A1:E81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28440,6 +28544,25 @@
       </c>
       <c r="E80" t="n">
         <v>11</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B81" t="n">
+        <v>2</v>
+      </c>
+      <c r="C81" t="n">
+        <v>2</v>
+      </c>
+      <c r="D81" t="n">
+        <v>100</v>
+      </c>
+      <c r="E81" t="n">
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -28453,7 +28576,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E270"/>
+  <dimension ref="A1:E273"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -34132,6 +34255,69 @@
         <v>14.3</v>
       </c>
     </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>ampliacion_marcador</t>
+        </is>
+      </c>
+      <c r="C271" t="n">
+        <v>2</v>
+      </c>
+      <c r="D271" t="n">
+        <v>1</v>
+      </c>
+      <c r="E271" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>cuidado_rival_presiona</t>
+        </is>
+      </c>
+      <c r="C272" t="n">
+        <v>2</v>
+      </c>
+      <c r="D272" t="n">
+        <v>0</v>
+      </c>
+      <c r="E272" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>partido_resuelto</t>
+        </is>
+      </c>
+      <c r="C273" t="n">
+        <v>1</v>
+      </c>
+      <c r="D273" t="n">
+        <v>0</v>
+      </c>
+      <c r="E273" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-10-31
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L512"/>
+  <dimension ref="A1:L518"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27047,6 +27047,318 @@
         <v>9</v>
       </c>
       <c r="L512" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B513" t="inlineStr">
+        <is>
+          <t>Villarreal vs Espanyol</t>
+        </is>
+      </c>
+      <c r="C513" t="inlineStr">
+        <is>
+          <t>Villarreal</t>
+        </is>
+      </c>
+      <c r="D513" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E513" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="F513" t="n">
+        <v>80.3</v>
+      </c>
+      <c r="G513" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H513" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I513" t="n">
+        <v>3</v>
+      </c>
+      <c r="J513" t="n">
+        <v>5</v>
+      </c>
+      <c r="K513" t="n">
+        <v>4</v>
+      </c>
+      <c r="L513" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B514" t="inlineStr">
+        <is>
+          <t>SV Elversberg vs Mainz</t>
+        </is>
+      </c>
+      <c r="C514" t="inlineStr">
+        <is>
+          <t>SV Elversberg</t>
+        </is>
+      </c>
+      <c r="D514" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E514" t="n">
+        <v>1.39</v>
+      </c>
+      <c r="F514" t="n">
+        <v>71.8</v>
+      </c>
+      <c r="G514" t="inlineStr">
+        <is>
+          <t>4-1</t>
+        </is>
+      </c>
+      <c r="H514" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I514" t="n">
+        <v>2</v>
+      </c>
+      <c r="J514" t="n">
+        <v>2</v>
+      </c>
+      <c r="K514" t="n">
+        <v>1</v>
+      </c>
+      <c r="L514" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B515" t="inlineStr">
+        <is>
+          <t>Le Havre AC vs Paris Saint-Germain</t>
+        </is>
+      </c>
+      <c r="C515" t="inlineStr">
+        <is>
+          <t>Paris Saint-Germain</t>
+        </is>
+      </c>
+      <c r="D515" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E515" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="F515" t="n">
+        <v>71.40000000000001</v>
+      </c>
+      <c r="G515" t="inlineStr">
+        <is>
+          <t>1-5</t>
+        </is>
+      </c>
+      <c r="H515" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I515" t="n">
+        <v>0</v>
+      </c>
+      <c r="J515" t="n">
+        <v>1</v>
+      </c>
+      <c r="K515" t="n">
+        <v>9</v>
+      </c>
+      <c r="L515" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B516" t="inlineStr">
+        <is>
+          <t>Casa Pia vs Sporting CP</t>
+        </is>
+      </c>
+      <c r="C516" t="inlineStr">
+        <is>
+          <t>Sporting CP</t>
+        </is>
+      </c>
+      <c r="D516" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E516" t="n">
+        <v>1.97</v>
+      </c>
+      <c r="F516" t="n">
+        <v>50.7</v>
+      </c>
+      <c r="G516" t="inlineStr">
+        <is>
+          <t>0-2</t>
+        </is>
+      </c>
+      <c r="H516" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I516" t="n">
+        <v>3</v>
+      </c>
+      <c r="J516" t="n">
+        <v>4</v>
+      </c>
+      <c r="K516" t="n">
+        <v>7</v>
+      </c>
+      <c r="L516" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B517" t="inlineStr">
+        <is>
+          <t>Zulte-Waregem vs Club Brugge</t>
+        </is>
+      </c>
+      <c r="C517" t="inlineStr">
+        <is>
+          <t>Club Brugge</t>
+        </is>
+      </c>
+      <c r="D517" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E517" t="n">
+        <v>1.23</v>
+      </c>
+      <c r="F517" t="n">
+        <v>81.3</v>
+      </c>
+      <c r="G517" t="inlineStr">
+        <is>
+          <t>2-4</t>
+        </is>
+      </c>
+      <c r="H517" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I517" t="n">
+        <v>4</v>
+      </c>
+      <c r="J517" t="n">
+        <v>4</v>
+      </c>
+      <c r="K517" t="n">
+        <v>8</v>
+      </c>
+      <c r="L517" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B518" t="inlineStr">
+        <is>
+          <t>Konyaspor vs Galatasaray</t>
+        </is>
+      </c>
+      <c r="C518" t="inlineStr">
+        <is>
+          <t>Galatasaray</t>
+        </is>
+      </c>
+      <c r="D518" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E518" t="n">
+        <v>1.42</v>
+      </c>
+      <c r="F518" t="n">
+        <v>70.2</v>
+      </c>
+      <c r="G518" t="inlineStr">
+        <is>
+          <t>0-4</t>
+        </is>
+      </c>
+      <c r="H518" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I518" t="n">
+        <v>0</v>
+      </c>
+      <c r="J518" t="n">
+        <v>0</v>
+      </c>
+      <c r="K518" t="n">
+        <v>9</v>
+      </c>
+      <c r="L518" t="inlineStr">
         <is>
           <t>si</t>
         </is>
@@ -27063,7 +27375,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E81"/>
+  <dimension ref="A1:E82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28563,6 +28875,25 @@
       </c>
       <c r="E81" t="n">
         <v>2</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B82" t="n">
+        <v>6</v>
+      </c>
+      <c r="C82" t="n">
+        <v>5</v>
+      </c>
+      <c r="D82" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="E82" t="n">
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -28576,7 +28907,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E273"/>
+  <dimension ref="A1:E279"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -34318,6 +34649,132 @@
         <v>0</v>
       </c>
     </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>alerta_1er_tiempo</t>
+        </is>
+      </c>
+      <c r="C274" t="n">
+        <v>1</v>
+      </c>
+      <c r="D274" t="n">
+        <v>0</v>
+      </c>
+      <c r="E274" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>posible_victoria_favorito</t>
+        </is>
+      </c>
+      <c r="C275" t="n">
+        <v>1</v>
+      </c>
+      <c r="D275" t="n">
+        <v>0</v>
+      </c>
+      <c r="E275" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>posible_empate</t>
+        </is>
+      </c>
+      <c r="C276" t="n">
+        <v>1</v>
+      </c>
+      <c r="D276" t="n">
+        <v>0</v>
+      </c>
+      <c r="E276" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>cuidado_rival_presiona</t>
+        </is>
+      </c>
+      <c r="C277" t="n">
+        <v>1</v>
+      </c>
+      <c r="D277" t="n">
+        <v>0</v>
+      </c>
+      <c r="E277" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>partido_resuelto</t>
+        </is>
+      </c>
+      <c r="C278" t="n">
+        <v>2</v>
+      </c>
+      <c r="D278" t="n">
+        <v>0</v>
+      </c>
+      <c r="E278" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>ampliacion_marcador</t>
+        </is>
+      </c>
+      <c r="C279" t="n">
+        <v>6</v>
+      </c>
+      <c r="D279" t="n">
+        <v>2</v>
+      </c>
+      <c r="E279" t="n">
+        <v>33.3</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>